<commit_message>
Organize forecast snapshots by source
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf9f06cd4a38f464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="Rc6caa618f378479e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rfde10151e93743e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rd669e632e5d34f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd14b94fe941343bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="Rf856e113023d4d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R1a842aca813c4c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf4e1f880aaff412d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -309,7 +309,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R324a08616b0e4166"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra222533b37de42c8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -365,7 +365,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -749,7 +749,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08da08a20ddd4959"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c05a71eb864101"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -927,7 +927,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N6" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O6" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -974,7 +974,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N7" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O7" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1021,7 +1021,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N8" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O8" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1068,7 +1068,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O9" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1115,7 +1115,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N10" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O10" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1162,7 +1162,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N11" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O11" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1209,7 +1209,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O12" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1256,7 +1256,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O13" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1303,7 +1303,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O14" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1350,7 +1350,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N15" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O15" s="16" t="str">
         <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1397,7 +1397,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N16" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O16" s="16" t="str">
         <x:v>Latest published state on or before evidence cutoff for each Epoch-covered U.S. site</x:v>
@@ -1444,7 +1444,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N17" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O17" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1491,7 +1491,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N18" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O18" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1538,7 +1538,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N19" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O19" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1585,7 +1585,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N20" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O20" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1632,7 +1632,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N21" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O21" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1679,7 +1679,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N22" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O22" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1726,7 +1726,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N23" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O23" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1773,7 +1773,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N24" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O24" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1820,7 +1820,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="N25" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="O25" s="16" t="str">
         <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
@@ -1832,9 +1832,9 @@
     <x:mergeCell ref="A3:O3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2266eb8538f04e3b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae4ec148f1224cb7"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d337250e6d249e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d544a0a3cac4d9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1863,9 +1863,9 @@
       <x:c r="C2" s="3"/>
       <x:c r="D2" s="3"/>
     </x:row>
-    <x:row r="3" ht="36" hidden="0" customHeight="1">
+    <x:row r="3" ht="48" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>All population, allocation, workload, and hardware-normalization assumptions read directly from compute-capacity.json.</x:v>
+        <x:v>All population, allocation, workload, and hardware-normalization assumptions read from the compute-capacity logical dataset in gate2-consolidated.json.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -2117,7 +2117,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R851bb1a45bc64406"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf41fec5c46af43d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2190,141 +2190,72 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="97.19999694824219" hidden="0" customHeight="1">
+    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>source-001</x:v>
+        <x:v>gate2-diffuse-personal-ai-gate-2-compute-supply-calculation-contract</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Personal AI forecast</x:v>
+        <x:v>Diffuse Personal AI</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>Model-harness capability report card — HTML</x:v>
+        <x:v>Gate 2 · Compute supply calculation contract</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>cross-report reference</x:v>
+        <x:v>methodology, normalization, model configuration</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>https://diffuse-personal-ai-countdown.buddywilliams.chatgpt.site/?report=capability</x:v>
+        <x:v>https://github.com/buwilliams/diffuse-personal-ai/blob/main/intent/02-model/06-report-card-calculations.md</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>Capability uses the same snapshot and shared model; its default 75% crossing is 2027-11-13.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="86.4000015258789" hidden="0" customHeight="1">
+        <x:v>Holds definitions and assumptions that are authored by the forecast rather than fetched as observations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="140.39999389648438" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
-        <x:v>source-002</x:v>
+        <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
         <x:v>Epoch AI</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>AI Data Centers</x:v>
+        <x:v>AI Data Center Timelines CSV</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
-        <x:v>capacity methodology</x:v>
+        <x:v>capacity observation, capacity projection</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
-        <x:v>https://epoch.ai/data/ai-data-centers</x:v>
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
-        <x:v>Defines dataset scope, H100e convention, coverage, and uncertainty.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="140.39999389648438" hidden="0" customHeight="1">
+        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="108" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>source-003</x:v>
+        <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>Epoch AI</x:v>
+        <x:v>U.S. Census Bureau</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
-        <x:v>AI Data Center Timelines CSV</x:v>
+        <x:v>Population on a Date</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
-        <x:v>2026-08-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>capacity observation, capacity projection</x:v>
+        <x:v>population</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
-        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+        <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="54" hidden="0" customHeight="1">
-      <x:c r="A9" s="16" t="str">
-        <x:v>source-004</x:v>
-      </x:c>
-      <x:c r="B9" s="16" t="str">
-        <x:v>Epoch AI</x:v>
-      </x:c>
-      <x:c r="C9" s="16" t="str">
-        <x:v>AI Data Centers CSV</x:v>
-      </x:c>
-      <x:c r="D9" s="16" t="str">
-        <x:v>2026-08-25</x:v>
-      </x:c>
-      <x:c r="E9" s="16" t="str">
-        <x:v>capacity registry</x:v>
-      </x:c>
-      <x:c r="F9" s="16" t="str">
-        <x:v>https://epoch.ai/data/data_centers/data_centers.csv</x:v>
-      </x:c>
-      <x:c r="G9" s="16" t="str">
-        <x:v>Provides the country filter and current site registry.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="108" hidden="0" customHeight="1">
-      <x:c r="A10" s="16" t="str">
-        <x:v>source-005</x:v>
-      </x:c>
-      <x:c r="B10" s="16" t="str">
-        <x:v>Personal AI forecast</x:v>
-      </x:c>
-      <x:c r="C10" s="16" t="str">
-        <x:v>Report-card calculation contract</x:v>
-      </x:c>
-      <x:c r="D10" s="16" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
-      <x:c r="E10" s="16" t="str">
-        <x:v>methodology</x:v>
-      </x:c>
-      <x:c r="F10" s="16" t="str">
-        <x:v>https://github.com/buwilliams/diffuse-personal-ai/blob/main/intent/02-model/06-report-card-calculations.md</x:v>
-      </x:c>
-      <x:c r="G10" s="16" t="str">
-        <x:v>Defines the serving envelope and high-autonomy token mix; assumptions remain editable.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="108" hidden="0" customHeight="1">
-      <x:c r="A11" s="16" t="str">
-        <x:v>source-006</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str">
-        <x:v>U.S. Census Bureau</x:v>
-      </x:c>
-      <x:c r="C11" s="16" t="str">
-        <x:v>Population on a Date</x:v>
-      </x:c>
-      <x:c r="D11" s="16" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="E11" s="16" t="str">
-        <x:v>population</x:v>
-      </x:c>
-      <x:c r="F11" s="16" t="str">
-        <x:v>https://www.census.gov/popclock/</x:v>
-      </x:c>
-      <x:c r="G11" s="16" t="str">
         <x:v>The model uses the rounded estimate of 342.8M residents; the selected 50% target is 171.4M users.</x:v>
       </x:c>
     </x:row>
@@ -2335,7 +2266,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R008262a85b9948d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f9b610c6d0b472e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expose source results and update default scenario
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd14b94fe941343bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="Rf856e113023d4d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R1a842aca813c4c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf4e1f880aaff412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R36bf5d850af84e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R70f94bf7e07a4c54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R2ddebd6fc5714166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R1c31b6ed56e147b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -309,7 +309,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra222533b37de42c8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R175df869f2df4d40"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -637,7 +637,7 @@
         <x:v>Current supported users</x:v>
       </x:c>
       <x:c r="B8" s="19" t="n">
-        <x:v>32212680.521781493</x:v>
+        <x:v>38655216.62613779</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
         <x:v>high-autonomy users</x:v>
@@ -648,10 +648,10 @@
         <x:v>Target users</x:v>
       </x:c>
       <x:c r="B9" s="19" t="n">
-        <x:v>171400000</x:v>
+        <x:v>85700000</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
-        <x:v>50% of U.S. population</x:v>
+        <x:v>25% of U.S. population</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -659,7 +659,7 @@
         <x:v>Required U.S. capacity</x:v>
       </x:c>
       <x:c r="B10" s="19" t="n">
-        <x:v>71959693.84890558</x:v>
+        <x:v>29983205.770377323</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
         <x:v>H100-equivalents</x:v>
@@ -670,7 +670,7 @@
         <x:v>Current supply score</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>0.18793862614808338</x:v>
+        <x:v>0.45105270275540016</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
         <x:v>supported users / target users</x:v>
@@ -681,7 +681,7 @@
         <x:v>Personal-AI inference share</x:v>
       </x:c>
       <x:c r="B12" s="20" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
         <x:v>scenario allocation</x:v>
@@ -703,7 +703,7 @@
         <x:v>Tokens per H100e/day</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:v>39896640</x:v>
+        <x:v>47875968</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
         <x:v>after personal-AI allocation</x:v>
@@ -736,7 +736,7 @@
         <x:v>Continuous base-case crossing</x:v>
       </x:c>
       <x:c r="B17" s="21" t="n">
-        <x:v>47168.337489398145</x:v>
+        <x:v>46750.994524664355</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
         <x:v>100% of selected target</x:v>
@@ -749,7 +749,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c05a71eb864101"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6d1133b5bbe4563"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -912,13 +912,13 @@
       </x:c>
       <x:c r="H6" s="23"/>
       <x:c r="I6" s="22" t="n">
-        <x:v>9801168168960</x:v>
+        <x:v>11761401802752</x:v>
       </x:c>
       <x:c r="J6" s="22" t="n">
-        <x:v>585144.3682961194</x:v>
+        <x:v>702173.2419553433</x:v>
       </x:c>
       <x:c r="K6" s="17" t="n">
-        <x:v>0.00341391113358296</x:v>
+        <x:v>0.008193386720599105</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str">
         <x:v>F</x:v>
@@ -959,13 +959,13 @@
         <x:v>0.9519637402300738</x:v>
       </x:c>
       <x:c r="I7" s="22" t="n">
-        <x:v>18960399400320</x:v>
+        <x:v>22752479280384</x:v>
       </x:c>
       <x:c r="J7" s="22" t="n">
-        <x:v>1131964.1433026865</x:v>
+        <x:v>1358356.9719632238</x:v>
       </x:c>
       <x:c r="K7" s="17" t="n">
-        <x:v>0.00660422487341124</x:v>
+        <x:v>0.015850139696186975</x:v>
       </x:c>
       <x:c r="L7" s="16" t="str">
         <x:v>F</x:v>
@@ -1006,13 +1006,13 @@
         <x:v>0.6037082683951738</x:v>
       </x:c>
       <x:c r="I8" s="22" t="n">
-        <x:v>28812555475200</x:v>
+        <x:v>34575066570240</x:v>
       </x:c>
       <x:c r="J8" s="22" t="n">
-        <x:v>1720152.565683582</x:v>
+        <x:v>2064183.0788202984</x:v>
       </x:c>
       <x:c r="K8" s="17" t="n">
-        <x:v>0.010035895949145753</x:v>
+        <x:v>0.024086150277949806</x:v>
       </x:c>
       <x:c r="L8" s="16" t="str">
         <x:v>F</x:v>
@@ -1053,13 +1053,13 @@
         <x:v>0.48746731270438204</x:v>
       </x:c>
       <x:c r="I9" s="22" t="n">
-        <x:v>40394669757120</x:v>
+        <x:v>48473603708544</x:v>
       </x:c>
       <x:c r="J9" s="22" t="n">
-        <x:v>2411622.0750519405</x:v>
+        <x:v>2893946.4900623285</x:v>
       </x:c>
       <x:c r="K9" s="17" t="n">
-        <x:v>0.01407014046121319</x:v>
+        <x:v>0.03376833710691165</x:v>
       </x:c>
       <x:c r="L9" s="16" t="str">
         <x:v>F</x:v>
@@ -1100,13 +1100,13 @@
         <x:v>0.416386256410302</x:v>
       </x:c>
       <x:c r="I10" s="22" t="n">
-        <x:v>53909935833600</x:v>
+        <x:v>64691923000320</x:v>
       </x:c>
       <x:c r="J10" s="22" t="n">
-        <x:v>3218503.6318567162</x:v>
+        <x:v>3862204.3582280595</x:v>
       </x:c>
       <x:c r="K10" s="17" t="n">
-        <x:v>0.018777734141521098</x:v>
+        <x:v>0.04506656193965063</x:v>
       </x:c>
       <x:c r="L10" s="16" t="str">
         <x:v>F</x:v>
@@ -1147,13 +1147,13 @@
         <x:v>0.8208396780997056</x:v>
       </x:c>
       <x:c r="I11" s="22" t="n">
-        <x:v>95228332496640</x:v>
+        <x:v>114273998995968</x:v>
       </x:c>
       <x:c r="J11" s="22" t="n">
-        <x:v>5685273.581888955</x:v>
+        <x:v>6822328.298266746</x:v>
       </x:c>
       <x:c r="K11" s="17" t="n">
-        <x:v>0.033169624165046416</x:v>
+        <x:v>0.07960709799611139</x:v>
       </x:c>
       <x:c r="L11" s="16" t="str">
         <x:v>F</x:v>
@@ -1194,13 +1194,13 @@
         <x:v>0.3954847159961119</x:v>
       </x:c>
       <x:c r="I12" s="22" t="n">
-        <x:v>125261884742400</x:v>
+        <x:v>150314261690880</x:v>
       </x:c>
       <x:c r="J12" s="22" t="n">
-        <x:v>7478321.477158209</x:v>
+        <x:v>8973985.772589851</x:v>
       </x:c>
       <x:c r="K12" s="17" t="n">
-        <x:v>0.04363081375238162</x:v>
+        <x:v>0.10471395300571588</x:v>
       </x:c>
       <x:c r="L12" s="16" t="str">
         <x:v>F</x:v>
@@ -1241,13 +1241,13 @@
         <x:v>0.7530343299629934</x:v>
       </x:c>
       <x:c r="I13" s="22" t="n">
-        <x:v>211108083480000</x:v>
+        <x:v>253329700176000</x:v>
       </x:c>
       <x:c r="J13" s="22" t="n">
-        <x:v>12603467.670447761</x:v>
+        <x:v>15124161.204537313</x:v>
       </x:c>
       <x:c r="K13" s="17" t="n">
-        <x:v>0.07353248349152719</x:v>
+        <x:v>0.17647796037966526</x:v>
       </x:c>
       <x:c r="L13" s="16" t="str">
         <x:v>F</x:v>
@@ -1288,13 +1288,13 @@
         <x:v>0.25200545793085993</x:v>
       </x:c>
       <x:c r="I14" s="22" t="n">
-        <x:v>251400458252160</x:v>
+        <x:v>301680549902592</x:v>
       </x:c>
       <x:c r="J14" s="22" t="n">
-        <x:v>15008982.582218507</x:v>
+        <x:v>18010779.09866221</x:v>
       </x:c>
       <x:c r="K14" s="17" t="n">
-        <x:v>0.08756699289509047</x:v>
+        <x:v>0.21016078294821713</x:v>
       </x:c>
       <x:c r="L14" s="16" t="str">
         <x:v>F</x:v>
@@ -1335,13 +1335,13 @@
         <x:v>0.8328482478612571</x:v>
       </x:c>
       <x:c r="I15" s="22" t="n">
-        <x:v>447794102347200</x:v>
+        <x:v>537352922816640</x:v>
       </x:c>
       <x:c r="J15" s="22" t="n">
-        <x:v>26733976.25953433</x:v>
+        <x:v>32080771.511441194</x:v>
       </x:c>
       <x:c r="K15" s="17" t="n">
-        <x:v>0.15597419054570788</x:v>
+        <x:v>0.3743380573096989</x:v>
       </x:c>
       <x:c r="L15" s="16" t="str">
         <x:v>F</x:v>
@@ -1382,13 +1382,13 @@
         <x:v>0.26895428526377074</x:v>
       </x:c>
       <x:c r="I16" s="22" t="n">
-        <x:v>539562398739840</x:v>
+        <x:v>647474878487808</x:v>
       </x:c>
       <x:c r="J16" s="22" t="n">
-        <x:v>32212680.521781493</x:v>
+        <x:v>38655216.62613779</x:v>
       </x:c>
       <x:c r="K16" s="17" t="n">
-        <x:v>0.18793862614808338</x:v>
+        <x:v>0.45105270275540016</x:v>
       </x:c>
       <x:c r="L16" s="16" t="str">
         <x:v>F</x:v>
@@ -1429,13 +1429,13 @@
         <x:v>0.36354567443740393</x:v>
       </x:c>
       <x:c r="I17" s="22" t="n">
-        <x:v>694192359772800</x:v>
+        <x:v>833030831727360</x:v>
       </x:c>
       <x:c r="J17" s="22" t="n">
-        <x:v>41444319.98643582</x:v>
+        <x:v>49733183.983722985</x:v>
       </x:c>
       <x:c r="K17" s="17" t="n">
-        <x:v>0.24179883305971892</x:v>
+        <x:v>0.5803171993433254</x:v>
       </x:c>
       <x:c r="L17" s="16" t="str">
         <x:v>F</x:v>
@@ -1476,19 +1476,19 @@
         <x:v>0.227240621716696</x:v>
       </x:c>
       <x:c r="I18" s="22" t="n">
-        <x:v>812617316904960</x:v>
+        <x:v>975140780285952</x:v>
       </x:c>
       <x:c r="J18" s="22" t="n">
-        <x:v>48514466.68089314</x:v>
+        <x:v>58217360.01707176</x:v>
       </x:c>
       <x:c r="K18" s="17" t="n">
-        <x:v>0.28304823034360055</x:v>
+        <x:v>0.6793157528246413</x:v>
       </x:c>
       <x:c r="L18" s="16" t="str">
-        <x:v>F</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="M18" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N18" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1523,19 +1523,19 @@
         <x:v>0.07394840621576648</x:v>
       </x:c>
       <x:c r="I19" s="22" t="n">
-        <x:v>855355714778880</x:v>
+        <x:v>1026426857734656</x:v>
       </x:c>
       <x:c r="J19" s="22" t="n">
-        <x:v>51066012.8226197</x:v>
+        <x:v>61279215.38714364</x:v>
       </x:c>
       <x:c r="K19" s="17" t="n">
-        <x:v>0.29793473058704606</x:v>
+        <x:v>0.7150433534089107</x:v>
       </x:c>
       <x:c r="L19" s="16" t="str">
-        <x:v>F</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="M19" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N19" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1570,19 +1570,19 @@
         <x:v>0.11649967427711161</x:v>
       </x:c>
       <x:c r="I20" s="22" t="n">
-        <x:v>927292309050240</x:v>
+        <x:v>1112750770860288</x:v>
       </x:c>
       <x:c r="J20" s="22" t="n">
-        <x:v>55360734.868671045</x:v>
+        <x:v>66432881.84240525</x:v>
       </x:c>
       <x:c r="K20" s="17" t="n">
-        <x:v>0.3229914519759104</x:v>
+        <x:v>0.775179484742185</x:v>
       </x:c>
       <x:c r="L20" s="16" t="str">
-        <x:v>F</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="M20" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N20" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1617,19 +1617,19 @@
         <x:v>0.37097724915453156</x:v>
       </x:c>
       <x:c r="I21" s="22" t="n">
-        <x:v>1199200877058240</x:v>
+        <x:v>1439041052469888</x:v>
       </x:c>
       <x:c r="J21" s="22" t="n">
-        <x:v>71594082.21243224</x:v>
+        <x:v>85912898.65491869</x:v>
       </x:c>
       <x:c r="K21" s="17" t="n">
-        <x:v>0.41770176319972135</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L21" s="16" t="str">
-        <x:v>F</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="M21" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N21" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1664,19 +1664,19 @@
         <x:v>0.3016709376392015</x:v>
       </x:c>
       <x:c r="I22" s="22" t="n">
-        <x:v>1478100413603520</x:v>
+        <x:v>1773720496324224</x:v>
       </x:c>
       <x:c r="J22" s="22" t="n">
-        <x:v>88244800.81215045</x:v>
+        <x:v>105893760.97458054</x:v>
       </x:c>
       <x:c r="K22" s="17" t="n">
-        <x:v>0.5148471459285324</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L22" s="16" t="str">
-        <x:v>F</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="M22" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N22" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1711,19 +1711,19 @@
         <x:v>0.3134085038100096</x:v>
       </x:c>
       <x:c r="I23" s="22" t="n">
-        <x:v>1836746830356480</x:v>
+        <x:v>2204096196427776</x:v>
       </x:c>
       <x:c r="J23" s="22" t="n">
-        <x:v>109656527.18546149</x:v>
+        <x:v>131587832.6225538</x:v>
       </x:c>
       <x:c r="K23" s="17" t="n">
-        <x:v>0.6397697035324474</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L23" s="16" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="M23" s="16" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N23" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1758,19 +1758,19 @@
         <x:v>0.03312351026722382</x:v>
       </x:c>
       <x:c r="I24" s="22" t="n">
-        <x:v>1879405395053760</x:v>
+        <x:v>2255286474064512</x:v>
       </x:c>
       <x:c r="J24" s="22" t="n">
-        <x:v>112203307.16738866</x:v>
+        <x:v>134643968.60086638</x:v>
       </x:c>
       <x:c r="K24" s="17" t="n">
-        <x:v>0.6546283965425242</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L24" s="16" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="M24" s="16" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N24" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1805,19 +1805,19 @@
         <x:v>0.39370043833106294</x:v>
       </x:c>
       <x:c r="I25" s="22" t="n">
-        <x:v>2469085394408640</x:v>
+        <x:v>2962902473290368</x:v>
       </x:c>
       <x:c r="J25" s="22" t="n">
-        <x:v>147408083.248277</x:v>
+        <x:v>176889699.8979324</x:v>
       </x:c>
       <x:c r="K25" s="17" t="n">
-        <x:v>0.860023822918769</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L25" s="16" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="M25" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N25" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -1832,9 +1832,9 @@
     <x:mergeCell ref="A3:O3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae4ec148f1224cb7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94f93e410454915"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d544a0a3cac4d9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6bb1bca94fe4fbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1908,7 +1908,7 @@
         <x:v>Selected target</x:v>
       </x:c>
       <x:c r="C7" s="24" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>share of residents</x:v>
@@ -2048,7 +2048,7 @@
         <x:v>Personal-AI inference share</x:v>
       </x:c>
       <x:c r="C17" s="24" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
         <x:v>scenario allocation</x:v>
@@ -2117,7 +2117,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf41fec5c46af43d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad31032fd71e4400"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2236,7 +2236,7 @@
         <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="108" hidden="0" customHeight="1">
+    <x:row r="8" ht="97.19999694824219" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
         <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
@@ -2256,7 +2256,7 @@
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>The model uses the rounded estimate of 342.8M residents; the selected 50% target is 171.4M users.</x:v>
+        <x:v>The model uses the rounded estimate of 342.8M residents; the selected 25% target is 85.7M users.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2266,7 +2266,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f9b610c6d0b472e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R474abccf99074d69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add compute buildout outlook evidence
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R36bf5d850af84e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R70f94bf7e07a4c54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R2ddebd6fc5714166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R1c31b6ed56e147b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R66430a2dcd3f4a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R3dc75373423f44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Ra516bff1d1514981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="4" r:id="R6402821b61f84997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R86a0a7989c7641ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -309,7 +310,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R175df869f2df4d40"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7c99044c73d467e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -365,7 +366,28 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Evidence ID"/>
+    <x:tableColumn id="2" name="Metric"/>
+    <x:tableColumn id="3" name="Value"/>
+    <x:tableColumn id="4" name="Unit"/>
+    <x:tableColumn id="5" name="Scope"/>
+    <x:tableColumn id="6" name="Metric date"/>
+    <x:tableColumn id="7" name="Evidence class"/>
+    <x:tableColumn id="8" name="Qualifier"/>
+    <x:tableColumn id="9" name="Source location"/>
+    <x:tableColumn id="10" name="Source ID"/>
+    <x:tableColumn id="11" name="Claim"/>
+    <x:tableColumn id="12" name="Caveat"/>
+    <x:tableColumn id="13" name="Countdown input"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -749,7 +771,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6d1133b5bbe4563"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R400a7f84d36c4d74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1832,9 +1854,9 @@
     <x:mergeCell ref="A3:O3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94f93e410454915"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7f79f9a0564981"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6bb1bca94fe4fbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R586f6a2e2d474f76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2117,12 +2139,749 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad31032fd71e4400"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05c1e9098a554d31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="62" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="68" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Independent Compute-Supply Diagnostics</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+      <x:c r="H1" s="3"/>
+      <x:c r="I1" s="3"/>
+      <x:c r="J1" s="3"/>
+      <x:c r="K1" s="3"/>
+      <x:c r="L1" s="3"/>
+      <x:c r="M1" s="3"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="3"/>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+      <x:c r="H2" s="3"/>
+      <x:c r="I2" s="3"/>
+      <x:c r="J2" s="3"/>
+      <x:c r="K2" s="3"/>
+      <x:c r="L2" s="3"/>
+      <x:c r="M2" s="3"/>
+    </x:row>
+    <x:row r="3" ht="24" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>Source-reported global build-rate, geography, performance, and allocation estimates. These retain their original units and do not directly enter the U.S. H100e countdown.</x:v>
+      </x:c>
+      <x:c r="B3" s="6"/>
+      <x:c r="C3" s="6"/>
+      <x:c r="D3" s="6"/>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="6"/>
+      <x:c r="G3" s="6"/>
+      <x:c r="H3" s="6"/>
+      <x:c r="I3" s="6"/>
+      <x:c r="J3" s="6"/>
+      <x:c r="K3" s="6"/>
+      <x:c r="L3" s="6"/>
+      <x:c r="M3" s="6"/>
+    </x:row>
+    <x:row r="4"/>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Evidence ID</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Metric date</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Evidence class</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Qualifier</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>Source location</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="str">
+        <x:v>Claim</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="str">
+        <x:v>Caveat</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>Countdown input</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>global-incremental-ai-compute-2026</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>Global incremental AI-compute capacity</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>Global additions in 2026</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>2026-12-31</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
+        <x:v>point estimate</x:v>
+      </x:c>
+      <x:c r="I6" s="16" t="str">
+        <x:v>05:54</x:v>
+      </x:c>
+      <x:c r="J6" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="str">
+        <x:v>Incremental global AI compute adds 30 GW in 2026.</x:v>
+      </x:c>
+      <x:c r="L6" s="16" t="str">
+        <x:v>Forward expert estimate in watts; not U.S.-specific and not directly comparable with the H100e countdown series.</x:v>
+      </x:c>
+      <x:c r="M6" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>global-incremental-ai-compute-2027</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>Global incremental AI-compute capacity</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>Global additions in 2027</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>2027-12-31</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>point estimate</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="str">
+        <x:v>05:54</x:v>
+      </x:c>
+      <x:c r="J7" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="str">
+        <x:v>Incremental global AI compute adds 50 GW in 2027.</x:v>
+      </x:c>
+      <x:c r="L7" s="16" t="str">
+        <x:v>Forward expert estimate in watts; not U.S.-specific and not directly comparable with the H100e countdown series.</x:v>
+      </x:c>
+      <x:c r="M7" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>global-incremental-ai-compute-2028</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>Global incremental AI-compute capacity</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str">
+        <x:v>Global additions in 2028</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>2028-12-31</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>approximate point estimate</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="str">
+        <x:v>05:54</x:v>
+      </x:c>
+      <x:c r="J8" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K8" s="16" t="str">
+        <x:v>Incremental global AI compute adds roughly 70 GW in 2028.</x:v>
+      </x:c>
+      <x:c r="L8" s="16" t="str">
+        <x:v>Forward expert estimate in watts; not U.S.-specific and not directly comparable with the H100e countdown series.</x:v>
+      </x:c>
+      <x:c r="M8" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>global-incremental-ai-compute-2029-lower</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>Global incremental AI-compute capacity</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>Global additions in 2029</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>2029-12-31</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>range lower bound</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="str">
+        <x:v>33:45</x:v>
+      </x:c>
+      <x:c r="J9" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K9" s="16" t="str">
+        <x:v>Incremental global AI compute in 2029 is estimated at 90–100 GW.</x:v>
+      </x:c>
+      <x:c r="L9" s="16" t="str">
+        <x:v>Lower bound of a forward expert range; not U.S.-specific and outside the visible four-year report window.</x:v>
+      </x:c>
+      <x:c r="M9" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>global-incremental-ai-compute-2029-upper</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>Global incremental AI-compute capacity</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str">
+        <x:v>Global additions in 2029</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="str">
+        <x:v>2029-12-31</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="str">
+        <x:v>range upper bound</x:v>
+      </x:c>
+      <x:c r="I10" s="16" t="str">
+        <x:v>33:45</x:v>
+      </x:c>
+      <x:c r="J10" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K10" s="16" t="str">
+        <x:v>Incremental global AI compute in 2029 is estimated at 90–100 GW.</x:v>
+      </x:c>
+      <x:c r="L10" s="16" t="str">
+        <x:v>Upper bound of a forward expert range; not U.S.-specific and outside the visible four-year report window.</x:v>
+      </x:c>
+      <x:c r="M10" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>global-ai-compute-stock-2028-lower</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>Global AI-compute capacity stock</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>GW</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>Global stock by end of 2028</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>2028-12-31</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>lower bound</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="str">
+        <x:v>33:32</x:v>
+      </x:c>
+      <x:c r="J11" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K11" s="16" t="str">
+        <x:v>Global AI-compute capacity would exceed 200 GW by the end of 2028.</x:v>
+      </x:c>
+      <x:c r="L11" s="16" t="str">
+        <x:v>Interview cross-check derived from the preceding annual additions; hardware generations and usable performance are heterogeneous.</x:v>
+      </x:c>
+      <x:c r="M11" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>us-share-new-ai-compute-watts-2026</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>U.S. share of new AI-compute watts</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str">
+        <x:v>Current new deployments</x:v>
+      </x:c>
+      <x:c r="F12" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H12" s="16" t="str">
+        <x:v>approximate point estimate</x:v>
+      </x:c>
+      <x:c r="I12" s="16" t="str">
+        <x:v>34:58</x:v>
+      </x:c>
+      <x:c r="J12" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K12" s="16" t="str">
+        <x:v>About 70% of watts currently being deployed for AI compute are in the United States.</x:v>
+      </x:c>
+      <x:c r="L12" s="16" t="str">
+        <x:v>Share of new watts, not share of installed H100-equivalent capacity; the denominator and site-coverage rule differ from Epoch.</x:v>
+      </x:c>
+      <x:c r="M12" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="97.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>openai-anthropic-share-incremental-compute-2026</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>OpenAI and Anthropic share of incremental compute</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str">
+        <x:v>Global additions in 2026</x:v>
+      </x:c>
+      <x:c r="F13" s="16" t="str">
+        <x:v>2026-12-31</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="str">
+        <x:v>approximate point estimate</x:v>
+      </x:c>
+      <x:c r="I13" s="16" t="str">
+        <x:v>04:06</x:v>
+      </x:c>
+      <x:c r="J13" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K13" s="16" t="str">
+        <x:v>OpenAI and Anthropic account for about 30% of incremental compute added in 2026.</x:v>
+      </x:c>
+      <x:c r="L13" s="16" t="str">
+        <x:v>Frontier-lab demand concentration estimate; it does not measure personal-AI inference supply.</x:v>
+      </x:c>
+      <x:c r="M13" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A14" s="16" t="str">
+        <x:v>openai-anthropic-share-incremental-compute-2027-lower</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="str">
+        <x:v>OpenAI and Anthropic share of incremental compute</x:v>
+      </x:c>
+      <x:c r="C14" s="16" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E14" s="16" t="str">
+        <x:v>Global additions in 2027</x:v>
+      </x:c>
+      <x:c r="F14" s="16" t="str">
+        <x:v>2027-12-31</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H14" s="16" t="str">
+        <x:v>range lower bound</x:v>
+      </x:c>
+      <x:c r="I14" s="16" t="str">
+        <x:v>04:15</x:v>
+      </x:c>
+      <x:c r="J14" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K14" s="16" t="str">
+        <x:v>OpenAI and Anthropic are estimated to take 40–50% of incremental compute in 2027.</x:v>
+      </x:c>
+      <x:c r="L14" s="16" t="str">
+        <x:v>Lower bound of a frontier-lab demand concentration estimate; it does not measure personal-AI inference supply.</x:v>
+      </x:c>
+      <x:c r="M14" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A15" s="16" t="str">
+        <x:v>openai-anthropic-share-incremental-compute-2027-upper</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>OpenAI and Anthropic share of incremental compute</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>Global additions in 2027</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="str">
+        <x:v>2027-12-31</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H15" s="16" t="str">
+        <x:v>range upper bound</x:v>
+      </x:c>
+      <x:c r="I15" s="16" t="str">
+        <x:v>04:15</x:v>
+      </x:c>
+      <x:c r="J15" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K15" s="16" t="str">
+        <x:v>OpenAI and Anthropic are estimated to take 40–50% of incremental compute in 2027.</x:v>
+      </x:c>
+      <x:c r="L15" s="16" t="str">
+        <x:v>Upper bound of a frontier-lab demand concentration estimate; it does not measure personal-AI inference supply.</x:v>
+      </x:c>
+      <x:c r="M15" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A16" s="16" t="str">
+        <x:v>frontier-lab-inference-allocation-2026</x:v>
+      </x:c>
+      <x:c r="B16" s="16" t="str">
+        <x:v>Frontier-lab compute allocated to inference</x:v>
+      </x:c>
+      <x:c r="C16" s="16" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E16" s="16" t="str">
+        <x:v>Current OpenAI and Anthropic compute budget</x:v>
+      </x:c>
+      <x:c r="F16" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G16" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H16" s="16" t="str">
+        <x:v>current allocation estimate</x:v>
+      </x:c>
+      <x:c r="I16" s="16" t="str">
+        <x:v>40:58</x:v>
+      </x:c>
+      <x:c r="J16" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K16" s="16" t="str">
+        <x:v>Frontier labs have allocated about 40% of compute to inference.</x:v>
+      </x:c>
+      <x:c r="L16" s="16" t="str">
+        <x:v>Lab-budget estimate, not a U.S.-fleet measurement and not the model's editable share of inference capacity allocated to personal AI.</x:v>
+      </x:c>
+      <x:c r="M16" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="108" hidden="0" customHeight="1">
+      <x:c r="A17" s="16" t="str">
+        <x:v>frontier-lab-research-allocation-2026</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>Frontier-lab compute allocated to research</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E17" s="16" t="str">
+        <x:v>Current OpenAI and Anthropic compute budget</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G17" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H17" s="16" t="str">
+        <x:v>current allocation estimate</x:v>
+      </x:c>
+      <x:c r="I17" s="16" t="str">
+        <x:v>40:58</x:v>
+      </x:c>
+      <x:c r="J17" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K17" s="16" t="str">
+        <x:v>Frontier labs have allocated about 50% of compute to research.</x:v>
+      </x:c>
+      <x:c r="L17" s="16" t="str">
+        <x:v>Lab-budget estimate, not a U.S.-fleet measurement; categories reflect the interviewee's definitions.</x:v>
+      </x:c>
+      <x:c r="M17" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="108" hidden="0" customHeight="1">
+      <x:c r="A18" s="16" t="str">
+        <x:v>frontier-lab-development-allocation-2026</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="str">
+        <x:v>Frontier-lab compute allocated to development</x:v>
+      </x:c>
+      <x:c r="C18" s="16" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D18" s="16" t="str">
+        <x:v>proportion</x:v>
+      </x:c>
+      <x:c r="E18" s="16" t="str">
+        <x:v>Current OpenAI and Anthropic compute budget</x:v>
+      </x:c>
+      <x:c r="F18" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H18" s="16" t="str">
+        <x:v>current allocation estimate</x:v>
+      </x:c>
+      <x:c r="I18" s="16" t="str">
+        <x:v>40:58</x:v>
+      </x:c>
+      <x:c r="J18" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K18" s="16" t="str">
+        <x:v>Frontier labs have allocated about 10% of compute to development.</x:v>
+      </x:c>
+      <x:c r="L18" s="16" t="str">
+        <x:v>Lab-budget estimate, not a U.S.-fleet measurement; categories reflect the interviewee's definitions.</x:v>
+      </x:c>
+      <x:c r="M18" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A19" s="16" t="str">
+        <x:v>new-chip-performance-per-watt-uplift-lower</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="str">
+        <x:v>New-chip performance-per-watt uplift</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D19" s="16" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E19" s="16" t="str">
+        <x:v>New chips versus chips deployed two years earlier</x:v>
+      </x:c>
+      <x:c r="F19" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H19" s="16" t="str">
+        <x:v>range lower bound</x:v>
+      </x:c>
+      <x:c r="I19" s="16" t="str">
+        <x:v>06:20</x:v>
+      </x:c>
+      <x:c r="J19" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K19" s="16" t="str">
+        <x:v>New chips deliver 3–5× more performance per watt than chips deployed two years earlier.</x:v>
+      </x:c>
+      <x:c r="L19" s="16" t="str">
+        <x:v>Lower bound across heterogeneous accelerators and workloads; H100e normalization may already capture part of this gain.</x:v>
+      </x:c>
+      <x:c r="M19" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A20" s="16" t="str">
+        <x:v>new-chip-performance-per-watt-uplift-upper</x:v>
+      </x:c>
+      <x:c r="B20" s="16" t="str">
+        <x:v>New-chip performance-per-watt uplift</x:v>
+      </x:c>
+      <x:c r="C20" s="16" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D20" s="16" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E20" s="16" t="str">
+        <x:v>New chips versus chips deployed two years earlier</x:v>
+      </x:c>
+      <x:c r="F20" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="G20" s="16" t="str">
+        <x:v>expert-estimate</x:v>
+      </x:c>
+      <x:c r="H20" s="16" t="str">
+        <x:v>range upper bound</x:v>
+      </x:c>
+      <x:c r="I20" s="16" t="str">
+        <x:v>06:20</x:v>
+      </x:c>
+      <x:c r="J20" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="K20" s="16" t="str">
+        <x:v>New chips deliver 3–5× more performance per watt than chips deployed two years earlier.</x:v>
+      </x:c>
+      <x:c r="L20" s="16" t="str">
+        <x:v>Upper bound across heterogeneous accelerators and workloads; H100e normalization may already capture part of this gain.</x:v>
+      </x:c>
+      <x:c r="M20" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M2"/>
+    <x:mergeCell ref="A3:M3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b2ca95cf3dd450c"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2213,49 +2972,72 @@
         <x:v>Holds definitions and assumptions that are authored by the forecast rather than fetched as observations.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="140.39999389648438" hidden="0" customHeight="1">
+    <x:row r="7" ht="291.6000061035156" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
+        <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>Dwarkesh Podcast</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>Dylan Patel – Anthropic &amp; OpenAI will have most of the world’s compute by 2028</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>capacity outlook, allocation cross-check, supply constraint context</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>https://www.dwarkesh.com/p/dylan-patel-3</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>Expert-interview estimates from Dylan Patel of SemiAnalysis. The official transcript accompanies the video at https://www.youtube.com/watch?v=aV26V1UvkJw. Global GW flows and frontier-lab allocations are not directly merged with the U.S. H100e countdown path.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="B7" s="16" t="str">
+      <x:c r="B8" s="16" t="str">
         <x:v>Epoch AI</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="str">
+      <x:c r="C8" s="16" t="str">
         <x:v>AI Data Center Timelines CSV</x:v>
       </x:c>
-      <x:c r="D7" s="16" t="str">
+      <x:c r="D8" s="16" t="str">
         <x:v>2026-08-25</x:v>
       </x:c>
-      <x:c r="E7" s="16" t="str">
+      <x:c r="E8" s="16" t="str">
         <x:v>capacity observation, capacity projection</x:v>
       </x:c>
-      <x:c r="F7" s="16" t="str">
+      <x:c r="F8" s="16" t="str">
         <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
       </x:c>
-      <x:c r="G7" s="16" t="str">
+      <x:c r="G8" s="16" t="str">
         <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="97.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A8" s="16" t="str">
+    <x:row r="9" ht="97.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A9" s="16" t="str">
         <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
-      <x:c r="B8" s="16" t="str">
+      <x:c r="B9" s="16" t="str">
         <x:v>U.S. Census Bureau</x:v>
       </x:c>
-      <x:c r="C8" s="16" t="str">
+      <x:c r="C9" s="16" t="str">
         <x:v>Population on a Date</x:v>
       </x:c>
-      <x:c r="D8" s="16" t="str">
+      <x:c r="D9" s="16" t="str">
         <x:v>2026-07-26</x:v>
       </x:c>
-      <x:c r="E8" s="16" t="str">
+      <x:c r="E9" s="16" t="str">
         <x:v>population</x:v>
       </x:c>
-      <x:c r="F8" s="16" t="str">
+      <x:c r="F9" s="16" t="str">
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
-      <x:c r="G8" s="16" t="str">
+      <x:c r="G9" s="16" t="str">
         <x:v>The model uses the rounded estimate of 342.8M residents; the selected 25% target is 85.7M users.</x:v>
       </x:c>
     </x:row>
@@ -2266,7 +3048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R474abccf99074d69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74abcd047adb4503"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Model compute as power times inference productivity
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R66430a2dcd3f4a7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R3dc75373423f44e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Ra516bff1d1514981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="4" r:id="R6402821b61f84997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R86a0a7989c7641ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdc804ad509144c49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R2f32dad36a8a4433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R78776243a84f4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="4" r:id="R084aaf8ffdb64308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="5" r:id="R3b5bba938faf444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rf97b19625c8c4a1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,12 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="202" formatCode="#,##0"/>
-    <x:numFmt numFmtId="203" formatCode="0.000"/>
-    <x:numFmt numFmtId="204" formatCode="0%"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="203" formatCode="0.0000"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0"/>
+    <x:numFmt numFmtId="205" formatCode="0%"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -95,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -153,6 +155,9 @@
     <x:xf numFmtId="204" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -172,7 +177,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>U.S. operational H100-equivalent capacity</a:t>
+              <a:t>Supported Personal-AI user-equivalents</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -187,7 +192,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>U.S. H100e</c:v>
+            <c:v>Supported users</c:v>
           </c:tx>
           <c:marker>
             <c:symbol val="none"/>
@@ -202,7 +207,35 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Quarterly Model'!$E$6:$E$25</c:f>
+              <c:f>'Quarterly Model'!$P$6:$P$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Selected target</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Quarterly Model'!$B$6:$B$25</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Quarterly Model'!$Q$6:$Q$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
@@ -271,6 +304,10 @@
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
@@ -288,13 +325,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -310,7 +347,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7c99044c73d467e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R918d344b1ee641f4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -320,7 +357,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComputeSummaryTable" displayName="ComputeSummaryTable" ref="A5:C17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComputeSummaryTable" displayName="ComputeSummaryTable" ref="A5:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Metric"/>
     <x:tableColumn id="2" name="Value"/>
@@ -331,23 +368,30 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComputeQuarterlyModelTable" displayName="ComputeQuarterlyModelTable" ref="A5:O25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComputeQuarterlyModelTable" displayName="ComputeQuarterlyModelTable" ref="A5:V25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="22">
     <x:tableColumn id="1" name="Quarter index"/>
     <x:tableColumn id="2" name="Quarter"/>
     <x:tableColumn id="3" name="Cutoff"/>
     <x:tableColumn id="4" name="Phase"/>
-    <x:tableColumn id="5" name="U.S. H100e"/>
-    <x:tableColumn id="6" name="Included sites"/>
-    <x:tableColumn id="7" name="log₂ H100e"/>
-    <x:tableColumn id="8" name="Log growth / quarter"/>
-    <x:tableColumn id="9" name="Compute-equivalent tokens/day"/>
-    <x:tableColumn id="10" name="Supported users"/>
-    <x:tableColumn id="11" name="Score vs target"/>
-    <x:tableColumn id="12" name="Letter"/>
-    <x:tableColumn id="13" name="GPA"/>
-    <x:tableColumn id="14" name="Source ID"/>
-    <x:tableColumn id="15" name="Method note"/>
+    <x:tableColumn id="5" name="U.S. IT power MW"/>
+    <x:tableColumn id="6" name="U.S. IT power GW"/>
+    <x:tableColumn id="7" name="U.S. facility power MW"/>
+    <x:tableColumn id="8" name="H100e audit bridge"/>
+    <x:tableColumn id="9" name="Included sites"/>
+    <x:tableColumn id="10" name="H100e / IT GW"/>
+    <x:tableColumn id="11" name="Productivity T token-eq / IT GW-day"/>
+    <x:tableColumn id="12" name="IT-power log growth / qtr"/>
+    <x:tableColumn id="13" name="Productivity log growth / qtr"/>
+    <x:tableColumn id="14" name="H100e log growth / qtr"/>
+    <x:tableColumn id="15" name="Personal-AI token-eq/day"/>
+    <x:tableColumn id="16" name="Supported users"/>
+    <x:tableColumn id="17" name="Target users"/>
+    <x:tableColumn id="18" name="Score vs target"/>
+    <x:tableColumn id="19" name="Letter"/>
+    <x:tableColumn id="20" name="GPA"/>
+    <x:tableColumn id="21" name="Source ID"/>
+    <x:tableColumn id="22" name="Method note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -366,7 +410,23 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSiteRegistryTable" displayName="ComputeSiteRegistryTable" ref="A5:H88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Site"/>
+    <x:tableColumn id="2" name="Country"/>
+    <x:tableColumn id="3" name="Current H100e"/>
+    <x:tableColumn id="4" name="Current facility power MW"/>
+    <x:tableColumn id="5" name="Owner"/>
+    <x:tableColumn id="6" name="Users"/>
+    <x:tableColumn id="7" name="Address"/>
+    <x:tableColumn id="8" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Metric"/>
@@ -386,8 +446,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -603,7 +663,7 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Compute Supply Report Card</x:v>
+        <x:v>U.S. Service-Capacity Report Card</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -613,9 +673,9 @@
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
     </x:row>
-    <x:row r="3" ht="48" hidden="0" customHeight="1">
+    <x:row r="3" ht="72" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Snapshot 2026-08-26. The supply gate passes only when modeled U.S. capacity can serve 100% of the selected target population.</x:v>
+        <x:v>Snapshot 2026-08-26. The supply gate combines operational IT power, inference productivity, allocation, and workload; it passes only at 100% of the selected population target.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -645,122 +705,166 @@
     </x:row>
     <x:row r="7" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A7" s="19" t="str">
-        <x:v>Current U.S. operational capacity</x:v>
+        <x:v>Current U.S. operational IT power</x:v>
       </x:c>
       <x:c r="B7" s="19" t="n">
+        <x:v>11.87932971</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="str">
+        <x:v>IT GW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" hidden="0" customHeight="1">
+      <x:c r="A8" s="19" t="str">
+        <x:v>Current reference inference productivity</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="n">
+        <x:v>227.10136510717322</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>trillion reference token-equivalents / IT GW-day</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A9" s="19" t="str">
+        <x:v>Current H100e audit bridge</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="n">
         <x:v>13524006</x:v>
       </x:c>
-      <x:c r="C7" s="19" t="str">
-        <x:v>H100-equivalents</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A8" s="19" t="str">
+      <x:c r="C9" s="19" t="str">
+        <x:v>secondary productivity calibration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A10" s="19" t="str">
         <x:v>Current supported users</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="B10" s="19" t="n">
         <x:v>38655216.62613779</x:v>
       </x:c>
-      <x:c r="C8" s="19" t="str">
-        <x:v>high-autonomy users</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A9" s="19" t="str">
+      <x:c r="C10" s="19" t="str">
+        <x:v>Personal-AI user-equivalents</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A11" s="19" t="str">
         <x:v>Target users</x:v>
       </x:c>
-      <x:c r="B9" s="19" t="n">
+      <x:c r="B11" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="C9" s="19" t="str">
+      <x:c r="C11" s="19" t="str">
         <x:v>25% of U.S. population</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A10" s="19" t="str">
-        <x:v>Required U.S. capacity</x:v>
-      </x:c>
-      <x:c r="B10" s="19" t="n">
-        <x:v>29983205.770377323</x:v>
-      </x:c>
-      <x:c r="C10" s="19" t="str">
-        <x:v>H100-equivalents</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A11" s="19" t="str">
-        <x:v>Current supply score</x:v>
-      </x:c>
-      <x:c r="B11" s="20" t="n">
-        <x:v>0.45105270275540016</x:v>
-      </x:c>
-      <x:c r="C11" s="19" t="str">
-        <x:v>supported users / target users</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A12" s="19" t="str">
-        <x:v>Personal-AI inference share</x:v>
+        <x:v>Current supply score</x:v>
       </x:c>
       <x:c r="B12" s="20" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.45105270275540016</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>scenario allocation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="32.400001525878906" hidden="0" customHeight="1">
+        <x:v>supported users / target users</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" hidden="0" customHeight="1">
       <x:c r="A13" s="19" t="str">
-        <x:v>Workload per user/day</x:v>
+        <x:v>Reference tokens per H100e/day</x:v>
       </x:c>
       <x:c r="B13" s="19" t="n">
-        <x:v>16750000</x:v>
+        <x:v>199483200</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:v>compute-equivalent tokens</x:v>
+        <x:v>excludes inference and Personal-AI allocations</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="str">
-        <x:v>Tokens per H100e/day</x:v>
+        <x:v>Workload per user/day</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:v>47875968</x:v>
+        <x:v>16750000</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>after personal-AI allocation</x:v>
+        <x:v>compute-equivalent tokens</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A15" s="19" t="str">
-        <x:v>Mean projected log velocity</x:v>
-      </x:c>
-      <x:c r="B15" s="19" t="n">
-        <x:v>0.24379055731655638</x:v>
+        <x:v>Fleet inference allocation</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="n">
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:v>log₂ H100e / quarter</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32.400001525878906" hidden="0" customHeight="1">
+        <x:v>scenario allocation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A16" s="19" t="str">
-        <x:v>Projected log acceleration</x:v>
-      </x:c>
-      <x:c r="B16" s="19" t="n">
-        <x:v>0.0033726529962799273</x:v>
+        <x:v>Personal-AI inference share</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="n">
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>log₂ H100e / quarter²</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
+        <x:v>share of inference allocated to Personal AI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A17" s="19" t="str">
+        <x:v>IT-power mean projected log velocity</x:v>
+      </x:c>
+      <x:c r="B17" s="19" t="n">
+        <x:v>0.15720673944051156</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="str">
+        <x:v>log₂ IT GW / quarter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A18" s="19" t="str">
+        <x:v>IT-power projected log acceleration</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="n">
+        <x:v>-0.0015030413270408216</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>log₂ IT GW / quarter²</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A19" s="19" t="str">
+        <x:v>Productivity mean projected log velocity</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="n">
+        <x:v>0.08658381787604459</x:v>
+      </x:c>
+      <x:c r="C19" s="19" t="str">
+        <x:v>log₂ token productivity / quarter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A20" s="19" t="str">
+        <x:v>Productivity projected log acceleration</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="n">
+        <x:v>0.004875694323320446</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>log₂ token productivity / quarter²</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A21" s="19" t="str">
         <x:v>Continuous base-case crossing</x:v>
       </x:c>
-      <x:c r="B17" s="21" t="n">
-        <x:v>46750.994524664355</x:v>
-      </x:c>
-      <x:c r="C17" s="19" t="str">
+      <x:c r="B21" s="21" t="n">
+        <x:v>46751.054552650465</x:v>
+      </x:c>
+      <x:c r="C21" s="19" t="str">
         <x:v>100% of selected target</x:v>
       </x:c>
     </x:row>
@@ -771,7 +875,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R400a7f84d36c4d74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21c61a0b63024c85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -785,31 +889,38 @@
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="9" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="9" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="55" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="3" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="3" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="3" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="3" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="3" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="3" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="3" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="9" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="9" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="58" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="3" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="3" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="3" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="3" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="3" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="3" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="3" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="3" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="3" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="3" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>U.S. Compute Capacity — Observed and Projected</x:v>
+        <x:v>U.S. AI Service Capacity — Observed and Projected</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -825,6 +936,13 @@
       <x:c r="M1" s="3"/>
       <x:c r="N1" s="3"/>
       <x:c r="O1" s="3"/>
+      <x:c r="P1" s="3"/>
+      <x:c r="Q1" s="3"/>
+      <x:c r="R1" s="3"/>
+      <x:c r="S1" s="3"/>
+      <x:c r="T1" s="3"/>
+      <x:c r="U1" s="3"/>
+      <x:c r="V1" s="3"/>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3"/>
@@ -842,10 +960,17 @@
       <x:c r="M2" s="3"/>
       <x:c r="N2" s="3"/>
       <x:c r="O2" s="3"/>
+      <x:c r="P2" s="3"/>
+      <x:c r="Q2" s="3"/>
+      <x:c r="R2" s="3"/>
+      <x:c r="S2" s="3"/>
+      <x:c r="T2" s="3"/>
+      <x:c r="U2" s="3"/>
+      <x:c r="V2" s="3"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Quarterly operational H100-equivalent supply from the selected snapshot, translated to supported users under the visible serving envelope.</x:v>
+        <x:v>Quarterly IT power and reference-token productivity from the selected snapshot, translated to supported Personal-AI user-equivalents. H100e remains a secondary audit bridge.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -861,6 +986,13 @@
       <x:c r="M3" s="6"/>
       <x:c r="N3" s="6"/>
       <x:c r="O3" s="6"/>
+      <x:c r="P3" s="6"/>
+      <x:c r="Q3" s="6"/>
+      <x:c r="R3" s="6"/>
+      <x:c r="S3" s="6"/>
+      <x:c r="T3" s="6"/>
+      <x:c r="U3" s="6"/>
+      <x:c r="V3" s="6"/>
     </x:row>
     <x:row r="4"/>
     <x:row r="5" ht="66" hidden="0" customHeight="1">
@@ -877,40 +1009,61 @@
         <x:v>Phase</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>U.S. H100e</x:v>
+        <x:v>U.S. IT power MW</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
+        <x:v>U.S. IT power GW</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>U.S. facility power MW</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>H100e audit bridge</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
         <x:v>Included sites</x:v>
       </x:c>
-      <x:c r="G5" s="12" t="str">
-        <x:v>log₂ H100e</x:v>
-      </x:c>
-      <x:c r="H5" s="12" t="str">
-        <x:v>Log growth / quarter</x:v>
-      </x:c>
-      <x:c r="I5" s="12" t="str">
-        <x:v>Compute-equivalent tokens/day</x:v>
-      </x:c>
       <x:c r="J5" s="12" t="str">
+        <x:v>H100e / IT GW</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="str">
+        <x:v>Productivity T token-eq / IT GW-day</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="str">
+        <x:v>IT-power log growth / qtr</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>Productivity log growth / qtr</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>H100e log growth / qtr</x:v>
+      </x:c>
+      <x:c r="O5" s="12" t="str">
+        <x:v>Personal-AI token-eq/day</x:v>
+      </x:c>
+      <x:c r="P5" s="12" t="str">
         <x:v>Supported users</x:v>
       </x:c>
-      <x:c r="K5" s="12" t="str">
+      <x:c r="Q5" s="12" t="str">
+        <x:v>Target users</x:v>
+      </x:c>
+      <x:c r="R5" s="12" t="str">
         <x:v>Score vs target</x:v>
       </x:c>
-      <x:c r="L5" s="12" t="str">
+      <x:c r="S5" s="12" t="str">
         <x:v>Letter</x:v>
       </x:c>
-      <x:c r="M5" s="12" t="str">
+      <x:c r="T5" s="12" t="str">
         <x:v>GPA</x:v>
       </x:c>
-      <x:c r="N5" s="12" t="str">
+      <x:c r="U5" s="12" t="str">
         <x:v>Source ID</x:v>
       </x:c>
-      <x:c r="O5" s="12" t="str">
+      <x:c r="V5" s="12" t="str">
         <x:v>Method note</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="75.5999984741211" hidden="0" customHeight="1">
+    <x:row r="6" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -924,38 +1077,55 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E6" s="22" t="n">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="n">
+        <x:v>0.473</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="n">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="n">
         <x:v>245664</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
+      <x:c r="I6" s="22" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G6" s="23" t="n">
-        <x:v>17.906326932760603</x:v>
-      </x:c>
-      <x:c r="H6" s="23"/>
-      <x:c r="I6" s="22" t="n">
+      <x:c r="J6" s="22" t="n">
+        <x:v>519374.2071881607</x:v>
+      </x:c>
+      <x:c r="K6" s="23" t="n">
+        <x:v>103.6064288473573</x:v>
+      </x:c>
+      <x:c r="L6" s="23"/>
+      <x:c r="M6" s="23"/>
+      <x:c r="N6" s="23"/>
+      <x:c r="O6" s="24" t="n">
         <x:v>11761401802752</x:v>
       </x:c>
-      <x:c r="J6" s="22" t="n">
+      <x:c r="P6" s="24" t="n">
         <x:v>702173.2419553433</x:v>
       </x:c>
-      <x:c r="K6" s="17" t="n">
+      <x:c r="Q6" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R6" s="17" t="n">
         <x:v>0.008193386720599105</x:v>
       </x:c>
-      <x:c r="L6" s="16" t="str">
+      <x:c r="S6" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M6" s="16" t="n">
+      <x:c r="T6" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N6" s="16" t="str">
+      <x:c r="U6" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O6" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V6" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -969,40 +1139,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E7" s="22" t="n">
+        <x:v>887</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:v>0.887</x:v>
+      </x:c>
+      <x:c r="G7" s="22" t="n">
+        <x:v>1121</x:v>
+      </x:c>
+      <x:c r="H7" s="22" t="n">
         <x:v>475238</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="n">
+      <x:c r="I7" s="22" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G7" s="23" t="n">
-        <x:v>18.858290672990677</x:v>
-      </x:c>
-      <x:c r="H7" s="23" t="n">
+      <x:c r="J7" s="22" t="n">
+        <x:v>535781.2852311161</x:v>
+      </x:c>
+      <x:c r="K7" s="23" t="n">
+        <x:v>106.87936527801578</x:v>
+      </x:c>
+      <x:c r="L7" s="23" t="n">
+        <x:v>0.9070939209616689</x:v>
+      </x:c>
+      <x:c r="M7" s="23" t="n">
+        <x:v>0.044869819268406275</x:v>
+      </x:c>
+      <x:c r="N7" s="23" t="n">
         <x:v>0.9519637402300738</x:v>
       </x:c>
-      <x:c r="I7" s="22" t="n">
+      <x:c r="O7" s="24" t="n">
         <x:v>22752479280384</x:v>
       </x:c>
-      <x:c r="J7" s="22" t="n">
+      <x:c r="P7" s="24" t="n">
         <x:v>1358356.9719632238</x:v>
       </x:c>
-      <x:c r="K7" s="17" t="n">
+      <x:c r="Q7" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R7" s="17" t="n">
         <x:v>0.015850139696186975</x:v>
       </x:c>
-      <x:c r="L7" s="16" t="str">
+      <x:c r="S7" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M7" s="16" t="n">
+      <x:c r="T7" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N7" s="16" t="str">
+      <x:c r="U7" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O7" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V7" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1016,40 +1207,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
+        <x:v>1335</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:v>1.335</x:v>
+      </x:c>
+      <x:c r="G8" s="22" t="n">
+        <x:v>1676</x:v>
+      </x:c>
+      <x:c r="H8" s="22" t="n">
         <x:v>722180</x:v>
       </x:c>
-      <x:c r="F8" s="22" t="n">
+      <x:c r="I8" s="22" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G8" s="23" t="n">
-        <x:v>19.46199894138585</x:v>
-      </x:c>
-      <x:c r="H8" s="23" t="n">
+      <x:c r="J8" s="22" t="n">
+        <x:v>540958.8014981274</x:v>
+      </x:c>
+      <x:c r="K8" s="23" t="n">
+        <x:v>107.91219279101125</x:v>
+      </x:c>
+      <x:c r="L8" s="23" t="n">
+        <x:v>0.5898337322738523</x:v>
+      </x:c>
+      <x:c r="M8" s="23" t="n">
+        <x:v>0.013874536121321057</x:v>
+      </x:c>
+      <x:c r="N8" s="23" t="n">
         <x:v>0.6037082683951738</x:v>
       </x:c>
-      <x:c r="I8" s="22" t="n">
+      <x:c r="O8" s="24" t="n">
         <x:v>34575066570240</x:v>
       </x:c>
-      <x:c r="J8" s="22" t="n">
+      <x:c r="P8" s="24" t="n">
         <x:v>2064183.0788202984</x:v>
       </x:c>
-      <x:c r="K8" s="17" t="n">
+      <x:c r="Q8" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R8" s="17" t="n">
         <x:v>0.024086150277949806</x:v>
       </x:c>
-      <x:c r="L8" s="16" t="str">
+      <x:c r="S8" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M8" s="16" t="n">
+      <x:c r="T8" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N8" s="16" t="str">
+      <x:c r="U8" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O8" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V8" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -1063,40 +1275,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
+        <x:v>1713</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>1.713</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>2165</x:v>
+      </x:c>
+      <x:c r="H9" s="22" t="n">
         <x:v>1012483</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="n">
+      <x:c r="I9" s="22" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="G9" s="23" t="n">
-        <x:v>19.949466254090233</x:v>
-      </x:c>
-      <x:c r="H9" s="23" t="n">
+      <x:c r="J9" s="22" t="n">
+        <x:v>591058.3771161705</x:v>
+      </x:c>
+      <x:c r="K9" s="23" t="n">
+        <x:v>117.90621645394046</x:v>
+      </x:c>
+      <x:c r="L9" s="23" t="n">
+        <x:v>0.35968540950908284</x:v>
+      </x:c>
+      <x:c r="M9" s="23" t="n">
+        <x:v>0.1277819031953058</x:v>
+      </x:c>
+      <x:c r="N9" s="23" t="n">
         <x:v>0.48746731270438204</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="n">
+      <x:c r="O9" s="24" t="n">
         <x:v>48473603708544</x:v>
       </x:c>
-      <x:c r="J9" s="22" t="n">
+      <x:c r="P9" s="24" t="n">
         <x:v>2893946.4900623285</x:v>
       </x:c>
-      <x:c r="K9" s="17" t="n">
+      <x:c r="Q9" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R9" s="17" t="n">
         <x:v>0.03376833710691165</x:v>
       </x:c>
-      <x:c r="L9" s="16" t="str">
+      <x:c r="S9" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M9" s="16" t="n">
+      <x:c r="T9" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N9" s="16" t="str">
+      <x:c r="U9" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O9" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V9" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -1110,40 +1343,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
+        <x:v>2267.32971</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="n">
+        <x:v>2.26732971</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="n">
+        <x:v>2874</x:v>
+      </x:c>
+      <x:c r="H10" s="22" t="n">
         <x:v>1351240</x:v>
       </x:c>
-      <x:c r="F10" s="22" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G10" s="23" t="n">
-        <x:v>20.365852510500535</x:v>
-      </x:c>
-      <x:c r="H10" s="23" t="n">
+      <x:c r="I10" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J10" s="22" t="n">
+        <x:v>595960.9641422641</x:v>
+      </x:c>
+      <x:c r="K10" s="23" t="n">
+        <x:v>118.88420020218409</x:v>
+      </x:c>
+      <x:c r="L10" s="23" t="n">
+        <x:v>0.4044690483884812</x:v>
+      </x:c>
+      <x:c r="M10" s="23" t="n">
+        <x:v>0.011917208021813508</x:v>
+      </x:c>
+      <x:c r="N10" s="23" t="n">
         <x:v>0.416386256410302</x:v>
       </x:c>
-      <x:c r="I10" s="22" t="n">
+      <x:c r="O10" s="24" t="n">
         <x:v>64691923000320</x:v>
       </x:c>
-      <x:c r="J10" s="22" t="n">
+      <x:c r="P10" s="24" t="n">
         <x:v>3862204.3582280595</x:v>
       </x:c>
-      <x:c r="K10" s="17" t="n">
+      <x:c r="Q10" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R10" s="17" t="n">
         <x:v>0.04506656193965063</x:v>
       </x:c>
-      <x:c r="L10" s="16" t="str">
+      <x:c r="S10" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M10" s="16" t="n">
+      <x:c r="T10" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N10" s="16" t="str">
+      <x:c r="U10" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O10" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V10" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -1157,40 +1411,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
+        <x:v>3342.32971</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>3.34232971</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>4187</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="n">
         <x:v>2386876</x:v>
       </x:c>
-      <x:c r="F11" s="22" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="G11" s="23" t="n">
-        <x:v>21.18669218860024</x:v>
-      </x:c>
-      <x:c r="H11" s="23" t="n">
+      <x:c r="I11" s="22" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="J11" s="22" t="n">
+        <x:v>714135.410656419</x:v>
+      </x:c>
+      <x:c r="K11" s="23" t="n">
+        <x:v>142.45801695105655</x:v>
+      </x:c>
+      <x:c r="L11" s="23" t="n">
+        <x:v>0.5598598578015919</x:v>
+      </x:c>
+      <x:c r="M11" s="23" t="n">
+        <x:v>0.26097982029811817</x:v>
+      </x:c>
+      <x:c r="N11" s="23" t="n">
         <x:v>0.8208396780997056</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="n">
+      <x:c r="O11" s="24" t="n">
         <x:v>114273998995968</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="n">
+      <x:c r="P11" s="24" t="n">
         <x:v>6822328.298266746</x:v>
       </x:c>
-      <x:c r="K11" s="17" t="n">
+      <x:c r="Q11" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R11" s="17" t="n">
         <x:v>0.07960709799611139</x:v>
       </x:c>
-      <x:c r="L11" s="16" t="str">
+      <x:c r="S11" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M11" s="16" t="n">
+      <x:c r="T11" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N11" s="16" t="str">
+      <x:c r="U11" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O11" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V11" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A12" s="16" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -1204,40 +1479,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
+        <x:v>3772.32971</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>3.77232971</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>4764</x:v>
+      </x:c>
+      <x:c r="H12" s="22" t="n">
         <x:v>3139660</x:v>
       </x:c>
-      <x:c r="F12" s="22" t="n">
+      <x:c r="I12" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="G12" s="23" t="n">
-        <x:v>21.582176904596352</x:v>
-      </x:c>
-      <x:c r="H12" s="23" t="n">
+      <x:c r="J12" s="22" t="n">
+        <x:v>832286.7409169279</x:v>
+      </x:c>
+      <x:c r="K12" s="23" t="n">
+        <x:v>166.02722239567973</x:v>
+      </x:c>
+      <x:c r="L12" s="23" t="n">
+        <x:v>0.17460171866453855</x:v>
+      </x:c>
+      <x:c r="M12" s="23" t="n">
+        <x:v>0.22088299733157157</x:v>
+      </x:c>
+      <x:c r="N12" s="23" t="n">
         <x:v>0.3954847159961119</x:v>
       </x:c>
-      <x:c r="I12" s="22" t="n">
+      <x:c r="O12" s="24" t="n">
         <x:v>150314261690880</x:v>
       </x:c>
-      <x:c r="J12" s="22" t="n">
+      <x:c r="P12" s="24" t="n">
         <x:v>8973985.772589851</x:v>
       </x:c>
-      <x:c r="K12" s="17" t="n">
+      <x:c r="Q12" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R12" s="17" t="n">
         <x:v>0.10471395300571588</x:v>
       </x:c>
-      <x:c r="L12" s="16" t="str">
+      <x:c r="S12" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M12" s="16" t="n">
+      <x:c r="T12" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N12" s="16" t="str">
+      <x:c r="U12" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O12" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V12" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A13" s="16" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -1251,40 +1547,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
+        <x:v>5642.32971</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>5.64232971</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>7211</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="n">
         <x:v>5291375</x:v>
       </x:c>
-      <x:c r="F13" s="22" t="n">
+      <x:c r="I13" s="22" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G13" s="23" t="n">
-        <x:v>22.335211234559345</x:v>
-      </x:c>
-      <x:c r="H13" s="23" t="n">
+      <x:c r="J13" s="22" t="n">
+        <x:v>937799.6806216416</x:v>
+      </x:c>
+      <x:c r="K13" s="23" t="n">
+        <x:v>187.07528124938307</x:v>
+      </x:c>
+      <x:c r="L13" s="23" t="n">
+        <x:v>0.580835196113413</x:v>
+      </x:c>
+      <x:c r="M13" s="23" t="n">
+        <x:v>0.1721991338495812</x:v>
+      </x:c>
+      <x:c r="N13" s="23" t="n">
         <x:v>0.7530343299629934</x:v>
       </x:c>
-      <x:c r="I13" s="22" t="n">
+      <x:c r="O13" s="24" t="n">
         <x:v>253329700176000</x:v>
       </x:c>
-      <x:c r="J13" s="22" t="n">
+      <x:c r="P13" s="24" t="n">
         <x:v>15124161.204537313</x:v>
       </x:c>
-      <x:c r="K13" s="17" t="n">
+      <x:c r="Q13" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R13" s="17" t="n">
         <x:v>0.17647796037966526</x:v>
       </x:c>
-      <x:c r="L13" s="16" t="str">
+      <x:c r="S13" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M13" s="16" t="n">
+      <x:c r="T13" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N13" s="16" t="str">
+      <x:c r="U13" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O13" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V13" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A14" s="16" t="n">
         <x:v>9</x:v>
       </x:c>
@@ -1298,40 +1615,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
+        <x:v>6620.32971</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>6.62032971</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>8454.2</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="n">
         <x:v>6301294</x:v>
       </x:c>
-      <x:c r="F14" s="22" t="n">
+      <x:c r="I14" s="22" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G14" s="23" t="n">
-        <x:v>22.587216692490205</x:v>
-      </x:c>
-      <x:c r="H14" s="23" t="n">
+      <x:c r="J14" s="22" t="n">
+        <x:v>951809.6946866412</x:v>
+      </x:c>
+      <x:c r="K14" s="23" t="n">
+        <x:v>189.8700436871142</x:v>
+      </x:c>
+      <x:c r="L14" s="23" t="n">
+        <x:v>0.2306120964759244</x:v>
+      </x:c>
+      <x:c r="M14" s="23" t="n">
+        <x:v>0.021393361454933313</x:v>
+      </x:c>
+      <x:c r="N14" s="23" t="n">
         <x:v>0.25200545793085993</x:v>
       </x:c>
-      <x:c r="I14" s="22" t="n">
+      <x:c r="O14" s="24" t="n">
         <x:v>301680549902592</x:v>
       </x:c>
-      <x:c r="J14" s="22" t="n">
+      <x:c r="P14" s="24" t="n">
         <x:v>18010779.09866221</x:v>
       </x:c>
-      <x:c r="K14" s="17" t="n">
+      <x:c r="Q14" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R14" s="17" t="n">
         <x:v>0.21016078294821713</x:v>
       </x:c>
-      <x:c r="L14" s="16" t="str">
+      <x:c r="S14" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M14" s="16" t="n">
+      <x:c r="T14" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N14" s="16" t="str">
+      <x:c r="U14" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O14" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="V14" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A15" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -1345,40 +1683,61 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
+        <x:v>10534.32971</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>10.53432971</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>13559.8</x:v>
+      </x:c>
+      <x:c r="H15" s="22" t="n">
         <x:v>11223855</x:v>
       </x:c>
-      <x:c r="F15" s="22" t="n">
+      <x:c r="I15" s="22" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G15" s="23" t="n">
-        <x:v>23.420064940351462</x:v>
-      </x:c>
-      <x:c r="H15" s="23" t="n">
+      <x:c r="J15" s="22" t="n">
+        <x:v>1065455.0701356395</x:v>
+      </x:c>
+      <x:c r="K15" s="23" t="n">
+        <x:v>212.5403868468818</x:v>
+      </x:c>
+      <x:c r="L15" s="23" t="n">
+        <x:v>0.670123545698909</x:v>
+      </x:c>
+      <x:c r="M15" s="23" t="n">
+        <x:v>0.16272470216235035</x:v>
+      </x:c>
+      <x:c r="N15" s="23" t="n">
         <x:v>0.8328482478612571</x:v>
       </x:c>
-      <x:c r="I15" s="22" t="n">
-        <x:v>537352922816640</x:v>
-      </x:c>
-      <x:c r="J15" s="22" t="n">
-        <x:v>32080771.511441194</x:v>
-      </x:c>
-      <x:c r="K15" s="17" t="n">
-        <x:v>0.3743380573096989</x:v>
-      </x:c>
-      <x:c r="L15" s="16" t="str">
+      <x:c r="O15" s="24" t="n">
+        <x:v>537352922816640.06</x:v>
+      </x:c>
+      <x:c r="P15" s="24" t="n">
+        <x:v>32080771.511441197</x:v>
+      </x:c>
+      <x:c r="Q15" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R15" s="17" t="n">
+        <x:v>0.37433805730969893</x:v>
+      </x:c>
+      <x:c r="S15" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M15" s="16" t="n">
+      <x:c r="T15" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N15" s="16" t="str">
+      <x:c r="U15" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O15" s="16" t="str">
-        <x:v>Latest published state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="97.19999694824219" hidden="0" customHeight="1">
+      <x:c r="V15" s="16" t="str">
+        <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -1392,40 +1751,61 @@
         <x:v>observed_qtd</x:v>
       </x:c>
       <x:c r="E16" s="22" t="n">
+        <x:v>11879.32971</x:v>
+      </x:c>
+      <x:c r="F16" s="22" t="n">
+        <x:v>11.87932971</x:v>
+      </x:c>
+      <x:c r="G16" s="22" t="n">
+        <x:v>15229.8</x:v>
+      </x:c>
+      <x:c r="H16" s="22" t="n">
         <x:v>13524006</x:v>
       </x:c>
-      <x:c r="F16" s="22" t="n">
+      <x:c r="I16" s="22" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="G16" s="23" t="n">
-        <x:v>23.689019225615233</x:v>
-      </x:c>
-      <x:c r="H16" s="23" t="n">
+      <x:c r="J16" s="22" t="n">
+        <x:v>1138448.5766579502</x:v>
+      </x:c>
+      <x:c r="K16" s="23" t="n">
+        <x:v>227.10136510717322</x:v>
+      </x:c>
+      <x:c r="L16" s="23" t="n">
+        <x:v>0.1733549148332778</x:v>
+      </x:c>
+      <x:c r="M16" s="23" t="n">
+        <x:v>0.0955993704304916</x:v>
+      </x:c>
+      <x:c r="N16" s="23" t="n">
         <x:v>0.26895428526377074</x:v>
       </x:c>
-      <x:c r="I16" s="22" t="n">
+      <x:c r="O16" s="24" t="n">
         <x:v>647474878487808</x:v>
       </x:c>
-      <x:c r="J16" s="22" t="n">
+      <x:c r="P16" s="24" t="n">
         <x:v>38655216.62613779</x:v>
       </x:c>
-      <x:c r="K16" s="17" t="n">
+      <x:c r="Q16" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R16" s="17" t="n">
         <x:v>0.45105270275540016</x:v>
       </x:c>
-      <x:c r="L16" s="16" t="str">
+      <x:c r="S16" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M16" s="16" t="n">
+      <x:c r="T16" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N16" s="16" t="str">
+      <x:c r="U16" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O16" s="16" t="str">
-        <x:v>Latest published state on or before evidence cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V16" s="16" t="str">
+        <x:v>observed_qtd: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -1439,40 +1819,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
+        <x:v>14026.32971</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>14.02632971</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>18051.3</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
         <x:v>17399770</x:v>
       </x:c>
-      <x:c r="F17" s="22" t="n">
+      <x:c r="I17" s="22" t="n">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="G17" s="23" t="n">
-        <x:v>24.052564900052637</x:v>
-      </x:c>
-      <x:c r="H17" s="23" t="n">
+      <x:c r="J17" s="22" t="n">
+        <x:v>1240507.6994300885</x:v>
+      </x:c>
+      <x:c r="K17" s="23" t="n">
+        <x:v>247.46044550695223</x:v>
+      </x:c>
+      <x:c r="L17" s="23" t="n">
+        <x:v>0.23968411173075843</x:v>
+      </x:c>
+      <x:c r="M17" s="23" t="n">
+        <x:v>0.12386156270665083</x:v>
+      </x:c>
+      <x:c r="N17" s="23" t="n">
         <x:v>0.36354567443740393</x:v>
       </x:c>
-      <x:c r="I17" s="22" t="n">
+      <x:c r="O17" s="24" t="n">
         <x:v>833030831727360</x:v>
       </x:c>
-      <x:c r="J17" s="22" t="n">
+      <x:c r="P17" s="24" t="n">
         <x:v>49733183.983722985</x:v>
       </x:c>
-      <x:c r="K17" s="17" t="n">
+      <x:c r="Q17" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R17" s="17" t="n">
         <x:v>0.5803171993433254</x:v>
       </x:c>
-      <x:c r="L17" s="16" t="str">
+      <x:c r="S17" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M17" s="16" t="n">
+      <x:c r="T17" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N17" s="16" t="str">
+      <x:c r="U17" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O17" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V17" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="n">
         <x:v>13</x:v>
       </x:c>
@@ -1486,40 +1887,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
+        <x:v>16045.32971</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>16.04532971</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>20792.8</x:v>
+      </x:c>
+      <x:c r="H18" s="22" t="n">
         <x:v>20368064</x:v>
       </x:c>
-      <x:c r="F18" s="22" t="n">
+      <x:c r="I18" s="22" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="G18" s="23" t="n">
-        <x:v>24.279805521769333</x:v>
-      </x:c>
-      <x:c r="H18" s="23" t="n">
+      <x:c r="J18" s="22" t="n">
+        <x:v>1269407.6325091608</x:v>
+      </x:c>
+      <x:c r="K18" s="23" t="n">
+        <x:v>253.22549663735143</x:v>
+      </x:c>
+      <x:c r="L18" s="23" t="n">
+        <x:v>0.1940158891305166</x:v>
+      </x:c>
+      <x:c r="M18" s="23" t="n">
+        <x:v>0.0332247325861772</x:v>
+      </x:c>
+      <x:c r="N18" s="23" t="n">
         <x:v>0.227240621716696</x:v>
       </x:c>
-      <x:c r="I18" s="22" t="n">
-        <x:v>975140780285952</x:v>
-      </x:c>
-      <x:c r="J18" s="22" t="n">
-        <x:v>58217360.01707176</x:v>
-      </x:c>
-      <x:c r="K18" s="17" t="n">
-        <x:v>0.6793157528246413</x:v>
-      </x:c>
-      <x:c r="L18" s="16" t="str">
+      <x:c r="O18" s="24" t="n">
+        <x:v>975140780285952.1</x:v>
+      </x:c>
+      <x:c r="P18" s="24" t="n">
+        <x:v>58217360.01707177</x:v>
+      </x:c>
+      <x:c r="Q18" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R18" s="17" t="n">
+        <x:v>0.6793157528246414</x:v>
+      </x:c>
+      <x:c r="S18" s="16" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="M18" s="16" t="n">
+      <x:c r="T18" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N18" s="16" t="str">
+      <x:c r="U18" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O18" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V18" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A19" s="16" t="n">
         <x:v>14</x:v>
       </x:c>
@@ -1533,40 +1955,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
+        <x:v>16634.32971</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>16.634329710000003</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>21589.8</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
         <x:v>21439292</x:v>
       </x:c>
-      <x:c r="F19" s="22" t="n">
+      <x:c r="I19" s="22" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="G19" s="23" t="n">
-        <x:v>24.3537539279851</x:v>
-      </x:c>
-      <x:c r="H19" s="23" t="n">
+      <x:c r="J19" s="22" t="n">
+        <x:v>1288858.1850768183</x:v>
+      </x:c>
+      <x:c r="K19" s="23" t="n">
+        <x:v>257.10555510531594</x:v>
+      </x:c>
+      <x:c r="L19" s="23" t="n">
+        <x:v>0.052010297783469106</x:v>
+      </x:c>
+      <x:c r="M19" s="23" t="n">
+        <x:v>0.021938108432294712</x:v>
+      </x:c>
+      <x:c r="N19" s="23" t="n">
         <x:v>0.07394840621576648</x:v>
       </x:c>
-      <x:c r="I19" s="22" t="n">
-        <x:v>1026426857734656</x:v>
-      </x:c>
-      <x:c r="J19" s="22" t="n">
-        <x:v>61279215.38714364</x:v>
-      </x:c>
-      <x:c r="K19" s="17" t="n">
+      <x:c r="O19" s="24" t="n">
+        <x:v>1026426857734656.1</x:v>
+      </x:c>
+      <x:c r="P19" s="24" t="n">
+        <x:v>61279215.38714365</x:v>
+      </x:c>
+      <x:c r="Q19" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R19" s="17" t="n">
         <x:v>0.7150433534089107</x:v>
       </x:c>
-      <x:c r="L19" s="16" t="str">
+      <x:c r="S19" s="16" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M19" s="16" t="n">
+      <x:c r="T19" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="N19" s="16" t="str">
+      <x:c r="U19" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O19" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V19" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A20" s="16" t="n">
         <x:v>15</x:v>
       </x:c>
@@ -1580,40 +2023,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
+        <x:v>17451.32971</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>17.451329710000003</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
+        <x:v>22700.2</x:v>
+      </x:c>
+      <x:c r="H20" s="22" t="n">
         <x:v>23242366</x:v>
       </x:c>
-      <x:c r="F20" s="22" t="n">
+      <x:c r="I20" s="22" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="G20" s="23" t="n">
-        <x:v>24.47025360226221</x:v>
-      </x:c>
-      <x:c r="H20" s="23" t="n">
+      <x:c r="J20" s="22" t="n">
+        <x:v>1331839.257307803</x:v>
+      </x:c>
+      <x:c r="K20" s="23" t="n">
+        <x:v>265.67955693338394</x:v>
+      </x:c>
+      <x:c r="L20" s="23" t="n">
+        <x:v>0.06917323410675813</x:v>
+      </x:c>
+      <x:c r="M20" s="23" t="n">
+        <x:v>0.0473264401703517</x:v>
+      </x:c>
+      <x:c r="N20" s="23" t="n">
         <x:v>0.11649967427711161</x:v>
       </x:c>
-      <x:c r="I20" s="22" t="n">
+      <x:c r="O20" s="24" t="n">
         <x:v>1112750770860288</x:v>
       </x:c>
-      <x:c r="J20" s="22" t="n">
+      <x:c r="P20" s="24" t="n">
         <x:v>66432881.84240525</x:v>
       </x:c>
-      <x:c r="K20" s="17" t="n">
+      <x:c r="Q20" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R20" s="17" t="n">
         <x:v>0.775179484742185</x:v>
       </x:c>
-      <x:c r="L20" s="16" t="str">
+      <x:c r="S20" s="16" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M20" s="16" t="n">
+      <x:c r="T20" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="N20" s="16" t="str">
+      <x:c r="U20" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O20" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V20" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A21" s="16" t="n">
         <x:v>16</x:v>
       </x:c>
@@ -1627,40 +2091,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E21" s="22" t="n">
+        <x:v>19777.32971</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>19.77732971</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>25804.3</x:v>
+      </x:c>
+      <x:c r="H21" s="22" t="n">
         <x:v>30057691</x:v>
       </x:c>
-      <x:c r="F21" s="22" t="n">
+      <x:c r="I21" s="22" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="G21" s="23" t="n">
-        <x:v>24.841230851416743</x:v>
-      </x:c>
-      <x:c r="H21" s="23" t="n">
+      <x:c r="J21" s="22" t="n">
+        <x:v>1519805.3246188208</x:v>
+      </x:c>
+      <x:c r="K21" s="23" t="n">
+        <x:v>303.17562953200115</x:v>
+      </x:c>
+      <x:c r="L21" s="23" t="n">
+        <x:v>0.18051068258604275</x:v>
+      </x:c>
+      <x:c r="M21" s="23" t="n">
+        <x:v>0.19046656656848882</x:v>
+      </x:c>
+      <x:c r="N21" s="23" t="n">
         <x:v>0.37097724915453156</x:v>
       </x:c>
-      <x:c r="I21" s="22" t="n">
-        <x:v>1439041052469888</x:v>
-      </x:c>
-      <x:c r="J21" s="22" t="n">
-        <x:v>85912898.65491869</x:v>
-      </x:c>
-      <x:c r="K21" s="17" t="n">
+      <x:c r="O21" s="24" t="n">
+        <x:v>1439041052469887.8</x:v>
+      </x:c>
+      <x:c r="P21" s="24" t="n">
+        <x:v>85912898.65491867</x:v>
+      </x:c>
+      <x:c r="Q21" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R21" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L21" s="16" t="str">
+      <x:c r="S21" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M21" s="16" t="n">
+      <x:c r="T21" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N21" s="16" t="str">
+      <x:c r="U21" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O21" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V21" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A22" s="16" t="n">
         <x:v>17</x:v>
       </x:c>
@@ -1674,40 +2159,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E22" s="22" t="n">
+        <x:v>23626.32971</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>23.62632971</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>30729.3</x:v>
+      </x:c>
+      <x:c r="H22" s="22" t="n">
         <x:v>37048243</x:v>
       </x:c>
-      <x:c r="F22" s="22" t="n">
+      <x:c r="I22" s="22" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="G22" s="23" t="n">
-        <x:v>25.142901789055944</x:v>
-      </x:c>
-      <x:c r="H22" s="23" t="n">
+      <x:c r="J22" s="22" t="n">
+        <x:v>1568091.3393974642</x:v>
+      </x:c>
+      <x:c r="K22" s="23" t="n">
+        <x:v>312.80787827529224</x:v>
+      </x:c>
+      <x:c r="L22" s="23" t="n">
+        <x:v>0.25654787787862965</x:v>
+      </x:c>
+      <x:c r="M22" s="23" t="n">
+        <x:v>0.04512305976057718</x:v>
+      </x:c>
+      <x:c r="N22" s="23" t="n">
         <x:v>0.3016709376392015</x:v>
       </x:c>
-      <x:c r="I22" s="22" t="n">
-        <x:v>1773720496324224</x:v>
-      </x:c>
-      <x:c r="J22" s="22" t="n">
-        <x:v>105893760.97458054</x:v>
-      </x:c>
-      <x:c r="K22" s="17" t="n">
+      <x:c r="O22" s="24" t="n">
+        <x:v>1773720496324224.2</x:v>
+      </x:c>
+      <x:c r="P22" s="24" t="n">
+        <x:v>105893760.97458056</x:v>
+      </x:c>
+      <x:c r="Q22" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R22" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L22" s="16" t="str">
+      <x:c r="S22" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M22" s="16" t="n">
+      <x:c r="T22" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N22" s="16" t="str">
+      <x:c r="U22" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O22" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V22" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A23" s="16" t="n">
         <x:v>18</x:v>
       </x:c>
@@ -1721,40 +2227,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E23" s="22" t="n">
+        <x:v>26122.32971</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>26.122329710000002</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>33779.3</x:v>
+      </x:c>
+      <x:c r="H23" s="22" t="n">
         <x:v>46037632</x:v>
       </x:c>
-      <x:c r="F23" s="22" t="n">
+      <x:c r="I23" s="22" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="G23" s="23" t="n">
-        <x:v>25.456310292865954</x:v>
-      </x:c>
-      <x:c r="H23" s="23" t="n">
+      <x:c r="J23" s="22" t="n">
+        <x:v>1762386.1466833923</x:v>
+      </x:c>
+      <x:c r="K23" s="23" t="n">
+        <x:v>351.5664281760725</x:v>
+      </x:c>
+      <x:c r="L23" s="23" t="n">
+        <x:v>0.1448880411016562</x:v>
+      </x:c>
+      <x:c r="M23" s="23" t="n">
+        <x:v>0.16852046270835075</x:v>
+      </x:c>
+      <x:c r="N23" s="23" t="n">
         <x:v>0.3134085038100096</x:v>
       </x:c>
-      <x:c r="I23" s="22" t="n">
+      <x:c r="O23" s="24" t="n">
         <x:v>2204096196427776</x:v>
       </x:c>
-      <x:c r="J23" s="22" t="n">
+      <x:c r="P23" s="24" t="n">
         <x:v>131587832.6225538</x:v>
       </x:c>
-      <x:c r="K23" s="17" t="n">
+      <x:c r="Q23" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R23" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L23" s="16" t="str">
+      <x:c r="S23" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M23" s="16" t="n">
+      <x:c r="T23" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N23" s="16" t="str">
+      <x:c r="U23" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O23" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V23" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A24" s="16" t="n">
         <x:v>19</x:v>
       </x:c>
@@ -1768,40 +2295,61 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E24" s="22" t="n">
+        <x:v>26757.32971</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>26.75732971</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>34541.3</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
         <x:v>47106859</x:v>
       </x:c>
-      <x:c r="F24" s="22" t="n">
+      <x:c r="I24" s="22" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="G24" s="23" t="n">
-        <x:v>25.489433803133178</x:v>
-      </x:c>
-      <x:c r="H24" s="23" t="n">
+      <x:c r="J24" s="22" t="n">
+        <x:v>1760521.6780056637</x:v>
+      </x:c>
+      <x:c r="K24" s="23" t="n">
+        <x:v>351.19449799793944</x:v>
+      </x:c>
+      <x:c r="L24" s="23" t="n">
+        <x:v>0.034650578303203616</x:v>
+      </x:c>
+      <x:c r="M24" s="23" t="n">
+        <x:v>-0.0015270680359833477</x:v>
+      </x:c>
+      <x:c r="N24" s="23" t="n">
         <x:v>0.03312351026722382</x:v>
       </x:c>
-      <x:c r="I24" s="22" t="n">
+      <x:c r="O24" s="24" t="n">
         <x:v>2255286474064512</x:v>
       </x:c>
-      <x:c r="J24" s="22" t="n">
+      <x:c r="P24" s="24" t="n">
         <x:v>134643968.60086638</x:v>
       </x:c>
-      <x:c r="K24" s="17" t="n">
+      <x:c r="Q24" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R24" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L24" s="16" t="str">
+      <x:c r="S24" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M24" s="16" t="n">
+      <x:c r="T24" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N24" s="16" t="str">
+      <x:c r="U24" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O24" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="V24" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A25" s="16" t="n">
         <x:v>20</x:v>
       </x:c>
@@ -1815,48 +2363,69 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E25" s="22" t="n">
+        <x:v>31674.32971</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>31.674329710000002</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>41462.3</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
         <x:v>61887051</x:v>
       </x:c>
-      <x:c r="F25" s="22" t="n">
+      <x:c r="I25" s="22" t="n">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="G25" s="23" t="n">
-        <x:v>25.88313424146424</x:v>
-      </x:c>
-      <x:c r="H25" s="23" t="n">
+      <x:c r="J25" s="22" t="n">
+        <x:v>1953855.111272061</x:v>
+      </x:c>
+      <x:c r="K25" s="23" t="n">
+        <x:v>389.7612699329068</x:v>
+      </x:c>
+      <x:c r="L25" s="23" t="n">
+        <x:v>0.2433799423435694</x:v>
+      </x:c>
+      <x:c r="M25" s="23" t="n">
+        <x:v>0.15032049598749353</x:v>
+      </x:c>
+      <x:c r="N25" s="23" t="n">
         <x:v>0.39370043833106294</x:v>
       </x:c>
-      <x:c r="I25" s="22" t="n">
+      <x:c r="O25" s="24" t="n">
         <x:v>2962902473290368</x:v>
       </x:c>
-      <x:c r="J25" s="22" t="n">
+      <x:c r="P25" s="24" t="n">
         <x:v>176889699.8979324</x:v>
       </x:c>
-      <x:c r="K25" s="17" t="n">
+      <x:c r="Q25" s="24" t="n">
+        <x:v>85700000</x:v>
+      </x:c>
+      <x:c r="R25" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L25" s="16" t="str">
+      <x:c r="S25" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M25" s="16" t="n">
+      <x:c r="T25" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N25" s="16" t="str">
+      <x:c r="U25" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="O25" s="16" t="str">
-        <x:v>Latest expected or projected state on or before cutoff for each Epoch-covered U.S. site</x:v>
+      <x:c r="V25" s="16" t="str">
+        <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O2"/>
-    <x:mergeCell ref="A3:O3"/>
+    <x:mergeCell ref="A1:V2"/>
+    <x:mergeCell ref="A3:V3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7f79f9a0564981"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201462959a504813"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R586f6a2e2d474f76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b79f065abae43f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1929,7 +2498,7 @@
       <x:c r="B7" s="16" t="str">
         <x:v>Selected target</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="n">
+      <x:c r="C7" s="25" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
@@ -1943,7 +2512,7 @@
       <x:c r="B8" s="16" t="str">
         <x:v>Supply gate share of selected target</x:v>
       </x:c>
-      <x:c r="C8" s="24" t="n">
+      <x:c r="C8" s="25" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
@@ -1985,7 +2554,7 @@
       <x:c r="B11" s="16" t="str">
         <x:v>Fleet share allocated to inference</x:v>
       </x:c>
-      <x:c r="C11" s="24" t="n">
+      <x:c r="C11" s="25" t="n">
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
@@ -1999,7 +2568,7 @@
       <x:c r="B12" s="16" t="str">
         <x:v>Sustained utilization</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="n">
+      <x:c r="C12" s="25" t="n">
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
@@ -2069,7 +2638,7 @@
       <x:c r="B17" s="16" t="str">
         <x:v>Personal-AI inference share</x:v>
       </x:c>
-      <x:c r="C17" s="24" t="n">
+      <x:c r="C17" s="25" t="n">
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
@@ -2139,12 +2708,2175 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05c1e9098a554d31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202f59c91a1c4920"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Epoch AI Data-Center Registry</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+      <x:c r="H1" s="3"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="3"/>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+      <x:c r="H2" s="3"/>
+    </x:row>
+    <x:row r="3" ht="24" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>Facility-level source rows used to identify U.S. sites and audit the timeline join. Facility power includes non-IT overhead and is not substituted for IT power in the gate.</x:v>
+      </x:c>
+      <x:c r="B3" s="6"/>
+      <x:c r="C3" s="6"/>
+      <x:c r="D3" s="6"/>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="6"/>
+      <x:c r="G3" s="6"/>
+      <x:c r="H3" s="6"/>
+    </x:row>
+    <x:row r="4"/>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Country</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Current H100e</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Current facility power MW</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Users</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>Colossus 2</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="n">
+        <x:v>1111672.5618999496</x:v>
+      </x:c>
+      <x:c r="D6" s="22" t="n">
+        <x:v>946</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>Anthropic #confident, Cursor #confident, SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>5420 Tulane Rd, Memphis, TN 38109</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>Microsoft Fairwater Atlanta</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="n">
+        <x:v>768768.7220818596</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="n">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>OpenAI #likely, Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>1435 Hwy 54 W, Fayetteville, GA 30214</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>Google Pryor (North)</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="n">
+        <x:v>763011.622031329</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="n">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>4581 Webb St, Pryor, OK 74361</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" hidden="0" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>Anthropic-Amazon New Carlisle</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="n">
+        <x:v>685912.076806468</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="n">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>Amazon #confident</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>Anthropic #confident</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>55001 Larrison Blvd, New Carlisle, IN 46552</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" hidden="0" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>Meta Prometheus</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="n">
+        <x:v>677109.6513390602</x:v>
+      </x:c>
+      <x:c r="D10" s="22" t="n">
+        <x:v>562</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>1 Community Cir, New Albany, OH 43054</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>Google New Albany</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="n">
+        <x:v>616472.9661445174</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>1101 Beech Rd SW, New Albany, OH 43054</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>OpenAI Stargate Abilene</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="n">
+        <x:v>509348.15563415864</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="n">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F12" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str">
+        <x:v>5502 Spinks Rd, Abilene, TX 79601</x:v>
+      </x:c>
+      <x:c r="H12" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>Microsoft Fairwater Wisconsin</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="n">
+        <x:v>445679.63617988885</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="n">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F13" s="16" t="str">
+        <x:v>OpenAI #likely, Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>4800 90th St, Mount Pleasant, WI 53403</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A14" s="16" t="str">
+        <x:v>Google Columbus</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="n">
+        <x:v>408792.3193532087</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="n">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="E14" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F14" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str">
+        <x:v>5076 S High St, Columbus, OH 43207</x:v>
+      </x:c>
+      <x:c r="H14" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A15" s="16" t="str">
+        <x:v>Google Mesa</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="n">
+        <x:v>343102.57705912075</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="n">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="str"/>
+      <x:c r="G15" s="16" t="str"/>
+      <x:c r="H15" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" hidden="0" customHeight="1">
+      <x:c r="A16" s="16" t="str">
+        <x:v>Google Council Bluffs (East)</x:v>
+      </x:c>
+      <x:c r="B16" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="n">
+        <x:v>289034.86609398684</x:v>
+      </x:c>
+      <x:c r="D16" s="22" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E16" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F16" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G16" s="16" t="str">
+        <x:v>10410 Bunge Ave, Council Bluffs, IA 51503</x:v>
+      </x:c>
+      <x:c r="H16" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A17" s="16" t="str">
+        <x:v>Google Lincoln</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="n">
+        <x:v>287518.9489641233</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="n">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="E17" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="str"/>
+      <x:c r="G17" s="16" t="str">
+        <x:v>5475 Cloud Ct, Lincoln, NE 68514</x:v>
+      </x:c>
+      <x:c r="H17" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" hidden="0" customHeight="1">
+      <x:c r="A18" s="16" t="str">
+        <x:v>Google Bristow</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="n">
+        <x:v>283675.08842849924</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="n">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="E18" s="16" t="str">
+        <x:v>Google</x:v>
+      </x:c>
+      <x:c r="F18" s="16" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="str">
+        <x:v>13001 Rollins Ford Road, Bristow, VA 20136</x:v>
+      </x:c>
+      <x:c r="H18" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A19" s="16" t="str">
+        <x:v>DayOne Nusajaya</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="str">
+        <x:v>Malaysia</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="n">
+        <x:v>281670.4396159676</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="n">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="E19" s="16" t="str"/>
+      <x:c r="F19" s="16" t="str"/>
+      <x:c r="G19" s="16" t="str"/>
+      <x:c r="H19" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="54" hidden="0" customHeight="1">
+      <x:c r="A20" s="16" t="str">
+        <x:v>Colossus 1</x:v>
+      </x:c>
+      <x:c r="B20" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="n">
+        <x:v>275795.85649317835</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="n">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="E20" s="16" t="str">
+        <x:v>SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="F20" s="16" t="str">
+        <x:v>Anthropic #confident</x:v>
+      </x:c>
+      <x:c r="G20" s="16" t="str">
+        <x:v>3231 Riverport Rd, Memphis, TN 38109</x:v>
+      </x:c>
+      <x:c r="H20" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A21" s="16" t="str">
+        <x:v>Google Omaha</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="n">
+        <x:v>267812.02627589693</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E21" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F21" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G21" s="16" t="str">
+        <x:v>11110 State St, Omaha, NE 68142</x:v>
+      </x:c>
+      <x:c r="H21" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A22" s="16" t="str">
+        <x:v>CoreWeave Denton TX</x:v>
+      </x:c>
+      <x:c r="B22" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="n">
+        <x:v>252652.85497726125</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="E22" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F22" s="16" t="str">
+        <x:v>OpenAI #likely</x:v>
+      </x:c>
+      <x:c r="G22" s="16" t="str">
+        <x:v>8171 Jim Christal Rd, Denton, TX 76207</x:v>
+      </x:c>
+      <x:c r="H22" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A23" s="16" t="str">
+        <x:v>Google Kansas City East</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="n">
+        <x:v>244567.9636179889</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F23" s="16" t="str"/>
+      <x:c r="G23" s="16" t="str"/>
+      <x:c r="H23" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="54" hidden="0" customHeight="1">
+      <x:c r="A24" s="16" t="str">
+        <x:v>QTS Richmond 1</x:v>
+      </x:c>
+      <x:c r="B24" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="n">
+        <x:v>242546.7407781708</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E24" s="16" t="str"/>
+      <x:c r="F24" s="16" t="str"/>
+      <x:c r="G24" s="16" t="str">
+        <x:v>6000 Technology Blvd, Sandston, VA 23150</x:v>
+      </x:c>
+      <x:c r="H24" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="54" hidden="0" customHeight="1">
+      <x:c r="A25" s="16" t="str">
+        <x:v>Meta Rosemount</x:v>
+      </x:c>
+      <x:c r="B25" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C25" s="22" t="n">
+        <x:v>215765.5381505811</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="E25" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F25" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G25" s="16" t="str">
+        <x:v>1772-2396 145th St, Rosemount, MN 55068, USA</x:v>
+      </x:c>
+      <x:c r="H25" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A26" s="16" t="str">
+        <x:v>Amazon Madison Mega Site</x:v>
+      </x:c>
+      <x:c r="B26" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C26" s="22" t="n">
+        <x:v>214348.14354550533</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="E26" s="16" t="str">
+        <x:v>Amazon #confident</x:v>
+      </x:c>
+      <x:c r="F26" s="16" t="str">
+        <x:v>Anthropic #speculative</x:v>
+      </x:c>
+      <x:c r="G26" s="16" t="str">
+        <x:v>Amazon Data Services Inc, Madison Mega Site Nissan Parkway and Highway 22 Canton, Mississippi Madison County</x:v>
+      </x:c>
+      <x:c r="H26" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="54" hidden="0" customHeight="1">
+      <x:c r="A27" s="16" t="str">
+        <x:v>Microsoft Goodyear</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C27" s="22" t="n">
+        <x:v>205154.11824153614</x:v>
+      </x:c>
+      <x:c r="D27" s="22" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F27" s="16" t="str">
+        <x:v>OpenAI #likely, Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="str">
+        <x:v>14250 W Broadway Rd, Goodyear, AZ 85338</x:v>
+      </x:c>
+      <x:c r="H27" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A28" s="16" t="str">
+        <x:v>Meta Jeffersonville</x:v>
+      </x:c>
+      <x:c r="B28" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C28" s="22" t="n">
+        <x:v>203132.89540171804</x:v>
+      </x:c>
+      <x:c r="D28" s="22" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="E28" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F28" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G28" s="16" t="str">
+        <x:v>500 8th St, Jeffersonville, IN 47130, USA</x:v>
+      </x:c>
+      <x:c r="H28" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A29" s="16" t="str">
+        <x:v>Google The Dalles</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C29" s="22" t="n">
+        <x:v>201616.97827185446</x:v>
+      </x:c>
+      <x:c r="D29" s="22" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E29" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F29" s="16" t="str"/>
+      <x:c r="G29" s="16" t="str">
+        <x:v>3500 River Rd, The Dalles, OR</x:v>
+      </x:c>
+      <x:c r="H29" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="54" hidden="0" customHeight="1">
+      <x:c r="A30" s="16" t="str">
+        <x:v>Google Midlothian</x:v>
+      </x:c>
+      <x:c r="B30" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C30" s="22" t="n">
+        <x:v>191005.5583628095</x:v>
+      </x:c>
+      <x:c r="D30" s="22" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="E30" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F30" s="16" t="str"/>
+      <x:c r="G30" s="16" t="str">
+        <x:v>3250 Railport Parkway, Midlothian, TX 76065</x:v>
+      </x:c>
+      <x:c r="H30" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="54" hidden="0" customHeight="1">
+      <x:c r="A31" s="16" t="str">
+        <x:v>QTS Richmond 2</x:v>
+      </x:c>
+      <x:c r="B31" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C31" s="22" t="n">
+        <x:v>182920.66700353715</x:v>
+      </x:c>
+      <x:c r="D31" s="22" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E31" s="16" t="str"/>
+      <x:c r="F31" s="16" t="str"/>
+      <x:c r="G31" s="16" t="str">
+        <x:v>6030–6070 Technology Blvd, Sandston, VA 23150</x:v>
+      </x:c>
+      <x:c r="H31" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A32" s="16" t="str">
+        <x:v>QTS Richmond 3</x:v>
+      </x:c>
+      <x:c r="B32" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C32" s="22" t="n">
+        <x:v>174835.77564426477</x:v>
+      </x:c>
+      <x:c r="D32" s="22" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="E32" s="16" t="str"/>
+      <x:c r="F32" s="16" t="str"/>
+      <x:c r="G32" s="16" t="str">
+        <x:v>3525–3543 Portugee Rd, Sandston, VA 23150</x:v>
+      </x:c>
+      <x:c r="H32" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A33" s="16" t="str">
+        <x:v>Meta Montgomery</x:v>
+      </x:c>
+      <x:c r="B33" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C33" s="22" t="n">
+        <x:v>174517.43304699342</x:v>
+      </x:c>
+      <x:c r="D33" s="22" t="n">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="E33" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F33" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G33" s="16" t="str">
+        <x:v>Co Rd 42, Montgomery, AL 36105, USA</x:v>
+      </x:c>
+      <x:c r="H33" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A34" s="16" t="str">
+        <x:v>Meta Kuna</x:v>
+      </x:c>
+      <x:c r="B34" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C34" s="22" t="n">
+        <x:v>173319.85851440122</x:v>
+      </x:c>
+      <x:c r="D34" s="22" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="E34" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F34" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G34" s="16" t="str">
+        <x:v>601 Kuna Mora Rd,  Kuna ID 83634</x:v>
+      </x:c>
+      <x:c r="H34" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A35" s="16" t="str">
+        <x:v>Meta Temple</x:v>
+      </x:c>
+      <x:c r="B35" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C35" s="22" t="n">
+        <x:v>173247.6719844078</x:v>
+      </x:c>
+      <x:c r="D35" s="22" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="E35" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F35" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G35" s="16" t="str">
+        <x:v>2310 Eberhardt Rd, Temple, TX 76504</x:v>
+      </x:c>
+      <x:c r="H35" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A36" s="16" t="str">
+        <x:v>Meta Cheyenne</x:v>
+      </x:c>
+      <x:c r="B36" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C36" s="22" t="n">
+        <x:v>172814.5528044467</x:v>
+      </x:c>
+      <x:c r="D36" s="22" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="E36" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F36" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G36" s="16" t="str">
+        <x:v>Cheyenne, WY 82007, USA</x:v>
+      </x:c>
+      <x:c r="H36" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A37" s="16" t="str">
+        <x:v>Amazon Ridgeland</x:v>
+      </x:c>
+      <x:c r="B37" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C37" s="22" t="n">
+        <x:v>171298.6356745831</x:v>
+      </x:c>
+      <x:c r="D37" s="22" t="n">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="E37" s="16" t="str">
+        <x:v>Amazon #confident</x:v>
+      </x:c>
+      <x:c r="F37" s="16" t="str">
+        <x:v>Anthropic #speculative</x:v>
+      </x:c>
+      <x:c r="G37" s="16" t="str">
+        <x:v>1626 County Line Road Ridgeland, Mississippi</x:v>
+      </x:c>
+      <x:c r="H37" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A38" s="16" t="str">
+        <x:v>Meta Huntsville</x:v>
+      </x:c>
+      <x:c r="B38" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C38" s="22" t="n">
+        <x:v>166760.9903991915</x:v>
+      </x:c>
+      <x:c r="D38" s="22" t="n">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="E38" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F38" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G38" s="16" t="str">
+        <x:v>5400 Prosperity Dr NW, Toney, AL</x:v>
+      </x:c>
+      <x:c r="H38" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A39" s="16" t="str">
+        <x:v>Meta Aiken</x:v>
+      </x:c>
+      <x:c r="B39" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C39" s="22" t="n">
+        <x:v>161697.82718544718</x:v>
+      </x:c>
+      <x:c r="D39" s="22" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="E39" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F39" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G39" s="16" t="str">
+        <x:v>7601 State Hwy 105, Trenton, SC 29847, USA</x:v>
+      </x:c>
+      <x:c r="H39" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A40" s="16" t="str">
+        <x:v>Coreweave Helios</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C40" s="22" t="n">
+        <x:v>159551.768236855</x:v>
+      </x:c>
+      <x:c r="D40" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="E40" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F40" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G40" s="16" t="str">
+        <x:v>984 County Road 112, Afton, TX 79220</x:v>
+      </x:c>
+      <x:c r="H40" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A41" s="16" t="str">
+        <x:v>Google Arcola</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C41" s="22" t="n">
+        <x:v>157150.07579585648</x:v>
+      </x:c>
+      <x:c r="D41" s="22" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E41" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F41" s="16" t="str"/>
+      <x:c r="G41" s="16" t="str">
+        <x:v>42575 Arcola Blvd, Sterling, VA 20166</x:v>
+      </x:c>
+      <x:c r="H41" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A42" s="16" t="str">
+        <x:v>Microsoft Project Osmium</x:v>
+      </x:c>
+      <x:c r="B42" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C42" s="22" t="n">
+        <x:v>155634.15866599293</x:v>
+      </x:c>
+      <x:c r="D42" s="22" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="E42" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F42" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G42" s="16" t="str">
+        <x:v>5855 SW Kerry St, Cumming, IA 50061</x:v>
+      </x:c>
+      <x:c r="H42" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A43" s="16" t="str">
+        <x:v>Google Storey County</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C43" s="22" t="n">
+        <x:v>153612.93582617483</x:v>
+      </x:c>
+      <x:c r="D43" s="22" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="E43" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F43" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G43" s="16" t="str"/>
+      <x:c r="H43" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="54" hidden="0" customHeight="1">
+      <x:c r="A44" s="16" t="str">
+        <x:v>Meta Eagle Mountain</x:v>
+      </x:c>
+      <x:c r="B44" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C44" s="22" t="n">
+        <x:v>151354.21930267813</x:v>
+      </x:c>
+      <x:c r="D44" s="22" t="n">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="E44" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F44" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G44" s="16" t="str">
+        <x:v>1275 N Community Cir, Eagle Mountain, UT 84005</x:v>
+      </x:c>
+      <x:c r="H44" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A45" s="16" t="str">
+        <x:v>Google Lancaster</x:v>
+      </x:c>
+      <x:c r="B45" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C45" s="22" t="n">
+        <x:v>130368.8731682668</x:v>
+      </x:c>
+      <x:c r="D45" s="22" t="n">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="E45" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F45" s="16" t="str"/>
+      <x:c r="G45" s="16" t="str">
+        <x:v>105 Whiley Rd, Lancaster, OH 43130</x:v>
+      </x:c>
+      <x:c r="H45" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A46" s="16" t="str">
+        <x:v>Meta-QTS Hillsboro 2</x:v>
+      </x:c>
+      <x:c r="B46" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C46" s="22" t="n">
+        <x:v>123839</x:v>
+      </x:c>
+      <x:c r="D46" s="22" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E46" s="16" t="str">
+        <x:v>Meta #likely</x:v>
+      </x:c>
+      <x:c r="F46" s="16" t="str">
+        <x:v>Meta #likely</x:v>
+      </x:c>
+      <x:c r="G46" s="16" t="str">
+        <x:v>4755 NE Huffman St, Hillsboro, OR 97124</x:v>
+      </x:c>
+      <x:c r="H46" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A47" s="16" t="str">
+        <x:v>Google Waltham Cross</x:v>
+      </x:c>
+      <x:c r="B47" s="16" t="str">
+        <x:v>United Kingdom</x:v>
+      </x:c>
+      <x:c r="C47" s="22" t="n">
+        <x:v>123799.89893885801</x:v>
+      </x:c>
+      <x:c r="D47" s="22" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E47" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F47" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="str">
+        <x:v>Land at Maxwell's Farm West, Great Cambridge Road, Cheshunt, EN8 8XH</x:v>
+      </x:c>
+      <x:c r="H47" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A48" s="16" t="str">
+        <x:v>VNET Bayin Ulanqab</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="C48" s="22" t="n">
+        <x:v>122789.28751894896</x:v>
+      </x:c>
+      <x:c r="D48" s="22" t="n">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="E48" s="16" t="str">
+        <x:v>VNET #confident</x:v>
+      </x:c>
+      <x:c r="F48" s="16" t="str">
+        <x:v>ByteDance #speculative</x:v>
+      </x:c>
+      <x:c r="G48" s="16" t="str">
+        <x:v>Bayin, Ulanqab, China</x:v>
+      </x:c>
+      <x:c r="H48" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A49" s="16" t="str">
+        <x:v>Huawei Horinger</x:v>
+      </x:c>
+      <x:c r="B49" s="16" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="C49" s="22" t="n">
+        <x:v>117230.92470944922</x:v>
+      </x:c>
+      <x:c r="D49" s="22" t="n">
+        <x:v>241.8</x:v>
+      </x:c>
+      <x:c r="E49" s="16" t="str">
+        <x:v>Huawei #confident</x:v>
+      </x:c>
+      <x:c r="F49" s="16" t="str"/>
+      <x:c r="G49" s="16" t="str">
+        <x:v>Huawei, Horinger, China</x:v>
+      </x:c>
+      <x:c r="H49" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A50" s="16" t="str">
+        <x:v>Google Red Oak</x:v>
+      </x:c>
+      <x:c r="B50" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C50" s="22" t="n">
+        <x:v>108135.42193026781</x:v>
+      </x:c>
+      <x:c r="D50" s="22" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E50" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F50" s="16" t="str"/>
+      <x:c r="G50" s="16" t="str">
+        <x:v>330 Austin Blvd, Red Oak, TX 75154</x:v>
+      </x:c>
+      <x:c r="H50" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A51" s="16" t="str">
+        <x:v>Meta Gallatin</x:v>
+      </x:c>
+      <x:c r="B51" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C51" s="22" t="n">
+        <x:v>99545.22486104093</x:v>
+      </x:c>
+      <x:c r="D51" s="22" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E51" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F51" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G51" s="16" t="str">
+        <x:v>1 Meta Lp, Gallatin, TN 37066</x:v>
+      </x:c>
+      <x:c r="H51" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="54" hidden="0" customHeight="1">
+      <x:c r="A52" s="16" t="str">
+        <x:v>Meta Los Lunas</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C52" s="22" t="n">
+        <x:v>99545.22486104093</x:v>
+      </x:c>
+      <x:c r="D52" s="22" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E52" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F52" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G52" s="16" t="str">
+        <x:v>4250 Messenger Lp, Los Lunas, NM 87031</x:v>
+      </x:c>
+      <x:c r="H52" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A53" s="16" t="str">
+        <x:v>CoreWeave Ellendale ND</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C53" s="22" t="n">
+        <x:v>93481.55634158666</x:v>
+      </x:c>
+      <x:c r="D53" s="22" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E53" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F53" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G53" s="16" t="str">
+        <x:v>9685 87th Ave SE, Ellendale, ND 58436</x:v>
+      </x:c>
+      <x:c r="H53" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A54" s="16" t="str">
+        <x:v>Meta Sarpy</x:v>
+      </x:c>
+      <x:c r="B54" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C54" s="22" t="n">
+        <x:v>91965.63921172309</x:v>
+      </x:c>
+      <x:c r="D54" s="22" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="E54" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F54" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G54" s="16" t="str">
+        <x:v>14436-14998 Fairview Rd, Springfield, NE 68059, USA</x:v>
+      </x:c>
+      <x:c r="H54" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="54" hidden="0" customHeight="1">
+      <x:c r="A55" s="16" t="str">
+        <x:v>CoreWeave Chester VA</x:v>
+      </x:c>
+      <x:c r="B55" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C55" s="22" t="n">
+        <x:v>88428.49924204143</x:v>
+      </x:c>
+      <x:c r="D55" s="22" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E55" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F55" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G55" s="16" t="str">
+        <x:v>1401 Meadowville Technology Parkway, Chester, VA</x:v>
+      </x:c>
+      <x:c r="H55" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A56" s="16" t="str">
+        <x:v>Oracle Batam</x:v>
+      </x:c>
+      <x:c r="B56" s="16" t="str">
+        <x:v>Indonesia</x:v>
+      </x:c>
+      <x:c r="C56" s="22" t="n">
+        <x:v>84386.05356240526</x:v>
+      </x:c>
+      <x:c r="D56" s="22" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E56" s="16" t="str">
+        <x:v>Oracle #likely</x:v>
+      </x:c>
+      <x:c r="F56" s="16" t="str"/>
+      <x:c r="G56" s="16" t="str"/>
+      <x:c r="H56" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="54" hidden="0" customHeight="1">
+      <x:c r="A57" s="16" t="str">
+        <x:v>AWS Berwick</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C57" s="22" t="n">
+        <x:v>81354.21930267812</x:v>
+      </x:c>
+      <x:c r="D57" s="22" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E57" s="16" t="str">
+        <x:v>Amazon #confident</x:v>
+      </x:c>
+      <x:c r="F57" s="16" t="str">
+        <x:v>Anthropic #speculative</x:v>
+      </x:c>
+      <x:c r="G57" s="16" t="str">
+        <x:v>1125 Electron Ave, Berwick, PA 18603</x:v>
+      </x:c>
+      <x:c r="H57" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A58" s="16" t="str">
+        <x:v>Google Papillion</x:v>
+      </x:c>
+      <x:c r="B58" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C58" s="22" t="n">
+        <x:v>80343.60788276908</x:v>
+      </x:c>
+      <x:c r="D58" s="22" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E58" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F58" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G58" s="16" t="str">
+        <x:v>14651-15249 Gold Coast Rd 68138 Papillion Nebraska, USA</x:v>
+      </x:c>
+      <x:c r="H58" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A59" s="16" t="str">
+        <x:v>CoreWeave Marble NC</x:v>
+      </x:c>
+      <x:c r="B59" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C59" s="22" t="n">
+        <x:v>78827.6907529055</x:v>
+      </x:c>
+      <x:c r="D59" s="22" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E59" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F59" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G59" s="16" t="str">
+        <x:v>155 Palmer Ln, Marble, NC 28905</x:v>
+      </x:c>
+      <x:c r="H59" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="54" hidden="0" customHeight="1">
+      <x:c r="A60" s="16" t="str">
+        <x:v>Microsoft SAT40</x:v>
+      </x:c>
+      <x:c r="B60" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C60" s="22" t="n">
+        <x:v>64679.13087417888</x:v>
+      </x:c>
+      <x:c r="D60" s="22" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="E60" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F60" s="16" t="str"/>
+      <x:c r="G60" s="16" t="str">
+        <x:v>15000 Lambda Drive, San Antonio, TX 78245</x:v>
+      </x:c>
+      <x:c r="H60" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="54" hidden="0" customHeight="1">
+      <x:c r="A61" s="16" t="str">
+        <x:v>STACK Infrastructure NVA02</x:v>
+      </x:c>
+      <x:c r="B61" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C61" s="22" t="n">
+        <x:v>61141.99090449722</x:v>
+      </x:c>
+      <x:c r="D61" s="22" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="E61" s="16" t="str"/>
+      <x:c r="F61" s="16" t="str"/>
+      <x:c r="G61" s="16" t="str">
+        <x:v>9590 Hornbaker Rd, Manassas, VA 20109</x:v>
+      </x:c>
+      <x:c r="H61" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A62" s="16" t="str">
+        <x:v>Anthropic Lake Mariner</x:v>
+      </x:c>
+      <x:c r="B62" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C62" s="22" t="n">
+        <x:v>58564.93178372915</x:v>
+      </x:c>
+      <x:c r="D62" s="22" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E62" s="16" t="str">
+        <x:v>AI XPV Platform #confident</x:v>
+      </x:c>
+      <x:c r="F62" s="16" t="str">
+        <x:v>Anthropic #likely</x:v>
+      </x:c>
+      <x:c r="G62" s="16" t="str">
+        <x:v>7725 Lake Rd, Barker, NY 14012</x:v>
+      </x:c>
+      <x:c r="H62" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A63" s="16" t="str">
+        <x:v>Microsoft-Nebius New Jersey</x:v>
+      </x:c>
+      <x:c r="B63" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C63" s="22" t="n">
+        <x:v>56846.89236988378</x:v>
+      </x:c>
+      <x:c r="D63" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E63" s="16" t="str">
+        <x:v>Nebius #confident</x:v>
+      </x:c>
+      <x:c r="F63" s="16" t="str">
+        <x:v>Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G63" s="16" t="str">
+        <x:v>3963 S Lincoln Ave, Vineland, New Jersey</x:v>
+      </x:c>
+      <x:c r="H63" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A64" s="16" t="str">
+        <x:v>CoreWeave Norway</x:v>
+      </x:c>
+      <x:c r="B64" s="16" t="str">
+        <x:v>Norway</x:v>
+      </x:c>
+      <x:c r="C64" s="22" t="n">
+        <x:v>50773.11773623042</x:v>
+      </x:c>
+      <x:c r="D64" s="22" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E64" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F64" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G64" s="16" t="str">
+        <x:v>Stølevegen 39, 4715 Øvrebø, Norway</x:v>
+      </x:c>
+      <x:c r="H64" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A65" s="16" t="str">
+        <x:v>Southgate Melbourne</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="str">
+        <x:v>Australia</x:v>
+      </x:c>
+      <x:c r="C65" s="22" t="n">
+        <x:v>46488.12531581607</x:v>
+      </x:c>
+      <x:c r="D65" s="22" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E65" s="16" t="str">
+        <x:v>Firmus #confident</x:v>
+      </x:c>
+      <x:c r="F65" s="16" t="str"/>
+      <x:c r="G65" s="16" t="str"/>
+      <x:c r="H65" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A66" s="16" t="str">
+        <x:v>Stream Phoenix</x:v>
+      </x:c>
+      <x:c r="B66" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C66" s="22" t="n">
+        <x:v>46134.4113188479</x:v>
+      </x:c>
+      <x:c r="D66" s="22" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E66" s="16" t="str"/>
+      <x:c r="F66" s="16" t="str"/>
+      <x:c r="G66" s="16" t="str">
+        <x:v>2950 S. Litchfield Road</x:v>
+      </x:c>
+      <x:c r="H66" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="54" hidden="0" customHeight="1">
+      <x:c r="A67" s="16" t="str">
+        <x:v>Microsoft SAT14</x:v>
+      </x:c>
+      <x:c r="B67" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C67" s="22" t="n">
+        <x:v>45174.33046993431</x:v>
+      </x:c>
+      <x:c r="D67" s="22" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="E67" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F67" s="16" t="str"/>
+      <x:c r="G67" s="16" t="str">
+        <x:v>3545 Wiseman Boulevard, San Antonio, TX 78251</x:v>
+      </x:c>
+      <x:c r="H67" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A68" s="16" t="str">
+        <x:v>Vantage TX1</x:v>
+      </x:c>
+      <x:c r="B68" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C68" s="22" t="n">
+        <x:v>38706.417382516425</x:v>
+      </x:c>
+      <x:c r="D68" s="22" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E68" s="16" t="str"/>
+      <x:c r="F68" s="16" t="str"/>
+      <x:c r="G68" s="16" t="str">
+        <x:v>14720 Omicron Dr, San Antonio, TX 78245</x:v>
+      </x:c>
+      <x:c r="H68" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="54" hidden="0" customHeight="1">
+      <x:c r="A69" s="16" t="str">
+        <x:v>CoreWeave Dalton 1 &amp; 2</x:v>
+      </x:c>
+      <x:c r="B69" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C69" s="22" t="n">
+        <x:v>32238.504295098533</x:v>
+      </x:c>
+      <x:c r="D69" s="22" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E69" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F69" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G69" s="16" t="str">
+        <x:v>2205 Industrial South Rd, Dalton, GA, 30721</x:v>
+      </x:c>
+      <x:c r="H69" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A70" s="16" t="str">
+        <x:v>Alibaba Zhangbei</x:v>
+      </x:c>
+      <x:c r="B70" s="16" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="C70" s="22" t="n">
+        <x:v>31884.79029813037</x:v>
+      </x:c>
+      <x:c r="D70" s="22" t="n">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="E70" s="16" t="str">
+        <x:v>Alibaba #confident</x:v>
+      </x:c>
+      <x:c r="F70" s="16" t="str">
+        <x:v>Alibaba #likely</x:v>
+      </x:c>
+      <x:c r="G70" s="16" t="str">
+        <x:v>Alibaba Zhangbei Yun Calculation Data Center, Zhangbei County, Zhangjiakou, Hebei, China, 076471</x:v>
+      </x:c>
+      <x:c r="H70" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A71" s="16" t="str">
+        <x:v>Start Campus Sines Data Campus</x:v>
+      </x:c>
+      <x:c r="B71" s="16" t="str">
+        <x:v>Portugal</x:v>
+      </x:c>
+      <x:c r="C71" s="22" t="n">
+        <x:v>31834.259727134915</x:v>
+      </x:c>
+      <x:c r="D71" s="22" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E71" s="16" t="str">
+        <x:v>Nscale #confident</x:v>
+      </x:c>
+      <x:c r="F71" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="G71" s="16" t="str">
+        <x:v>Start Campus - Sustainable Data Center Services, Sines, Portugal</x:v>
+      </x:c>
+      <x:c r="H71" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="54" hidden="0" customHeight="1">
+      <x:c r="A72" s="16" t="str">
+        <x:v>xAI QTS Atlanta</x:v>
+      </x:c>
+      <x:c r="B72" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C72" s="22" t="n">
+        <x:v>11470.43961596766</x:v>
+      </x:c>
+      <x:c r="D72" s="22" t="n">
+        <x:v>17.32971</x:v>
+      </x:c>
+      <x:c r="E72" s="16" t="str">
+        <x:v>SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="F72" s="16" t="str">
+        <x:v>SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="G72" s="16" t="str">
+        <x:v>1025 Jefferson Street NW, Atlanta, GA 30318</x:v>
+      </x:c>
+      <x:c r="H72" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="54" hidden="0" customHeight="1">
+      <x:c r="A73" s="16" t="str">
+        <x:v>CoreWeave Muskogee OK</x:v>
+      </x:c>
+      <x:c r="B73" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C73" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D73" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E73" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F73" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G73" s="16" t="str">
+        <x:v>1525 W 43rd St S, Muskogee, OK 74401, USA</x:v>
+      </x:c>
+      <x:c r="H73" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A74" s="16" t="str">
+        <x:v>Crusoe Abilene Expansion</x:v>
+      </x:c>
+      <x:c r="B74" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C74" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D74" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E74" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F74" s="16" t="str">
+        <x:v>Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G74" s="16" t="str">
+        <x:v>5502 Spinks Rd, Abilene, TX 79601</x:v>
+      </x:c>
+      <x:c r="H74" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A75" s="16" t="str">
+        <x:v>Goodnight</x:v>
+      </x:c>
+      <x:c r="B75" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C75" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D75" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E75" s="16" t="str">
+        <x:v>Google #speculative</x:v>
+      </x:c>
+      <x:c r="F75" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G75" s="16" t="str">
+        <x:v>10001 Lima Rd, Claude, TX 79019</x:v>
+      </x:c>
+      <x:c r="H75" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A76" s="16" t="str">
+        <x:v>Google Cedar Rapids</x:v>
+      </x:c>
+      <x:c r="B76" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C76" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D76" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E76" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F76" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G76" s="16" t="str">
+        <x:v>5800 EDGEWOOD RD SW CEDAR RAPIDS, IA 52404</x:v>
+      </x:c>
+      <x:c r="H76" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A77" s="16" t="str">
+        <x:v>Google Fort Wayne</x:v>
+      </x:c>
+      <x:c r="B77" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C77" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D77" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E77" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F77" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G77" s="16" t="str">
+        <x:v>6015 Adams Center Road, Fort Wayne, IN 46806</x:v>
+      </x:c>
+      <x:c r="H77" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A78" s="16" t="str">
+        <x:v>Meta Hyperion</x:v>
+      </x:c>
+      <x:c r="B78" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C78" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D78" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E78" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F78" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G78" s="16" t="str">
+        <x:v>Holly Ridge, LA 71269</x:v>
+      </x:c>
+      <x:c r="H78" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A79" s="16" t="str">
+        <x:v>Microsoft Narvik Norway</x:v>
+      </x:c>
+      <x:c r="B79" s="16" t="str">
+        <x:v>Norway</x:v>
+      </x:c>
+      <x:c r="C79" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D79" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E79" s="16" t="str">
+        <x:v>Nscale #likely</x:v>
+      </x:c>
+      <x:c r="F79" s="16" t="str">
+        <x:v>Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G79" s="16" t="str"/>
+      <x:c r="H79" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A80" s="16" t="str">
+        <x:v>OpenAI Stargate Lordstown</x:v>
+      </x:c>
+      <x:c r="B80" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C80" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D80" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E80" s="16" t="str">
+        <x:v>Softbank #confident</x:v>
+      </x:c>
+      <x:c r="F80" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G80" s="16" t="str">
+        <x:v>2300 Hallock Young Rd, Warren, OH 44481</x:v>
+      </x:c>
+      <x:c r="H80" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A81" s="16" t="str">
+        <x:v>OpenAI Stargate Michigan</x:v>
+      </x:c>
+      <x:c r="B81" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C81" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D81" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E81" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F81" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G81" s="16" t="str"/>
+      <x:c r="H81" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A82" s="16" t="str">
+        <x:v>OpenAI Stargate Milam</x:v>
+      </x:c>
+      <x:c r="B82" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C82" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D82" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E82" s="16" t="str">
+        <x:v>Softbank #confident</x:v>
+      </x:c>
+      <x:c r="F82" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G82" s="16" t="str"/>
+      <x:c r="H82" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A83" s="16" t="str">
+        <x:v>OpenAI Stargate New Mexico</x:v>
+      </x:c>
+      <x:c r="B83" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C83" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D83" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E83" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F83" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G83" s="16" t="str"/>
+      <x:c r="H83" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A84" s="16" t="str">
+        <x:v>OpenAI Stargate Shackelford</x:v>
+      </x:c>
+      <x:c r="B84" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C84" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D84" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E84" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F84" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G84" s="16" t="str">
+        <x:v>175 Private Road 1604, Abilene, TX 79601, Shackelford County</x:v>
+      </x:c>
+      <x:c r="H84" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A85" s="16" t="str">
+        <x:v>OpenAI Stargate UAE</x:v>
+      </x:c>
+      <x:c r="B85" s="16" t="str">
+        <x:v>United Arab Emirates</x:v>
+      </x:c>
+      <x:c r="C85" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D85" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E85" s="16" t="str">
+        <x:v>G42 #likely</x:v>
+      </x:c>
+      <x:c r="F85" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G85" s="16" t="str">
+        <x:v>Nexus L&amp;T Project Office, Al Bihouth, Al Dhafrah, Abu Dhabi, United Arab Emirates</x:v>
+      </x:c>
+      <x:c r="H85" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A86" s="16" t="str">
+        <x:v>OpenAI Stargate Wisconsin</x:v>
+      </x:c>
+      <x:c r="B86" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C86" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D86" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E86" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F86" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G86" s="16" t="str"/>
+      <x:c r="H86" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A87" s="16" t="str">
+        <x:v>QTS Cedar Rapids</x:v>
+      </x:c>
+      <x:c r="B87" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C87" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D87" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E87" s="16" t="str"/>
+      <x:c r="F87" s="16" t="str"/>
+      <x:c r="G87" s="16" t="str">
+        <x:v>6200 76th Ave SW, Fairfax, IA 52228</x:v>
+      </x:c>
+      <x:c r="H87" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="54" hidden="0" customHeight="1">
+      <x:c r="A88" s="16" t="str">
+        <x:v>QTS Eagle Mountain</x:v>
+      </x:c>
+      <x:c r="B88" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C88" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D88" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E88" s="16" t="str"/>
+      <x:c r="F88" s="16" t="str">
+        <x:v>Meta #speculative</x:v>
+      </x:c>
+      <x:c r="G88" s="16" t="str">
+        <x:v>652 E Hyperscale Way, Eagle Mountain, UT 84013</x:v>
+      </x:c>
+      <x:c r="H88" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redf870736ded42b4"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2197,7 +4929,7 @@
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Source-reported global build-rate, geography, performance, and allocation estimates. These retain their original units and do not directly enter the U.S. H100e countdown.</x:v>
+        <x:v>Source-reported global build-rate, geography, performance, and allocation estimates. These retain their original units and do not directly enter the U.S. service-capacity countdown.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -2876,12 +5608,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b2ca95cf3dd450c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4a5a31959e94ab3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2995,7 +5727,7 @@
         <x:v>Expert-interview estimates from Dylan Patel of SemiAnalysis. The official transcript accompanies the video at https://www.youtube.com/watch?v=aV26V1UvkJw. Global GW flows and frontier-lab allocations are not directly merged with the U.S. H100e countdown path.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="140.39999389648438" hidden="0" customHeight="1">
+    <x:row r="8" ht="205.1999969482422" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
@@ -3009,35 +5741,58 @@
         <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>capacity observation, capacity projection</x:v>
+        <x:v>IT-power observation, IT-power projection, H100e productivity audit bridge</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
         <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="97.19999694824219" hidden="0" customHeight="1">
+        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff. U.S. geography is joined from Epoch’s data-center registry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="183.60000610351562" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>Epoch AI</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>AI Data Centers CSV</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>site registry, geography filter, facility audit</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_centers.csv</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>Country identifies the U.S. sites included in the quarterly timeline reconstruction. Current power is facility power, not IT power, and is retained only as an audit field.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="97.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A10" s="16" t="str">
         <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
+      <x:c r="B10" s="16" t="str">
         <x:v>U.S. Census Bureau</x:v>
       </x:c>
-      <x:c r="C9" s="16" t="str">
+      <x:c r="C10" s="16" t="str">
         <x:v>Population on a Date</x:v>
       </x:c>
-      <x:c r="D9" s="16" t="str">
+      <x:c r="D10" s="16" t="str">
         <x:v>2026-07-26</x:v>
       </x:c>
-      <x:c r="E9" s="16" t="str">
+      <x:c r="E10" s="16" t="str">
         <x:v>population</x:v>
       </x:c>
-      <x:c r="F9" s="16" t="str">
+      <x:c r="F10" s="16" t="str">
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
-      <x:c r="G9" s="16" t="str">
+      <x:c r="G10" s="16" t="str">
         <x:v>The model uses the rounded estimate of 342.8M residents; the selected 25% target is 85.7M users.</x:v>
       </x:c>
     </x:row>
@@ -3048,7 +5803,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74abcd047adb4503"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1fee499889d4d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct Epoch registry power provenance
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdc804ad509144c49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R2f32dad36a8a4433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R78776243a84f4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="4" r:id="R084aaf8ffdb64308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="5" r:id="R3b5bba938faf444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rf97b19625c8c4a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R39642e09814f4ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R3aa31b6328924413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rd65e9d4273eb4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="4" r:id="R11f5ea82184b433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="5" r:id="Reed9ec21704c4bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R90f63269603b4675"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -347,7 +347,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R918d344b1ee641f4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45d5d254cd5f4077"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -415,7 +415,7 @@
     <x:tableColumn id="1" name="Site"/>
     <x:tableColumn id="2" name="Country"/>
     <x:tableColumn id="3" name="Current H100e"/>
-    <x:tableColumn id="4" name="Current facility power MW"/>
+    <x:tableColumn id="4" name="Current IT power MW"/>
     <x:tableColumn id="5" name="Owner"/>
     <x:tableColumn id="6" name="Users"/>
     <x:tableColumn id="7" name="Address"/>
@@ -875,7 +875,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21c61a0b63024c85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ee2e39b16bf4db9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2423,9 +2423,9 @@
     <x:mergeCell ref="A3:V3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201462959a504813"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2de7559930ca47a6"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b79f065abae43f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec980a7eaccd4377"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2708,7 +2708,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202f59c91a1c4920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27de98fdc1d446ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2751,7 +2751,7 @@
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Facility-level source rows used to identify U.S. sites and audit the timeline join. Facility power includes non-IT overhead and is not substituted for IT power in the gate.</x:v>
+        <x:v>Facility-level source rows used to identify U.S. sites and audit current IT power. The quarterly gate path is reconstructed from the dated timeline.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -2762,7 +2762,7 @@
       <x:c r="H3" s="6"/>
     </x:row>
     <x:row r="4"/>
-    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>Site</x:v>
       </x:c>
@@ -2773,7 +2773,7 @@
         <x:v>Current H100e</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Current facility power MW</x:v>
+        <x:v>Current IT power MW</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>Owner</x:v>
@@ -4871,7 +4871,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redf870736ded42b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf05bb1b0646f4b83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5608,7 +5608,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4a5a31959e94ab3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76dbd5e7c0da4135"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5750,7 +5750,7 @@
         <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff. U.S. geography is joined from Epoch’s data-center registry.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="183.60000610351562" hidden="0" customHeight="1">
+    <x:row r="9" ht="270" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
@@ -5770,7 +5770,7 @@
         <x:v>https://epoch.ai/data/data_centers/data_centers.csv</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
-        <x:v>Country identifies the U.S. sites included in the quarterly timeline reconstruction. Current power is facility power, not IT power, and is retained only as an audit field.</x:v>
+        <x:v>Country identifies the U.S. sites included in the quarterly timeline reconstruction. Current power is the registry’s current IT-power estimate and is retained as a facility-level audit field; the quarterly gate path is reconstructed from the dated timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="97.19999694824219" hidden="0" customHeight="1">
@@ -5803,7 +5803,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1fee499889d4d1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8736dfb99f9d470f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct capability and compute forecast models
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R39642e09814f4ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R3aa31b6328924413"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rd65e9d4273eb4168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="4" r:id="R11f5ea82184b433c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="5" r:id="Reed9ec21704c4bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R90f63269603b4675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R14841b2bf70f4d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R0a091bef3a9248cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R9d80095689d04485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="R1a7fc35224b24bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R848ea7aeb0bb48e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="Rdc294570e7164d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Radf4a4a525064650"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,13 +19,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
-    <x:numFmt numFmtId="200" formatCode="0.0%"/>
-    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
-    <x:numFmt numFmtId="203" formatCode="0.0000"/>
-    <x:numFmt numFmtId="204" formatCode="#,##0"/>
-    <x:numFmt numFmtId="205" formatCode="0%"/>
+  <x:numFmts count="8">
+    <x:numFmt numFmtId="200" formatCode="#,##0.0000"/>
+    <x:numFmt numFmtId="201" formatCode="0.0%"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="0%"/>
+    <x:numFmt numFmtId="204" formatCode="0.000000"/>
+    <x:numFmt numFmtId="205" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="206" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="207" formatCode="0.0000"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -97,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -137,15 +140,6 @@
     <x:xf numFmtId="201" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="202" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -156,6 +150,33 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -177,7 +198,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Supported Personal-AI user-equivalents</a:t>
+              <a:t>Service-capacity gate crossing (chart capped at 5× target)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -207,9 +228,9 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Quarterly Model'!$P$6:$P$25</c:f>
+              <c:f>'Quarterly Model'!$Q$6:$Q$25</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0,,"M"</c:formatCode>
                 <c:ptCount val="0"/>
               </c:numCache>
             </c:numRef>
@@ -235,9 +256,9 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Quarterly Model'!$Q$6:$Q$25</c:f>
+              <c:f>'Quarterly Model'!$R$6:$R$25</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0,,"M"</c:formatCode>
                 <c:ptCount val="0"/>
               </c:numCache>
             </c:numRef>
@@ -284,6 +305,8 @@
         <c:axId val="48672768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="428500000"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -297,7 +320,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
+        <c:numFmt formatCode="0,,&quot;M&quot;"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:crossAx val="48650112"/>
@@ -347,7 +370,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45d5d254cd5f4077"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R90d224de0a6d4a2e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -357,7 +380,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComputeSummaryTable" displayName="ComputeSummaryTable" ref="A5:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComputeSummaryTable" displayName="ComputeSummaryTable" ref="A5:C24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Metric"/>
     <x:tableColumn id="2" name="Value"/>
@@ -368,8 +391,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComputeQuarterlyModelTable" displayName="ComputeQuarterlyModelTable" ref="A5:V25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="22">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ComputeQuarterlyModelTable" displayName="ComputeQuarterlyModelTable" ref="A5:W25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="23">
     <x:tableColumn id="1" name="Quarter index"/>
     <x:tableColumn id="2" name="Quarter"/>
     <x:tableColumn id="3" name="Cutoff"/>
@@ -380,25 +403,26 @@
     <x:tableColumn id="8" name="H100e audit bridge"/>
     <x:tableColumn id="9" name="Included sites"/>
     <x:tableColumn id="10" name="H100e / IT GW"/>
-    <x:tableColumn id="11" name="Productivity T token-eq / IT GW-day"/>
-    <x:tableColumn id="12" name="IT-power log growth / qtr"/>
-    <x:tableColumn id="13" name="Productivity log growth / qtr"/>
-    <x:tableColumn id="14" name="H100e log growth / qtr"/>
-    <x:tableColumn id="15" name="Personal-AI token-eq/day"/>
-    <x:tableColumn id="16" name="Supported users"/>
-    <x:tableColumn id="17" name="Target users"/>
-    <x:tableColumn id="18" name="Score vs target"/>
-    <x:tableColumn id="19" name="Letter"/>
-    <x:tableColumn id="20" name="GPA"/>
-    <x:tableColumn id="21" name="Source ID"/>
-    <x:tableColumn id="22" name="Method note"/>
+    <x:tableColumn id="11" name="H100e audit productivity T/GW-day"/>
+    <x:tableColumn id="12" name="Independent productivity T/GW-day"/>
+    <x:tableColumn id="13" name="IT-power log growth / qtr"/>
+    <x:tableColumn id="14" name="Productivity log growth / qtr"/>
+    <x:tableColumn id="15" name="H100e log growth / qtr"/>
+    <x:tableColumn id="16" name="Personal-AI token-eq/day"/>
+    <x:tableColumn id="17" name="Supported users"/>
+    <x:tableColumn id="18" name="Target users"/>
+    <x:tableColumn id="19" name="Score vs target"/>
+    <x:tableColumn id="20" name="Letter"/>
+    <x:tableColumn id="21" name="GPA"/>
+    <x:tableColumn id="22" name="Source ID"/>
+    <x:tableColumn id="23" name="Method note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ComputeAssumptionsTable" displayName="ComputeAssumptionsTable" ref="A5:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ComputeAssumptionsTable" displayName="ComputeAssumptionsTable" ref="A5:D18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Group"/>
     <x:tableColumn id="2" name="Variable"/>
@@ -410,7 +434,34 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComputeSiteRegistryTable" displayName="ComputeSiteRegistryTable" ref="A5:H88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="InferenceProductivityTable" displayName="InferenceProductivityTable" ref="A5:S8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="19">
+    <x:tableColumn id="1" name="Observation ID"/>
+    <x:tableColumn id="2" name="Release"/>
+    <x:tableColumn id="3" name="Date"/>
+    <x:tableColumn id="4" name="Model"/>
+    <x:tableColumn id="5" name="Scenario"/>
+    <x:tableColumn id="6" name="Submitter"/>
+    <x:tableColumn id="7" name="System"/>
+    <x:tableColumn id="8" name="Accelerator"/>
+    <x:tableColumn id="9" name="Count"/>
+    <x:tableColumn id="10" name="Active parameters"/>
+    <x:tableColumn id="11" name="Measured tokens/s"/>
+    <x:tableColumn id="12" name="Measured system W"/>
+    <x:tableColumn id="13" name="Tokens/J"/>
+    <x:tableColumn id="14" name="Reference productivity T/GW-day"/>
+    <x:tableColumn id="15" name="Role"/>
+    <x:tableColumn id="16" name="Raw result ID"/>
+    <x:tableColumn id="17" name="Source ID"/>
+    <x:tableColumn id="18" name="Source location"/>
+    <x:tableColumn id="19" name="Comparability note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSiteRegistryTable" displayName="ComputeSiteRegistryTable" ref="A5:H88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Site"/>
     <x:tableColumn id="2" name="Country"/>
@@ -425,8 +476,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Metric"/>
@@ -446,8 +497,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -693,178 +744,211 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="64.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A6" s="19" t="str">
+      <x:c r="A6" s="23" t="str">
         <x:v>Snapshot</x:v>
       </x:c>
-      <x:c r="B6" s="19" t="str">
+      <x:c r="B6" s="23" t="str">
         <x:v>2026-08-26</x:v>
       </x:c>
-      <x:c r="C6" s="19" t="str">
+      <x:c r="C6" s="23" t="str">
         <x:v>Latest immutable snapshot selected automatically</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A7" s="19" t="str">
+      <x:c r="A7" s="23" t="str">
         <x:v>Current U.S. operational IT power</x:v>
       </x:c>
-      <x:c r="B7" s="19" t="n">
+      <x:c r="B7" s="24" t="n">
         <x:v>11.87932971</x:v>
       </x:c>
-      <x:c r="C7" s="19" t="str">
+      <x:c r="C7" s="23" t="str">
         <x:v>IT GW</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" hidden="0" customHeight="1">
-      <x:c r="A8" s="19" t="str">
+      <x:c r="A8" s="23" t="str">
         <x:v>Current reference inference productivity</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="B8" s="24" t="n">
+        <x:v>45.688453485748845</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>trillion reference token-equivalents / IT GW-day</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>Productivity baseline result</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>mlperf-v5-1-llama31-405b-server-b200</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>llama3.1-405b Server</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>Measured baseline goodput</x:v>
+      </x:c>
+      <x:c r="B10" s="24" t="n">
+        <x:v>1249.04</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>tokens / second</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A11" s="23" t="str">
+        <x:v>Measured baseline system power</x:v>
+      </x:c>
+      <x:c r="B11" s="24" t="n">
+        <x:v>9566.1823383085</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str">
+        <x:v>watts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>Current H100e audit cross-check</x:v>
+      </x:c>
+      <x:c r="B12" s="24" t="n">
+        <x:v>13524006</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>audit only; excluded from capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>H100e-derived audit productivity</x:v>
+      </x:c>
+      <x:c r="B13" s="24" t="n">
         <x:v>227.10136510717322</x:v>
       </x:c>
-      <x:c r="C8" s="19" t="str">
-        <x:v>trillion reference token-equivalents / IT GW-day</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A9" s="19" t="str">
-        <x:v>Current H100e audit bridge</x:v>
-      </x:c>
-      <x:c r="B9" s="19" t="n">
-        <x:v>13524006</x:v>
-      </x:c>
-      <x:c r="C9" s="19" t="str">
-        <x:v>secondary productivity calibration</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A10" s="19" t="str">
+      <x:c r="C13" s="23" t="str">
+        <x:v>trillion reference token-equivalents / IT GW-day; audit only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A14" s="23" t="str">
         <x:v>Current supported users</x:v>
       </x:c>
-      <x:c r="B10" s="19" t="n">
-        <x:v>38655216.62613779</x:v>
-      </x:c>
-      <x:c r="C10" s="19" t="str">
+      <x:c r="B14" s="24" t="n">
+        <x:v>7776690.668377926</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
         <x:v>Personal-AI user-equivalents</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A11" s="19" t="str">
+    <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A15" s="23" t="str">
         <x:v>Target users</x:v>
       </x:c>
-      <x:c r="B11" s="19" t="n">
+      <x:c r="B15" s="24" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="C11" s="19" t="str">
+      <x:c r="C15" s="23" t="str">
         <x:v>25% of U.S. population</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A12" s="19" t="str">
+    <x:row r="16" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
         <x:v>Current supply score</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="n">
-        <x:v>0.45105270275540016</x:v>
-      </x:c>
-      <x:c r="C12" s="19" t="str">
+      <x:c r="B16" s="25" t="n">
+        <x:v>0.09074318166135269</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
         <x:v>supported users / target users</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="54" hidden="0" customHeight="1">
-      <x:c r="A13" s="19" t="str">
-        <x:v>Reference tokens per H100e/day</x:v>
-      </x:c>
-      <x:c r="B13" s="19" t="n">
-        <x:v>199483200</x:v>
-      </x:c>
-      <x:c r="C13" s="19" t="str">
-        <x:v>excludes inference and Personal-AI allocations</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A14" s="19" t="str">
+    <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="str">
         <x:v>Workload per user/day</x:v>
       </x:c>
-      <x:c r="B14" s="19" t="n">
+      <x:c r="B17" s="26" t="n">
         <x:v>16750000</x:v>
       </x:c>
-      <x:c r="C14" s="19" t="str">
+      <x:c r="C17" s="23" t="str">
         <x:v>compute-equivalent tokens</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A15" s="19" t="str">
+    <x:row r="18" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="str">
         <x:v>Fleet inference allocation</x:v>
       </x:c>
-      <x:c r="B15" s="20" t="n">
+      <x:c r="B18" s="27" t="n">
         <x:v>0.4</x:v>
       </x:c>
-      <x:c r="C15" s="19" t="str">
+      <x:c r="C18" s="23" t="str">
         <x:v>scenario allocation</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A16" s="19" t="str">
+    <x:row r="19" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="str">
         <x:v>Personal-AI inference share</x:v>
       </x:c>
-      <x:c r="B16" s="20" t="n">
+      <x:c r="B19" s="27" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="C16" s="19" t="str">
+      <x:c r="C19" s="23" t="str">
         <x:v>share of inference allocated to Personal AI</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A17" s="19" t="str">
+    <x:row r="20" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="str">
         <x:v>IT-power mean projected log velocity</x:v>
       </x:c>
-      <x:c r="B17" s="19" t="n">
+      <x:c r="B20" s="28" t="n">
         <x:v>0.15720673944051156</x:v>
       </x:c>
-      <x:c r="C17" s="19" t="str">
+      <x:c r="C20" s="23" t="str">
         <x:v>log₂ IT GW / quarter</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A18" s="19" t="str">
+    <x:row r="21" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="str">
         <x:v>IT-power projected log acceleration</x:v>
       </x:c>
-      <x:c r="B18" s="19" t="n">
+      <x:c r="B21" s="28" t="n">
         <x:v>-0.0015030413270408216</x:v>
       </x:c>
-      <x:c r="C18" s="19" t="str">
+      <x:c r="C21" s="23" t="str">
         <x:v>log₂ IT GW / quarter²</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A19" s="19" t="str">
-        <x:v>Productivity mean projected log velocity</x:v>
-      </x:c>
-      <x:c r="B19" s="19" t="n">
-        <x:v>0.08658381787604459</x:v>
-      </x:c>
-      <x:c r="C19" s="19" t="str">
-        <x:v>log₂ token productivity / quarter</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A20" s="19" t="str">
-        <x:v>Productivity projected log acceleration</x:v>
-      </x:c>
-      <x:c r="B20" s="19" t="n">
-        <x:v>0.004875694323320446</x:v>
-      </x:c>
-      <x:c r="C20" s="19" t="str">
-        <x:v>log₂ token productivity / quarter²</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A21" s="19" t="str">
+    <x:row r="22" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>Productivity measured log velocity</x:v>
+      </x:c>
+      <x:c r="B22" s="28" t="n">
+        <x:v>0.8530245754425125</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>log₂ token productivity / quarter; matched MLPerf series</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="54" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="str">
+        <x:v>Productivity measured log acceleration</x:v>
+      </x:c>
+      <x:c r="B23" s="28" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str">
+        <x:v>log₂ token productivity / quarter²; zero with two points</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="str">
         <x:v>Continuous base-case crossing</x:v>
       </x:c>
-      <x:c r="B21" s="21" t="n">
-        <x:v>46751.054552650465</x:v>
-      </x:c>
-      <x:c r="C21" s="19" t="str">
+      <x:c r="B24" s="29" t="n">
+        <x:v>46603.441982048615</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
         <x:v>100% of selected target</x:v>
       </x:c>
     </x:row>
@@ -875,7 +959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ee2e39b16bf4db9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9325a32037e4a17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -894,19 +978,19 @@
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="9" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="9" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="58" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="3" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="9" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="58" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="3" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="3" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="3" hidden="0" customWidth="1"/>
@@ -943,6 +1027,7 @@
       <x:c r="T1" s="3"/>
       <x:c r="U1" s="3"/>
       <x:c r="V1" s="3"/>
+      <x:c r="W1" s="3"/>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3"/>
@@ -967,6 +1052,7 @@
       <x:c r="T2" s="3"/>
       <x:c r="U2" s="3"/>
       <x:c r="V2" s="3"/>
+      <x:c r="W2" s="3"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -993,6 +1079,7 @@
       <x:c r="T3" s="6"/>
       <x:c r="U3" s="6"/>
       <x:c r="V3" s="6"/>
+      <x:c r="W3" s="6"/>
     </x:row>
     <x:row r="4"/>
     <x:row r="5" ht="66" hidden="0" customHeight="1">
@@ -1027,39 +1114,42 @@
         <x:v>H100e / IT GW</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
-        <x:v>Productivity T token-eq / IT GW-day</x:v>
+        <x:v>H100e audit productivity T/GW-day</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
+        <x:v>Independent productivity T/GW-day</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
         <x:v>IT-power log growth / qtr</x:v>
       </x:c>
-      <x:c r="M5" s="12" t="str">
+      <x:c r="N5" s="12" t="str">
         <x:v>Productivity log growth / qtr</x:v>
       </x:c>
-      <x:c r="N5" s="12" t="str">
+      <x:c r="O5" s="12" t="str">
         <x:v>H100e log growth / qtr</x:v>
       </x:c>
-      <x:c r="O5" s="12" t="str">
+      <x:c r="P5" s="12" t="str">
         <x:v>Personal-AI token-eq/day</x:v>
       </x:c>
-      <x:c r="P5" s="12" t="str">
+      <x:c r="Q5" s="12" t="str">
         <x:v>Supported users</x:v>
       </x:c>
-      <x:c r="Q5" s="12" t="str">
+      <x:c r="R5" s="12" t="str">
         <x:v>Target users</x:v>
       </x:c>
-      <x:c r="R5" s="12" t="str">
+      <x:c r="S5" s="12" t="str">
         <x:v>Score vs target</x:v>
       </x:c>
-      <x:c r="S5" s="12" t="str">
+      <x:c r="T5" s="12" t="str">
         <x:v>Letter</x:v>
       </x:c>
-      <x:c r="T5" s="12" t="str">
+      <x:c r="U5" s="12" t="str">
         <x:v>GPA</x:v>
       </x:c>
-      <x:c r="U5" s="12" t="str">
+      <x:c r="V5" s="12" t="str">
         <x:v>Source ID</x:v>
       </x:c>
-      <x:c r="V5" s="12" t="str">
+      <x:c r="W5" s="12" t="str">
         <x:v>Method note</x:v>
       </x:c>
     </x:row>
@@ -1070,58 +1160,61 @@
       <x:c r="B6" s="16" t="str">
         <x:v>2024-Q1</x:v>
       </x:c>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="22" t="str">
         <x:v>2024-03-31</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
+      <x:c r="E6" s="30" t="n">
         <x:v>473</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="n">
+      <x:c r="F6" s="30" t="n">
         <x:v>0.473</x:v>
       </x:c>
-      <x:c r="G6" s="22" t="n">
+      <x:c r="G6" s="30" t="n">
         <x:v>603</x:v>
       </x:c>
-      <x:c r="H6" s="22" t="n">
+      <x:c r="H6" s="30" t="n">
         <x:v>245664</x:v>
       </x:c>
-      <x:c r="I6" s="22" t="n">
+      <x:c r="I6" s="30" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J6" s="22" t="n">
+      <x:c r="J6" s="30" t="n">
         <x:v>519374.2071881607</x:v>
       </x:c>
-      <x:c r="K6" s="23" t="n">
+      <x:c r="K6" s="31" t="n">
         <x:v>103.6064288473573</x:v>
       </x:c>
-      <x:c r="L6" s="23"/>
-      <x:c r="M6" s="23"/>
-      <x:c r="N6" s="23"/>
-      <x:c r="O6" s="24" t="n">
-        <x:v>11761401802752</x:v>
-      </x:c>
-      <x:c r="P6" s="24" t="n">
-        <x:v>702173.2419553433</x:v>
-      </x:c>
-      <x:c r="Q6" s="24" t="n">
+      <x:c r="L6" s="31" t="n">
+        <x:v>0.12357955167820671</x:v>
+      </x:c>
+      <x:c r="M6" s="31"/>
+      <x:c r="N6" s="31"/>
+      <x:c r="O6" s="31"/>
+      <x:c r="P6" s="19" t="n">
+        <x:v>14028750706.510025</x:v>
+      </x:c>
+      <x:c r="Q6" s="19" t="n">
+        <x:v>837.5373556125388</x:v>
+      </x:c>
+      <x:c r="R6" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R6" s="17" t="n">
-        <x:v>0.008193386720599105</x:v>
-      </x:c>
-      <x:c r="S6" s="16" t="str">
+      <x:c r="S6" s="18" t="n">
+        <x:v>0.000009772897965140476</x:v>
+      </x:c>
+      <x:c r="T6" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T6" s="16" t="n">
+      <x:c r="U6" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U6" s="16" t="str">
+      <x:c r="V6" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V6" s="16" t="str">
+      <x:c r="W6" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1132,64 +1225,67 @@
       <x:c r="B7" s="16" t="str">
         <x:v>2024-Q2</x:v>
       </x:c>
-      <x:c r="C7" s="18" t="str">
+      <x:c r="C7" s="22" t="str">
         <x:v>2024-06-30</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="n">
+      <x:c r="E7" s="30" t="n">
         <x:v>887</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="n">
+      <x:c r="F7" s="30" t="n">
         <x:v>0.887</x:v>
       </x:c>
-      <x:c r="G7" s="22" t="n">
+      <x:c r="G7" s="30" t="n">
         <x:v>1121</x:v>
       </x:c>
-      <x:c r="H7" s="22" t="n">
+      <x:c r="H7" s="30" t="n">
         <x:v>475238</x:v>
       </x:c>
-      <x:c r="I7" s="22" t="n">
+      <x:c r="I7" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="J7" s="22" t="n">
+      <x:c r="J7" s="30" t="n">
         <x:v>535781.2852311161</x:v>
       </x:c>
-      <x:c r="K7" s="23" t="n">
+      <x:c r="K7" s="31" t="n">
         <x:v>106.87936527801578</x:v>
       </x:c>
-      <x:c r="L7" s="23" t="n">
+      <x:c r="L7" s="31" t="n">
+        <x:v>0.22321974084820626</x:v>
+      </x:c>
+      <x:c r="M7" s="31" t="n">
         <x:v>0.9070939209616689</x:v>
       </x:c>
-      <x:c r="M7" s="23" t="n">
-        <x:v>0.044869819268406275</x:v>
-      </x:c>
-      <x:c r="N7" s="23" t="n">
+      <x:c r="N7" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O7" s="31" t="n">
         <x:v>0.9519637402300738</x:v>
       </x:c>
-      <x:c r="O7" s="24" t="n">
-        <x:v>22752479280384</x:v>
-      </x:c>
-      <x:c r="P7" s="24" t="n">
-        <x:v>1358356.9719632238</x:v>
-      </x:c>
-      <x:c r="Q7" s="24" t="n">
+      <x:c r="P7" s="19" t="n">
+        <x:v>47519018431.76615</x:v>
+      </x:c>
+      <x:c r="Q7" s="19" t="n">
+        <x:v>2836.9563242845466</x:v>
+      </x:c>
+      <x:c r="R7" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R7" s="17" t="n">
-        <x:v>0.015850139696186975</x:v>
-      </x:c>
-      <x:c r="S7" s="16" t="str">
+      <x:c r="S7" s="18" t="n">
+        <x:v>0.00003310334100682085</x:v>
+      </x:c>
+      <x:c r="T7" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T7" s="16" t="n">
+      <x:c r="U7" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U7" s="16" t="str">
+      <x:c r="V7" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V7" s="16" t="str">
+      <x:c r="W7" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1200,64 +1296,67 @@
       <x:c r="B8" s="16" t="str">
         <x:v>2024-Q3</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
+      <x:c r="C8" s="22" t="str">
         <x:v>2024-09-30</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="n">
+      <x:c r="E8" s="30" t="n">
         <x:v>1335</x:v>
       </x:c>
-      <x:c r="F8" s="22" t="n">
+      <x:c r="F8" s="30" t="n">
         <x:v>1.335</x:v>
       </x:c>
-      <x:c r="G8" s="22" t="n">
+      <x:c r="G8" s="30" t="n">
         <x:v>1676</x:v>
       </x:c>
-      <x:c r="H8" s="22" t="n">
+      <x:c r="H8" s="30" t="n">
         <x:v>722180</x:v>
       </x:c>
-      <x:c r="I8" s="22" t="n">
+      <x:c r="I8" s="30" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="J8" s="22" t="n">
+      <x:c r="J8" s="30" t="n">
         <x:v>540958.8014981274</x:v>
       </x:c>
-      <x:c r="K8" s="23" t="n">
+      <x:c r="K8" s="31" t="n">
         <x:v>107.91219279101125</x:v>
       </x:c>
-      <x:c r="L8" s="23" t="n">
+      <x:c r="L8" s="31" t="n">
+        <x:v>0.40319819927884876</x:v>
+      </x:c>
+      <x:c r="M8" s="31" t="n">
         <x:v>0.5898337322738523</x:v>
       </x:c>
-      <x:c r="M8" s="23" t="n">
-        <x:v>0.013874536121321057</x:v>
-      </x:c>
-      <x:c r="N8" s="23" t="n">
+      <x:c r="N8" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O8" s="31" t="n">
         <x:v>0.6037082683951738</x:v>
       </x:c>
-      <x:c r="O8" s="24" t="n">
-        <x:v>34575066570240</x:v>
-      </x:c>
-      <x:c r="P8" s="24" t="n">
-        <x:v>2064183.0788202984</x:v>
-      </x:c>
-      <x:c r="Q8" s="24" t="n">
+      <x:c r="P8" s="19" t="n">
+        <x:v>129184703048.94315</x:v>
+      </x:c>
+      <x:c r="Q8" s="19" t="n">
+        <x:v>7712.5195850115315</x:v>
+      </x:c>
+      <x:c r="R8" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R8" s="17" t="n">
-        <x:v>0.024086150277949806</x:v>
-      </x:c>
-      <x:c r="S8" s="16" t="str">
+      <x:c r="S8" s="18" t="n">
+        <x:v>0.0000899943942241719</x:v>
+      </x:c>
+      <x:c r="T8" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T8" s="16" t="n">
+      <x:c r="U8" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U8" s="16" t="str">
+      <x:c r="V8" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V8" s="16" t="str">
+      <x:c r="W8" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1268,64 +1367,67 @@
       <x:c r="B9" s="16" t="str">
         <x:v>2024-Q4</x:v>
       </x:c>
-      <x:c r="C9" s="18" t="str">
+      <x:c r="C9" s="22" t="str">
         <x:v>2024-12-31</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E9" s="22" t="n">
+      <x:c r="E9" s="30" t="n">
         <x:v>1713</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="n">
+      <x:c r="F9" s="30" t="n">
         <x:v>1.713</x:v>
       </x:c>
-      <x:c r="G9" s="22" t="n">
+      <x:c r="G9" s="30" t="n">
         <x:v>2165</x:v>
       </x:c>
-      <x:c r="H9" s="22" t="n">
+      <x:c r="H9" s="30" t="n">
         <x:v>1012483</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="n">
+      <x:c r="I9" s="30" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="J9" s="22" t="n">
+      <x:c r="J9" s="30" t="n">
         <x:v>591058.3771161705</x:v>
       </x:c>
-      <x:c r="K9" s="23" t="n">
+      <x:c r="K9" s="31" t="n">
         <x:v>117.90621645394046</x:v>
       </x:c>
-      <x:c r="L9" s="23" t="n">
+      <x:c r="L9" s="31" t="n">
+        <x:v>0.7282903711112904</x:v>
+      </x:c>
+      <x:c r="M9" s="31" t="n">
         <x:v>0.35968540950908284</x:v>
       </x:c>
-      <x:c r="M9" s="23" t="n">
-        <x:v>0.1277819031953058</x:v>
-      </x:c>
-      <x:c r="N9" s="23" t="n">
+      <x:c r="N9" s="31" t="n">
+        <x:v>0.8530245754425181</x:v>
+      </x:c>
+      <x:c r="O9" s="31" t="n">
         <x:v>0.48746731270438204</x:v>
       </x:c>
-      <x:c r="O9" s="24" t="n">
-        <x:v>48473603708544</x:v>
-      </x:c>
-      <x:c r="P9" s="24" t="n">
-        <x:v>2893946.4900623285</x:v>
-      </x:c>
-      <x:c r="Q9" s="24" t="n">
+      <x:c r="P9" s="19" t="n">
+        <x:v>299414737371.27374</x:v>
+      </x:c>
+      <x:c r="Q9" s="19" t="n">
+        <x:v>17875.506708732762</x:v>
+      </x:c>
+      <x:c r="R9" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R9" s="17" t="n">
-        <x:v>0.03376833710691165</x:v>
-      </x:c>
-      <x:c r="S9" s="16" t="str">
+      <x:c r="S9" s="18" t="n">
+        <x:v>0.00020858234199221427</x:v>
+      </x:c>
+      <x:c r="T9" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T9" s="16" t="n">
+      <x:c r="U9" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U9" s="16" t="str">
+      <x:c r="V9" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V9" s="16" t="str">
+      <x:c r="W9" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1336,64 +1438,67 @@
       <x:c r="B10" s="16" t="str">
         <x:v>2025-Q1</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
+      <x:c r="C10" s="22" t="str">
         <x:v>2025-03-31</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E10" s="22" t="n">
+      <x:c r="E10" s="30" t="n">
         <x:v>2267.32971</x:v>
       </x:c>
-      <x:c r="F10" s="22" t="n">
+      <x:c r="F10" s="30" t="n">
         <x:v>2.26732971</x:v>
       </x:c>
-      <x:c r="G10" s="22" t="n">
+      <x:c r="G10" s="30" t="n">
         <x:v>2874</x:v>
       </x:c>
-      <x:c r="H10" s="22" t="n">
+      <x:c r="H10" s="30" t="n">
         <x:v>1351240</x:v>
       </x:c>
-      <x:c r="I10" s="22" t="n">
+      <x:c r="I10" s="30" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="J10" s="22" t="n">
+      <x:c r="J10" s="30" t="n">
         <x:v>595960.9641422641</x:v>
       </x:c>
-      <x:c r="K10" s="23" t="n">
+      <x:c r="K10" s="31" t="n">
         <x:v>118.88420020218409</x:v>
       </x:c>
-      <x:c r="L10" s="23" t="n">
+      <x:c r="L10" s="31" t="n">
+        <x:v>1.3154990910229631</x:v>
+      </x:c>
+      <x:c r="M10" s="31" t="n">
         <x:v>0.4044690483884812</x:v>
       </x:c>
-      <x:c r="M10" s="23" t="n">
-        <x:v>0.011917208021813508</x:v>
-      </x:c>
-      <x:c r="N10" s="23" t="n">
+      <x:c r="N10" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O10" s="31" t="n">
         <x:v>0.416386256410302</x:v>
       </x:c>
-      <x:c r="O10" s="24" t="n">
-        <x:v>64691923000320</x:v>
-      </x:c>
-      <x:c r="P10" s="24" t="n">
-        <x:v>3862204.3582280595</x:v>
-      </x:c>
-      <x:c r="Q10" s="24" t="n">
+      <x:c r="P10" s="19" t="n">
+        <x:v>715840841413.046</x:v>
+      </x:c>
+      <x:c r="Q10" s="19" t="n">
+        <x:v>42736.76665152513</x:v>
+      </x:c>
+      <x:c r="R10" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R10" s="17" t="n">
-        <x:v>0.04506656193965063</x:v>
-      </x:c>
-      <x:c r="S10" s="16" t="str">
+      <x:c r="S10" s="18" t="n">
+        <x:v>0.0004986787240551357</x:v>
+      </x:c>
+      <x:c r="T10" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T10" s="16" t="n">
+      <x:c r="U10" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U10" s="16" t="str">
+      <x:c r="V10" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V10" s="16" t="str">
+      <x:c r="W10" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1404,64 +1509,67 @@
       <x:c r="B11" s="16" t="str">
         <x:v>2025-Q2</x:v>
       </x:c>
-      <x:c r="C11" s="18" t="str">
+      <x:c r="C11" s="22" t="str">
         <x:v>2025-06-30</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E11" s="22" t="n">
+      <x:c r="E11" s="30" t="n">
         <x:v>3342.32971</x:v>
       </x:c>
-      <x:c r="F11" s="22" t="n">
+      <x:c r="F11" s="30" t="n">
         <x:v>3.34232971</x:v>
       </x:c>
-      <x:c r="G11" s="22" t="n">
+      <x:c r="G11" s="30" t="n">
         <x:v>4187</x:v>
       </x:c>
-      <x:c r="H11" s="22" t="n">
+      <x:c r="H11" s="30" t="n">
         <x:v>2386876</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="n">
+      <x:c r="I11" s="30" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="n">
+      <x:c r="J11" s="30" t="n">
         <x:v>714135.410656419</x:v>
       </x:c>
-      <x:c r="K11" s="23" t="n">
+      <x:c r="K11" s="31" t="n">
         <x:v>142.45801695105655</x:v>
       </x:c>
-      <x:c r="L11" s="23" t="n">
+      <x:c r="L11" s="31" t="n">
+        <x:v>2.3761646825587324</x:v>
+      </x:c>
+      <x:c r="M11" s="31" t="n">
         <x:v>0.5598598578015919</x:v>
       </x:c>
-      <x:c r="M11" s="23" t="n">
-        <x:v>0.26097982029811817</x:v>
-      </x:c>
-      <x:c r="N11" s="23" t="n">
+      <x:c r="N11" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O11" s="31" t="n">
         <x:v>0.8208396780997056</x:v>
       </x:c>
-      <x:c r="O11" s="24" t="n">
-        <x:v>114273998995968</x:v>
-      </x:c>
-      <x:c r="P11" s="24" t="n">
-        <x:v>6822328.298266746</x:v>
-      </x:c>
-      <x:c r="Q11" s="24" t="n">
+      <x:c r="P11" s="19" t="n">
+        <x:v>1906062195448.505</x:v>
+      </x:c>
+      <x:c r="Q11" s="19" t="n">
+        <x:v>113794.75793722417</x:v>
+      </x:c>
+      <x:c r="R11" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R11" s="17" t="n">
-        <x:v>0.07960709799611139</x:v>
-      </x:c>
-      <x:c r="S11" s="16" t="str">
+      <x:c r="S11" s="18" t="n">
+        <x:v>0.0013278268137365714</x:v>
+      </x:c>
+      <x:c r="T11" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T11" s="16" t="n">
+      <x:c r="U11" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U11" s="16" t="str">
+      <x:c r="V11" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V11" s="16" t="str">
+      <x:c r="W11" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1472,64 +1580,67 @@
       <x:c r="B12" s="16" t="str">
         <x:v>2025-Q3</x:v>
       </x:c>
-      <x:c r="C12" s="18" t="str">
+      <x:c r="C12" s="22" t="str">
         <x:v>2025-09-30</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E12" s="22" t="n">
+      <x:c r="E12" s="30" t="n">
         <x:v>3772.32971</x:v>
       </x:c>
-      <x:c r="F12" s="22" t="n">
+      <x:c r="F12" s="30" t="n">
         <x:v>3.77232971</x:v>
       </x:c>
-      <x:c r="G12" s="22" t="n">
+      <x:c r="G12" s="30" t="n">
         <x:v>4764</x:v>
       </x:c>
-      <x:c r="H12" s="22" t="n">
+      <x:c r="H12" s="30" t="n">
         <x:v>3139660</x:v>
       </x:c>
-      <x:c r="I12" s="22" t="n">
+      <x:c r="I12" s="30" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="J12" s="22" t="n">
+      <x:c r="J12" s="30" t="n">
         <x:v>832286.7409169279</x:v>
       </x:c>
-      <x:c r="K12" s="23" t="n">
+      <x:c r="K12" s="31" t="n">
         <x:v>166.02722239567973</x:v>
       </x:c>
-      <x:c r="L12" s="23" t="n">
+      <x:c r="L12" s="31" t="n">
+        <x:v>4.292027746099666</x:v>
+      </x:c>
+      <x:c r="M12" s="31" t="n">
         <x:v>0.17460171866453855</x:v>
       </x:c>
-      <x:c r="M12" s="23" t="n">
-        <x:v>0.22088299733157157</x:v>
-      </x:c>
-      <x:c r="N12" s="23" t="n">
+      <x:c r="N12" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O12" s="31" t="n">
         <x:v>0.3954847159961119</x:v>
       </x:c>
-      <x:c r="O12" s="24" t="n">
-        <x:v>150314261690880</x:v>
-      </x:c>
-      <x:c r="P12" s="24" t="n">
-        <x:v>8973985.772589851</x:v>
-      </x:c>
-      <x:c r="Q12" s="24" t="n">
+      <x:c r="P12" s="19" t="n">
+        <x:v>3885826507861.4653</x:v>
+      </x:c>
+      <x:c r="Q12" s="19" t="n">
+        <x:v>231989.642260386</x:v>
+      </x:c>
+      <x:c r="R12" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R12" s="17" t="n">
-        <x:v>0.10471395300571588</x:v>
-      </x:c>
-      <x:c r="S12" s="16" t="str">
+      <x:c r="S12" s="18" t="n">
+        <x:v>0.0027069969925365926</x:v>
+      </x:c>
+      <x:c r="T12" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T12" s="16" t="n">
+      <x:c r="U12" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U12" s="16" t="str">
+      <x:c r="V12" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V12" s="16" t="str">
+      <x:c r="W12" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1540,64 +1651,67 @@
       <x:c r="B13" s="16" t="str">
         <x:v>2025-Q4</x:v>
       </x:c>
-      <x:c r="C13" s="18" t="str">
+      <x:c r="C13" s="22" t="str">
         <x:v>2025-12-31</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E13" s="22" t="n">
+      <x:c r="E13" s="30" t="n">
         <x:v>5642.32971</x:v>
       </x:c>
-      <x:c r="F13" s="22" t="n">
+      <x:c r="F13" s="30" t="n">
         <x:v>5.64232971</x:v>
       </x:c>
-      <x:c r="G13" s="22" t="n">
+      <x:c r="G13" s="30" t="n">
         <x:v>7211</x:v>
       </x:c>
-      <x:c r="H13" s="22" t="n">
+      <x:c r="H13" s="30" t="n">
         <x:v>5291375</x:v>
       </x:c>
-      <x:c r="I13" s="22" t="n">
+      <x:c r="I13" s="30" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="J13" s="22" t="n">
+      <x:c r="J13" s="30" t="n">
         <x:v>937799.6806216416</x:v>
       </x:c>
-      <x:c r="K13" s="23" t="n">
+      <x:c r="K13" s="31" t="n">
         <x:v>187.07528124938307</x:v>
       </x:c>
-      <x:c r="L13" s="23" t="n">
+      <x:c r="L13" s="31" t="n">
+        <x:v>7.752620139717122</x:v>
+      </x:c>
+      <x:c r="M13" s="31" t="n">
         <x:v>0.580835196113413</x:v>
       </x:c>
-      <x:c r="M13" s="23" t="n">
-        <x:v>0.1721991338495812</x:v>
-      </x:c>
-      <x:c r="N13" s="23" t="n">
+      <x:c r="N13" s="31" t="n">
+        <x:v>0.8530245754425181</x:v>
+      </x:c>
+      <x:c r="O13" s="31" t="n">
         <x:v>0.7530343299629934</x:v>
       </x:c>
-      <x:c r="O13" s="24" t="n">
-        <x:v>253329700176000</x:v>
-      </x:c>
-      <x:c r="P13" s="24" t="n">
-        <x:v>15124161.204537313</x:v>
-      </x:c>
-      <x:c r="Q13" s="24" t="n">
+      <x:c r="P13" s="19" t="n">
+        <x:v>10498281346720.865</x:v>
+      </x:c>
+      <x:c r="Q13" s="19" t="n">
+        <x:v>626763.0654758726</x:v>
+      </x:c>
+      <x:c r="R13" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R13" s="17" t="n">
-        <x:v>0.17647796037966526</x:v>
-      </x:c>
-      <x:c r="S13" s="16" t="str">
+      <x:c r="S13" s="18" t="n">
+        <x:v>0.007313454672997347</x:v>
+      </x:c>
+      <x:c r="T13" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T13" s="16" t="n">
+      <x:c r="U13" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U13" s="16" t="str">
+      <x:c r="V13" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V13" s="16" t="str">
+      <x:c r="W13" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1608,64 +1722,67 @@
       <x:c r="B14" s="16" t="str">
         <x:v>2026-Q1</x:v>
       </x:c>
-      <x:c r="C14" s="18" t="str">
+      <x:c r="C14" s="22" t="str">
         <x:v>2026-03-31</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E14" s="22" t="n">
+      <x:c r="E14" s="30" t="n">
         <x:v>6620.32971</x:v>
       </x:c>
-      <x:c r="F14" s="22" t="n">
+      <x:c r="F14" s="30" t="n">
         <x:v>6.62032971</x:v>
       </x:c>
-      <x:c r="G14" s="22" t="n">
+      <x:c r="G14" s="30" t="n">
         <x:v>8454.2</x:v>
       </x:c>
-      <x:c r="H14" s="22" t="n">
+      <x:c r="H14" s="30" t="n">
         <x:v>6301294</x:v>
       </x:c>
-      <x:c r="I14" s="22" t="n">
+      <x:c r="I14" s="30" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J14" s="22" t="n">
+      <x:c r="J14" s="30" t="n">
         <x:v>951809.6946866412</x:v>
       </x:c>
-      <x:c r="K14" s="23" t="n">
+      <x:c r="K14" s="31" t="n">
         <x:v>189.8700436871142</x:v>
       </x:c>
-      <x:c r="L14" s="23" t="n">
+      <x:c r="L14" s="31" t="n">
+        <x:v>14.003432080644302</x:v>
+      </x:c>
+      <x:c r="M14" s="31" t="n">
         <x:v>0.2306120964759244</x:v>
       </x:c>
-      <x:c r="M14" s="23" t="n">
-        <x:v>0.021393361454933313</x:v>
-      </x:c>
-      <x:c r="N14" s="23" t="n">
+      <x:c r="N14" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O14" s="31" t="n">
         <x:v>0.25200545793085993</x:v>
       </x:c>
-      <x:c r="O14" s="24" t="n">
-        <x:v>301680549902592</x:v>
-      </x:c>
-      <x:c r="P14" s="24" t="n">
-        <x:v>18010779.09866221</x:v>
-      </x:c>
-      <x:c r="Q14" s="24" t="n">
+      <x:c r="P14" s="19" t="n">
+        <x:v>22249760986909.582</x:v>
+      </x:c>
+      <x:c r="Q14" s="19" t="n">
+        <x:v>1328343.93951699</x:v>
+      </x:c>
+      <x:c r="R14" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R14" s="17" t="n">
-        <x:v>0.21016078294821713</x:v>
-      </x:c>
-      <x:c r="S14" s="16" t="str">
+      <x:c r="S14" s="18" t="n">
+        <x:v>0.015499929282578645</x:v>
+      </x:c>
+      <x:c r="T14" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T14" s="16" t="n">
+      <x:c r="U14" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U14" s="16" t="str">
+      <x:c r="V14" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V14" s="16" t="str">
+      <x:c r="W14" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1676,64 +1793,67 @@
       <x:c r="B15" s="16" t="str">
         <x:v>2026-Q2</x:v>
       </x:c>
-      <x:c r="C15" s="18" t="str">
+      <x:c r="C15" s="22" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
         <x:v>observed_quarter_end</x:v>
       </x:c>
-      <x:c r="E15" s="22" t="n">
+      <x:c r="E15" s="30" t="n">
         <x:v>10534.32971</x:v>
       </x:c>
-      <x:c r="F15" s="22" t="n">
+      <x:c r="F15" s="30" t="n">
         <x:v>10.53432971</x:v>
       </x:c>
-      <x:c r="G15" s="22" t="n">
+      <x:c r="G15" s="30" t="n">
         <x:v>13559.8</x:v>
       </x:c>
-      <x:c r="H15" s="22" t="n">
+      <x:c r="H15" s="30" t="n">
         <x:v>11223855</x:v>
       </x:c>
-      <x:c r="I15" s="22" t="n">
+      <x:c r="I15" s="30" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="J15" s="22" t="n">
+      <x:c r="J15" s="30" t="n">
         <x:v>1065455.0701356395</x:v>
       </x:c>
-      <x:c r="K15" s="23" t="n">
+      <x:c r="K15" s="31" t="n">
         <x:v>212.5403868468818</x:v>
       </x:c>
-      <x:c r="L15" s="23" t="n">
+      <x:c r="L15" s="31" t="n">
+        <x:v>25.294172357627367</x:v>
+      </x:c>
+      <x:c r="M15" s="31" t="n">
         <x:v>0.670123545698909</x:v>
       </x:c>
-      <x:c r="M15" s="23" t="n">
-        <x:v>0.16272470216235035</x:v>
-      </x:c>
-      <x:c r="N15" s="23" t="n">
+      <x:c r="N15" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O15" s="31" t="n">
         <x:v>0.8328482478612571</x:v>
       </x:c>
-      <x:c r="O15" s="24" t="n">
-        <x:v>537352922816640.06</x:v>
-      </x:c>
-      <x:c r="P15" s="24" t="n">
-        <x:v>32080771.511441197</x:v>
-      </x:c>
-      <x:c r="Q15" s="24" t="n">
+      <x:c r="P15" s="19" t="n">
+        <x:v>63949716325635.53</x:v>
+      </x:c>
+      <x:c r="Q15" s="19" t="n">
+        <x:v>3817893.5119782407</x:v>
+      </x:c>
+      <x:c r="R15" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R15" s="17" t="n">
-        <x:v>0.37433805730969893</x:v>
-      </x:c>
-      <x:c r="S15" s="16" t="str">
+      <x:c r="S15" s="18" t="n">
+        <x:v>0.04454951589239487</x:v>
+      </x:c>
+      <x:c r="T15" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T15" s="16" t="n">
+      <x:c r="U15" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U15" s="16" t="str">
+      <x:c r="V15" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V15" s="16" t="str">
+      <x:c r="W15" s="16" t="str">
         <x:v>observed_quarter_end: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1744,64 +1864,67 @@
       <x:c r="B16" s="16" t="str">
         <x:v>2026-Q3</x:v>
       </x:c>
-      <x:c r="C16" s="18" t="str">
+      <x:c r="C16" s="22" t="str">
         <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
         <x:v>observed_qtd</x:v>
       </x:c>
-      <x:c r="E16" s="22" t="n">
+      <x:c r="E16" s="30" t="n">
         <x:v>11879.32971</x:v>
       </x:c>
-      <x:c r="F16" s="22" t="n">
+      <x:c r="F16" s="30" t="n">
         <x:v>11.87932971</x:v>
       </x:c>
-      <x:c r="G16" s="22" t="n">
+      <x:c r="G16" s="30" t="n">
         <x:v>15229.8</x:v>
       </x:c>
-      <x:c r="H16" s="22" t="n">
+      <x:c r="H16" s="30" t="n">
         <x:v>13524006</x:v>
       </x:c>
-      <x:c r="I16" s="22" t="n">
+      <x:c r="I16" s="30" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="J16" s="22" t="n">
+      <x:c r="J16" s="30" t="n">
         <x:v>1138448.5766579502</x:v>
       </x:c>
-      <x:c r="K16" s="23" t="n">
+      <x:c r="K16" s="31" t="n">
         <x:v>227.10136510717322</x:v>
       </x:c>
-      <x:c r="L16" s="23" t="n">
+      <x:c r="L16" s="31" t="n">
+        <x:v>45.688453485748845</x:v>
+      </x:c>
+      <x:c r="M16" s="31" t="n">
         <x:v>0.1733549148332778</x:v>
       </x:c>
-      <x:c r="M16" s="23" t="n">
-        <x:v>0.0955993704304916</x:v>
-      </x:c>
-      <x:c r="N16" s="23" t="n">
+      <x:c r="N16" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O16" s="31" t="n">
         <x:v>0.26895428526377074</x:v>
       </x:c>
-      <x:c r="O16" s="24" t="n">
-        <x:v>647474878487808</x:v>
-      </x:c>
-      <x:c r="P16" s="24" t="n">
-        <x:v>38655216.62613779</x:v>
-      </x:c>
-      <x:c r="Q16" s="24" t="n">
+      <x:c r="P16" s="19" t="n">
+        <x:v>130259568695330.25</x:v>
+      </x:c>
+      <x:c r="Q16" s="19" t="n">
+        <x:v>7776690.668377926</x:v>
+      </x:c>
+      <x:c r="R16" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R16" s="17" t="n">
-        <x:v>0.45105270275540016</x:v>
-      </x:c>
-      <x:c r="S16" s="16" t="str">
+      <x:c r="S16" s="18" t="n">
+        <x:v>0.09074318166135269</x:v>
+      </x:c>
+      <x:c r="T16" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T16" s="16" t="n">
+      <x:c r="U16" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U16" s="16" t="str">
+      <x:c r="V16" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V16" s="16" t="str">
+      <x:c r="W16" s="16" t="str">
         <x:v>observed_qtd: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1812,64 +1935,67 @@
       <x:c r="B17" s="16" t="str">
         <x:v>2026-Q4</x:v>
       </x:c>
-      <x:c r="C17" s="18" t="str">
+      <x:c r="C17" s="22" t="str">
         <x:v>2026-12-31</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E17" s="22" t="n">
+      <x:c r="E17" s="30" t="n">
         <x:v>14026.32971</x:v>
       </x:c>
-      <x:c r="F17" s="22" t="n">
+      <x:c r="F17" s="30" t="n">
         <x:v>14.02632971</x:v>
       </x:c>
-      <x:c r="G17" s="22" t="n">
+      <x:c r="G17" s="30" t="n">
         <x:v>18051.3</x:v>
       </x:c>
-      <x:c r="H17" s="22" t="n">
+      <x:c r="H17" s="30" t="n">
         <x:v>17399770</x:v>
       </x:c>
-      <x:c r="I17" s="22" t="n">
+      <x:c r="I17" s="30" t="n">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="J17" s="22" t="n">
+      <x:c r="J17" s="30" t="n">
         <x:v>1240507.6994300885</x:v>
       </x:c>
-      <x:c r="K17" s="23" t="n">
+      <x:c r="K17" s="31" t="n">
         <x:v>247.46044550695223</x:v>
       </x:c>
-      <x:c r="L17" s="23" t="n">
+      <x:c r="L17" s="31" t="n">
+        <x:v>82.52631287577897</x:v>
+      </x:c>
+      <x:c r="M17" s="31" t="n">
         <x:v>0.23968411173075843</x:v>
       </x:c>
-      <x:c r="M17" s="23" t="n">
-        <x:v>0.12386156270665083</x:v>
-      </x:c>
-      <x:c r="N17" s="23" t="n">
+      <x:c r="N17" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O17" s="31" t="n">
         <x:v>0.36354567443740393</x:v>
       </x:c>
-      <x:c r="O17" s="24" t="n">
-        <x:v>833030831727360</x:v>
-      </x:c>
-      <x:c r="P17" s="24" t="n">
-        <x:v>49733183.983722985</x:v>
-      </x:c>
-      <x:c r="Q17" s="24" t="n">
+      <x:c r="P17" s="19" t="n">
+        <x:v>277809905795110.62</x:v>
+      </x:c>
+      <x:c r="Q17" s="19" t="n">
+        <x:v>16585666.017618544</x:v>
+      </x:c>
+      <x:c r="R17" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R17" s="17" t="n">
-        <x:v>0.5803171993433254</x:v>
-      </x:c>
-      <x:c r="S17" s="16" t="str">
+      <x:c r="S17" s="18" t="n">
+        <x:v>0.19353169215424207</x:v>
+      </x:c>
+      <x:c r="T17" s="16" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="T17" s="16" t="n">
+      <x:c r="U17" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="U17" s="16" t="str">
+      <x:c r="V17" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V17" s="16" t="str">
+      <x:c r="W17" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1880,64 +2006,67 @@
       <x:c r="B18" s="16" t="str">
         <x:v>2027-Q1</x:v>
       </x:c>
-      <x:c r="C18" s="18" t="str">
+      <x:c r="C18" s="22" t="str">
         <x:v>2027-03-31</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E18" s="22" t="n">
+      <x:c r="E18" s="30" t="n">
         <x:v>16045.32971</x:v>
       </x:c>
-      <x:c r="F18" s="22" t="n">
+      <x:c r="F18" s="30" t="n">
         <x:v>16.04532971</x:v>
       </x:c>
-      <x:c r="G18" s="22" t="n">
+      <x:c r="G18" s="30" t="n">
         <x:v>20792.8</x:v>
       </x:c>
-      <x:c r="H18" s="22" t="n">
+      <x:c r="H18" s="30" t="n">
         <x:v>20368064</x:v>
       </x:c>
-      <x:c r="I18" s="22" t="n">
+      <x:c r="I18" s="30" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="J18" s="22" t="n">
+      <x:c r="J18" s="30" t="n">
         <x:v>1269407.6325091608</x:v>
       </x:c>
-      <x:c r="K18" s="23" t="n">
+      <x:c r="K18" s="31" t="n">
         <x:v>253.22549663735143</x:v>
       </x:c>
-      <x:c r="L18" s="23" t="n">
+      <x:c r="L18" s="31" t="n">
+        <x:v>149.06594111344396</x:v>
+      </x:c>
+      <x:c r="M18" s="31" t="n">
         <x:v>0.1940158891305166</x:v>
       </x:c>
-      <x:c r="M18" s="23" t="n">
-        <x:v>0.0332247325861772</x:v>
-      </x:c>
-      <x:c r="N18" s="23" t="n">
+      <x:c r="N18" s="31" t="n">
+        <x:v>0.8530245754425181</x:v>
+      </x:c>
+      <x:c r="O18" s="31" t="n">
         <x:v>0.227240621716696</x:v>
       </x:c>
-      <x:c r="O18" s="24" t="n">
-        <x:v>975140780285952.1</x:v>
-      </x:c>
-      <x:c r="P18" s="24" t="n">
-        <x:v>58217360.01707177</x:v>
-      </x:c>
-      <x:c r="Q18" s="24" t="n">
+      <x:c r="P18" s="19" t="n">
+        <x:v>574034921687196.8</x:v>
+      </x:c>
+      <x:c r="Q18" s="19" t="n">
+        <x:v>34270741.59326548</x:v>
+      </x:c>
+      <x:c r="R18" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R18" s="17" t="n">
-        <x:v>0.6793157528246414</x:v>
-      </x:c>
-      <x:c r="S18" s="16" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="T18" s="16" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U18" s="16" t="str">
+      <x:c r="S18" s="18" t="n">
+        <x:v>0.3998919672493055</x:v>
+      </x:c>
+      <x:c r="T18" s="16" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="U18" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V18" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V18" s="16" t="str">
+      <x:c r="W18" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -1948,64 +2077,67 @@
       <x:c r="B19" s="16" t="str">
         <x:v>2027-Q2</x:v>
       </x:c>
-      <x:c r="C19" s="18" t="str">
+      <x:c r="C19" s="22" t="str">
         <x:v>2027-06-30</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E19" s="22" t="n">
+      <x:c r="E19" s="30" t="n">
         <x:v>16634.32971</x:v>
       </x:c>
-      <x:c r="F19" s="22" t="n">
+      <x:c r="F19" s="30" t="n">
         <x:v>16.634329710000003</x:v>
       </x:c>
-      <x:c r="G19" s="22" t="n">
+      <x:c r="G19" s="30" t="n">
         <x:v>21589.8</x:v>
       </x:c>
-      <x:c r="H19" s="22" t="n">
+      <x:c r="H19" s="30" t="n">
         <x:v>21439292</x:v>
       </x:c>
-      <x:c r="I19" s="22" t="n">
+      <x:c r="I19" s="30" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="J19" s="22" t="n">
+      <x:c r="J19" s="30" t="n">
         <x:v>1288858.1850768183</x:v>
       </x:c>
-      <x:c r="K19" s="23" t="n">
+      <x:c r="K19" s="31" t="n">
         <x:v>257.10555510531594</x:v>
       </x:c>
-      <x:c r="L19" s="23" t="n">
+      <x:c r="L19" s="31" t="n">
+        <x:v>269.25539292521074</x:v>
+      </x:c>
+      <x:c r="M19" s="31" t="n">
         <x:v>0.052010297783469106</x:v>
       </x:c>
-      <x:c r="M19" s="23" t="n">
-        <x:v>0.021938108432294712</x:v>
-      </x:c>
-      <x:c r="N19" s="23" t="n">
+      <x:c r="N19" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O19" s="31" t="n">
         <x:v>0.07394840621576648</x:v>
       </x:c>
-      <x:c r="O19" s="24" t="n">
-        <x:v>1026426857734656.1</x:v>
-      </x:c>
-      <x:c r="P19" s="24" t="n">
-        <x:v>61279215.38714365</x:v>
-      </x:c>
-      <x:c r="Q19" s="24" t="n">
+      <x:c r="P19" s="19" t="n">
+        <x:v>1074931915707253.8</x:v>
+      </x:c>
+      <x:c r="Q19" s="19" t="n">
+        <x:v>64175039.74371664</x:v>
+      </x:c>
+      <x:c r="R19" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R19" s="17" t="n">
-        <x:v>0.7150433534089107</x:v>
-      </x:c>
-      <x:c r="S19" s="16" t="str">
+      <x:c r="S19" s="18" t="n">
+        <x:v>0.7488336026104626</x:v>
+      </x:c>
+      <x:c r="T19" s="16" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="T19" s="16" t="n">
+      <x:c r="U19" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="U19" s="16" t="str">
+      <x:c r="V19" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V19" s="16" t="str">
+      <x:c r="W19" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2016,64 +2148,67 @@
       <x:c r="B20" s="16" t="str">
         <x:v>2027-Q3</x:v>
       </x:c>
-      <x:c r="C20" s="18" t="str">
+      <x:c r="C20" s="22" t="str">
         <x:v>2027-09-30</x:v>
       </x:c>
       <x:c r="D20" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E20" s="22" t="n">
+      <x:c r="E20" s="30" t="n">
         <x:v>17451.32971</x:v>
       </x:c>
-      <x:c r="F20" s="22" t="n">
+      <x:c r="F20" s="30" t="n">
         <x:v>17.451329710000003</x:v>
       </x:c>
-      <x:c r="G20" s="22" t="n">
+      <x:c r="G20" s="30" t="n">
         <x:v>22700.2</x:v>
       </x:c>
-      <x:c r="H20" s="22" t="n">
+      <x:c r="H20" s="30" t="n">
         <x:v>23242366</x:v>
       </x:c>
-      <x:c r="I20" s="22" t="n">
+      <x:c r="I20" s="30" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="J20" s="22" t="n">
+      <x:c r="J20" s="30" t="n">
         <x:v>1331839.257307803</x:v>
       </x:c>
-      <x:c r="K20" s="23" t="n">
+      <x:c r="K20" s="31" t="n">
         <x:v>265.67955693338394</x:v>
       </x:c>
-      <x:c r="L20" s="23" t="n">
+      <x:c r="L20" s="31" t="n">
+        <x:v>486.3516513415762</x:v>
+      </x:c>
+      <x:c r="M20" s="31" t="n">
         <x:v>0.06917323410675813</x:v>
       </x:c>
-      <x:c r="M20" s="23" t="n">
-        <x:v>0.0473264401703517</x:v>
-      </x:c>
-      <x:c r="N20" s="23" t="n">
+      <x:c r="N20" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O20" s="31" t="n">
         <x:v>0.11649967427711161</x:v>
       </x:c>
-      <x:c r="O20" s="24" t="n">
-        <x:v>1112750770860288</x:v>
-      </x:c>
-      <x:c r="P20" s="24" t="n">
-        <x:v>66432881.84240525</x:v>
-      </x:c>
-      <x:c r="Q20" s="24" t="n">
+      <x:c r="P20" s="19" t="n">
+        <x:v>2036995925415554.5</x:v>
+      </x:c>
+      <x:c r="Q20" s="19" t="n">
+        <x:v>121611697.0397346</x:v>
+      </x:c>
+      <x:c r="R20" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R20" s="17" t="n">
-        <x:v>0.775179484742185</x:v>
-      </x:c>
-      <x:c r="S20" s="16" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="T20" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U20" s="16" t="str">
+      <x:c r="S20" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T20" s="16" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="U20" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="V20" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V20" s="16" t="str">
+      <x:c r="W20" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2084,64 +2219,67 @@
       <x:c r="B21" s="16" t="str">
         <x:v>2027-Q4</x:v>
       </x:c>
-      <x:c r="C21" s="18" t="str">
+      <x:c r="C21" s="22" t="str">
         <x:v>2027-12-31</x:v>
       </x:c>
       <x:c r="D21" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E21" s="22" t="n">
+      <x:c r="E21" s="30" t="n">
         <x:v>19777.32971</x:v>
       </x:c>
-      <x:c r="F21" s="22" t="n">
+      <x:c r="F21" s="30" t="n">
         <x:v>19.77732971</x:v>
       </x:c>
-      <x:c r="G21" s="22" t="n">
+      <x:c r="G21" s="30" t="n">
         <x:v>25804.3</x:v>
       </x:c>
-      <x:c r="H21" s="22" t="n">
+      <x:c r="H21" s="30" t="n">
         <x:v>30057691</x:v>
       </x:c>
-      <x:c r="I21" s="22" t="n">
+      <x:c r="I21" s="30" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="J21" s="22" t="n">
+      <x:c r="J21" s="30" t="n">
         <x:v>1519805.3246188208</x:v>
       </x:c>
-      <x:c r="K21" s="23" t="n">
+      <x:c r="K21" s="31" t="n">
         <x:v>303.17562953200115</x:v>
       </x:c>
-      <x:c r="L21" s="23" t="n">
+      <x:c r="L21" s="31" t="n">
+        <x:v>878.489103571566</x:v>
+      </x:c>
+      <x:c r="M21" s="31" t="n">
         <x:v>0.18051068258604275</x:v>
       </x:c>
-      <x:c r="M21" s="23" t="n">
-        <x:v>0.19046656656848882</x:v>
-      </x:c>
-      <x:c r="N21" s="23" t="n">
+      <x:c r="N21" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O21" s="31" t="n">
         <x:v>0.37097724915453156</x:v>
       </x:c>
-      <x:c r="O21" s="24" t="n">
-        <x:v>1439041052469887.8</x:v>
-      </x:c>
-      <x:c r="P21" s="24" t="n">
-        <x:v>85912898.65491867</x:v>
-      </x:c>
-      <x:c r="Q21" s="24" t="n">
+      <x:c r="P21" s="19" t="n">
+        <x:v>4169800475514528</x:v>
+      </x:c>
+      <x:c r="Q21" s="19" t="n">
+        <x:v>248943311.9710166</x:v>
+      </x:c>
+      <x:c r="R21" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R21" s="17" t="n">
+      <x:c r="S21" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S21" s="16" t="str">
+      <x:c r="T21" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="T21" s="16" t="n">
+      <x:c r="U21" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="U21" s="16" t="str">
+      <x:c r="V21" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V21" s="16" t="str">
+      <x:c r="W21" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2152,64 +2290,67 @@
       <x:c r="B22" s="16" t="str">
         <x:v>2028-Q1</x:v>
       </x:c>
-      <x:c r="C22" s="18" t="str">
+      <x:c r="C22" s="22" t="str">
         <x:v>2028-03-31</x:v>
       </x:c>
       <x:c r="D22" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E22" s="22" t="n">
+      <x:c r="E22" s="30" t="n">
         <x:v>23626.32971</x:v>
       </x:c>
-      <x:c r="F22" s="22" t="n">
+      <x:c r="F22" s="30" t="n">
         <x:v>23.62632971</x:v>
       </x:c>
-      <x:c r="G22" s="22" t="n">
+      <x:c r="G22" s="30" t="n">
         <x:v>30729.3</x:v>
       </x:c>
-      <x:c r="H22" s="22" t="n">
+      <x:c r="H22" s="30" t="n">
         <x:v>37048243</x:v>
       </x:c>
-      <x:c r="I22" s="22" t="n">
+      <x:c r="I22" s="30" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="J22" s="22" t="n">
+      <x:c r="J22" s="30" t="n">
         <x:v>1568091.3393974642</x:v>
       </x:c>
-      <x:c r="K22" s="23" t="n">
+      <x:c r="K22" s="31" t="n">
         <x:v>312.80787827529224</x:v>
       </x:c>
-      <x:c r="L22" s="23" t="n">
+      <x:c r="L22" s="31" t="n">
+        <x:v>1586.800626594274</x:v>
+      </x:c>
+      <x:c r="M22" s="31" t="n">
         <x:v>0.25654787787862965</x:v>
       </x:c>
-      <x:c r="M22" s="23" t="n">
-        <x:v>0.04512305976057718</x:v>
-      </x:c>
-      <x:c r="N22" s="23" t="n">
+      <x:c r="N22" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O22" s="31" t="n">
         <x:v>0.3016709376392015</x:v>
       </x:c>
-      <x:c r="O22" s="24" t="n">
-        <x:v>1773720496324224.2</x:v>
-      </x:c>
-      <x:c r="P22" s="24" t="n">
-        <x:v>105893760.97458056</x:v>
-      </x:c>
-      <x:c r="Q22" s="24" t="n">
+      <x:c r="P22" s="19" t="n">
+        <x:v>8997665949108219</x:v>
+      </x:c>
+      <x:c r="Q22" s="19" t="n">
+        <x:v>537174086.5139235</x:v>
+      </x:c>
+      <x:c r="R22" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R22" s="17" t="n">
+      <x:c r="S22" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S22" s="16" t="str">
+      <x:c r="T22" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="T22" s="16" t="n">
+      <x:c r="U22" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="U22" s="16" t="str">
+      <x:c r="V22" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V22" s="16" t="str">
+      <x:c r="W22" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2220,64 +2361,67 @@
       <x:c r="B23" s="16" t="str">
         <x:v>2028-Q2</x:v>
       </x:c>
-      <x:c r="C23" s="18" t="str">
+      <x:c r="C23" s="22" t="str">
         <x:v>2028-06-30</x:v>
       </x:c>
       <x:c r="D23" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E23" s="22" t="n">
+      <x:c r="E23" s="30" t="n">
         <x:v>26122.32971</x:v>
       </x:c>
-      <x:c r="F23" s="22" t="n">
+      <x:c r="F23" s="30" t="n">
         <x:v>26.122329710000002</x:v>
       </x:c>
-      <x:c r="G23" s="22" t="n">
+      <x:c r="G23" s="30" t="n">
         <x:v>33779.3</x:v>
       </x:c>
-      <x:c r="H23" s="22" t="n">
+      <x:c r="H23" s="30" t="n">
         <x:v>46037632</x:v>
       </x:c>
-      <x:c r="I23" s="22" t="n">
+      <x:c r="I23" s="30" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="J23" s="22" t="n">
+      <x:c r="J23" s="30" t="n">
         <x:v>1762386.1466833923</x:v>
       </x:c>
-      <x:c r="K23" s="23" t="n">
+      <x:c r="K23" s="31" t="n">
         <x:v>351.5664281760725</x:v>
       </x:c>
-      <x:c r="L23" s="23" t="n">
+      <x:c r="L23" s="31" t="n">
+        <x:v>2866.2122481919423</x:v>
+      </x:c>
+      <x:c r="M23" s="31" t="n">
         <x:v>0.1448880411016562</x:v>
       </x:c>
-      <x:c r="M23" s="23" t="n">
-        <x:v>0.16852046270835075</x:v>
-      </x:c>
-      <x:c r="N23" s="23" t="n">
+      <x:c r="N23" s="31" t="n">
+        <x:v>0.8530245754425181</x:v>
+      </x:c>
+      <x:c r="O23" s="31" t="n">
         <x:v>0.3134085038100096</x:v>
       </x:c>
-      <x:c r="O23" s="24" t="n">
-        <x:v>2204096196427776</x:v>
-      </x:c>
-      <x:c r="P23" s="24" t="n">
-        <x:v>131587832.6225538</x:v>
-      </x:c>
-      <x:c r="Q23" s="24" t="n">
+      <x:c r="P23" s="19" t="n">
+        <x:v>17969313927866468</x:v>
+      </x:c>
+      <x:c r="Q23" s="19" t="n">
+        <x:v>1072794861.3651623</x:v>
+      </x:c>
+      <x:c r="R23" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R23" s="17" t="n">
+      <x:c r="S23" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S23" s="16" t="str">
+      <x:c r="T23" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="T23" s="16" t="n">
+      <x:c r="U23" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="U23" s="16" t="str">
+      <x:c r="V23" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V23" s="16" t="str">
+      <x:c r="W23" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2288,64 +2432,67 @@
       <x:c r="B24" s="16" t="str">
         <x:v>2028-Q3</x:v>
       </x:c>
-      <x:c r="C24" s="18" t="str">
+      <x:c r="C24" s="22" t="str">
         <x:v>2028-09-30</x:v>
       </x:c>
       <x:c r="D24" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E24" s="22" t="n">
+      <x:c r="E24" s="30" t="n">
         <x:v>26757.32971</x:v>
       </x:c>
-      <x:c r="F24" s="22" t="n">
+      <x:c r="F24" s="30" t="n">
         <x:v>26.75732971</x:v>
       </x:c>
-      <x:c r="G24" s="22" t="n">
+      <x:c r="G24" s="30" t="n">
         <x:v>34541.3</x:v>
       </x:c>
-      <x:c r="H24" s="22" t="n">
+      <x:c r="H24" s="30" t="n">
         <x:v>47106859</x:v>
       </x:c>
-      <x:c r="I24" s="22" t="n">
+      <x:c r="I24" s="30" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="J24" s="22" t="n">
+      <x:c r="J24" s="30" t="n">
         <x:v>1760521.6780056637</x:v>
       </x:c>
-      <x:c r="K24" s="23" t="n">
+      <x:c r="K24" s="31" t="n">
         <x:v>351.19449799793944</x:v>
       </x:c>
-      <x:c r="L24" s="23" t="n">
+      <x:c r="L24" s="31" t="n">
+        <x:v>5177.192719741742</x:v>
+      </x:c>
+      <x:c r="M24" s="31" t="n">
         <x:v>0.034650578303203616</x:v>
       </x:c>
-      <x:c r="M24" s="23" t="n">
-        <x:v>-0.0015270680359833477</x:v>
-      </x:c>
-      <x:c r="N24" s="23" t="n">
+      <x:c r="N24" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O24" s="31" t="n">
         <x:v>0.03312351026722382</x:v>
       </x:c>
-      <x:c r="O24" s="24" t="n">
-        <x:v>2255286474064512</x:v>
-      </x:c>
-      <x:c r="P24" s="24" t="n">
-        <x:v>134643968.60086638</x:v>
-      </x:c>
-      <x:c r="Q24" s="24" t="n">
+      <x:c r="P24" s="19" t="n">
+        <x:v>33246684617841944</x:v>
+      </x:c>
+      <x:c r="Q24" s="19" t="n">
+        <x:v>1984876693.602504</x:v>
+      </x:c>
+      <x:c r="R24" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R24" s="17" t="n">
+      <x:c r="S24" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S24" s="16" t="str">
+      <x:c r="T24" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="T24" s="16" t="n">
+      <x:c r="U24" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="U24" s="16" t="str">
+      <x:c r="V24" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V24" s="16" t="str">
+      <x:c r="W24" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
@@ -2356,76 +2503,79 @@
       <x:c r="B25" s="16" t="str">
         <x:v>2028-Q4</x:v>
       </x:c>
-      <x:c r="C25" s="18" t="str">
+      <x:c r="C25" s="22" t="str">
         <x:v>2028-12-31</x:v>
       </x:c>
       <x:c r="D25" s="16" t="str">
         <x:v>projected</x:v>
       </x:c>
-      <x:c r="E25" s="22" t="n">
+      <x:c r="E25" s="30" t="n">
         <x:v>31674.32971</x:v>
       </x:c>
-      <x:c r="F25" s="22" t="n">
+      <x:c r="F25" s="30" t="n">
         <x:v>31.674329710000002</x:v>
       </x:c>
-      <x:c r="G25" s="22" t="n">
+      <x:c r="G25" s="30" t="n">
         <x:v>41462.3</x:v>
       </x:c>
-      <x:c r="H25" s="22" t="n">
+      <x:c r="H25" s="30" t="n">
         <x:v>61887051</x:v>
       </x:c>
-      <x:c r="I25" s="22" t="n">
+      <x:c r="I25" s="30" t="n">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="J25" s="22" t="n">
+      <x:c r="J25" s="30" t="n">
         <x:v>1953855.111272061</x:v>
       </x:c>
-      <x:c r="K25" s="23" t="n">
+      <x:c r="K25" s="31" t="n">
         <x:v>389.7612699329068</x:v>
       </x:c>
-      <x:c r="L25" s="23" t="n">
+      <x:c r="L25" s="31" t="n">
+        <x:v>9351.47928219723</x:v>
+      </x:c>
+      <x:c r="M25" s="31" t="n">
         <x:v>0.2433799423435694</x:v>
       </x:c>
-      <x:c r="M25" s="23" t="n">
-        <x:v>0.15032049598749353</x:v>
-      </x:c>
-      <x:c r="N25" s="23" t="n">
+      <x:c r="N25" s="31" t="n">
+        <x:v>0.853024575442511</x:v>
+      </x:c>
+      <x:c r="O25" s="31" t="n">
         <x:v>0.39370043833106294</x:v>
       </x:c>
-      <x:c r="O25" s="24" t="n">
-        <x:v>2962902473290368</x:v>
-      </x:c>
-      <x:c r="P25" s="24" t="n">
-        <x:v>176889699.8979324</x:v>
-      </x:c>
-      <x:c r="Q25" s="24" t="n">
+      <x:c r="P25" s="19" t="n">
+        <x:v>71088441134531810</x:v>
+      </x:c>
+      <x:c r="Q25" s="19" t="n">
+        <x:v>4244086037.882496</x:v>
+      </x:c>
+      <x:c r="R25" s="19" t="n">
         <x:v>85700000</x:v>
       </x:c>
-      <x:c r="R25" s="17" t="n">
+      <x:c r="S25" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S25" s="16" t="str">
+      <x:c r="T25" s="16" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="T25" s="16" t="n">
+      <x:c r="U25" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="U25" s="16" t="str">
+      <x:c r="V25" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
       </x:c>
-      <x:c r="V25" s="16" t="str">
+      <x:c r="W25" s="16" t="str">
         <x:v>epoch_projected_pipeline: Latest published state on or before cutoff for each Epoch-covered U.S. site. U.S. sites are selected through Epoch's data-center registry; IT power is the physical source metric and H100e is retained as a productivity audit bridge.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:V2"/>
-    <x:mergeCell ref="A3:V3"/>
+    <x:mergeCell ref="A1:W2"/>
+    <x:mergeCell ref="A3:W3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2de7559930ca47a6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e6cf5e1565b4a4d"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec980a7eaccd4377"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f0a82152cfd496b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2484,7 +2634,7 @@
       <x:c r="B6" s="16" t="str">
         <x:v>U.S. residents</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="n">
+      <x:c r="C6" s="19" t="n">
         <x:v>342800000</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
@@ -2498,7 +2648,7 @@
       <x:c r="B7" s="16" t="str">
         <x:v>Selected target</x:v>
       </x:c>
-      <x:c r="C7" s="25" t="n">
+      <x:c r="C7" s="20" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
@@ -2512,192 +2662,150 @@
       <x:c r="B8" s="16" t="str">
         <x:v>Supply gate share of selected target</x:v>
       </x:c>
-      <x:c r="C8" s="25" t="n">
+      <x:c r="C8" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>100% in the default</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
         <x:v>Serving</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Dense 8-bit ops / H100e-second</x:v>
-      </x:c>
-      <x:c r="C9" s="16" t="n">
-        <x:v>1979000000000000</x:v>
+        <x:v>Seconds per day</x:v>
+      </x:c>
+      <x:c r="C9" s="19" t="n">
+        <x:v>86400</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
-        <x:v>ops/s</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
+        <x:v>seconds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
         <x:v>Serving</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Seconds per day</x:v>
-      </x:c>
-      <x:c r="C10" s="16" t="n">
-        <x:v>86400</x:v>
+        <x:v>Fleet share allocated to inference</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="n">
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
-        <x:v>seconds</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="32.400001525878906" hidden="0" customHeight="1">
+        <x:v>share</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="str">
         <x:v>Serving</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Fleet share allocated to inference</x:v>
-      </x:c>
-      <x:c r="C11" s="25" t="n">
-        <x:v>0.4</x:v>
+        <x:v>Reference active model parameters</x:v>
+      </x:c>
+      <x:c r="C11" s="19" t="n">
+        <x:v>100000000000</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
-        <x:v>share</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
+        <x:v>parameters used to normalize measured tokens</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A12" s="16" t="str">
         <x:v>Serving</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
+        <x:v>Personal-AI inference share</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>scenario allocation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>Audit only</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>Dense 8-bit ops / H100e-second</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="n">
+        <x:v>1979000000000000</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>excluded from capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A14" s="16" t="str">
+        <x:v>Audit only</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="str">
         <x:v>Sustained utilization</x:v>
       </x:c>
-      <x:c r="C12" s="25" t="n">
+      <x:c r="C14" s="20" t="n">
         <x:v>0.35</x:v>
       </x:c>
-      <x:c r="D12" s="16" t="str">
-        <x:v>share of peak</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A13" s="16" t="str">
-        <x:v>Serving</x:v>
-      </x:c>
-      <x:c r="B13" s="16" t="str">
-        <x:v>Active model parameters</x:v>
-      </x:c>
-      <x:c r="C13" s="16" t="n">
-        <x:v>100000000000</x:v>
-      </x:c>
-      <x:c r="D13" s="16" t="str">
-        <x:v>parameters</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A14" s="16" t="str">
-        <x:v>Serving</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="str">
-        <x:v>Forward-pass ops / parameter-token</x:v>
-      </x:c>
-      <x:c r="C14" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="D14" s="16" t="str">
-        <x:v>ops</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
+        <x:v>excluded from capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64.80000305175781" hidden="0" customHeight="1">
       <x:c r="A15" s="16" t="str">
-        <x:v>Serving</x:v>
+        <x:v>Workload</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>System overhead</x:v>
-      </x:c>
-      <x:c r="C15" s="16" t="n">
-        <x:v>1.5</x:v>
+        <x:v>Uncached input</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="n">
+        <x:v>2000000</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
-        <x:v>multiplier</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="21.600000381469727" hidden="0" customHeight="1">
+        <x:v>1× compute weight = 2,000,000 compute-equivalent tokens</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="75.5999984741211" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="str">
-        <x:v>Serving</x:v>
+        <x:v>Workload</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Serving goodput</x:v>
-      </x:c>
-      <x:c r="C16" s="16" t="n">
-        <x:v>1</x:v>
+        <x:v>Visible output</x:v>
+      </x:c>
+      <x:c r="C16" s="19" t="n">
+        <x:v>300000</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
-        <x:v>multiplier</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
+        <x:v>2.5× compute weight = 750,000 compute-equivalent tokens</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="75.5999984741211" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:v>Serving</x:v>
+        <x:v>Workload</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
-        <x:v>Personal-AI inference share</x:v>
-      </x:c>
-      <x:c r="C17" s="25" t="n">
-        <x:v>0.6</x:v>
+        <x:v>Internal reasoning</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="n">
+        <x:v>5000000</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
-        <x:v>scenario allocation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="64.80000305175781" hidden="0" customHeight="1">
+        <x:v>2.5× compute weight = 12,500,000 compute-equivalent tokens</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="75.5999984741211" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="str">
         <x:v>Workload</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
-        <x:v>Uncached input</x:v>
-      </x:c>
-      <x:c r="C18" s="16" t="n">
-        <x:v>2000000</x:v>
+        <x:v>Cached/reused context</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="n">
+        <x:v>10000000</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
-        <x:v>1× compute weight = 2,000,000 compute-equivalent tokens</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A19" s="16" t="str">
-        <x:v>Workload</x:v>
-      </x:c>
-      <x:c r="B19" s="16" t="str">
-        <x:v>Visible output</x:v>
-      </x:c>
-      <x:c r="C19" s="16" t="n">
-        <x:v>300000</x:v>
-      </x:c>
-      <x:c r="D19" s="16" t="str">
-        <x:v>2.5× compute weight = 750,000 compute-equivalent tokens</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A20" s="16" t="str">
-        <x:v>Workload</x:v>
-      </x:c>
-      <x:c r="B20" s="16" t="str">
-        <x:v>Internal reasoning</x:v>
-      </x:c>
-      <x:c r="C20" s="16" t="n">
-        <x:v>5000000</x:v>
-      </x:c>
-      <x:c r="D20" s="16" t="str">
-        <x:v>2.5× compute weight = 12,500,000 compute-equivalent tokens</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A21" s="16" t="str">
-        <x:v>Workload</x:v>
-      </x:c>
-      <x:c r="B21" s="16" t="str">
-        <x:v>Cached/reused context</x:v>
-      </x:c>
-      <x:c r="C21" s="16" t="n">
-        <x:v>10000000</x:v>
-      </x:c>
-      <x:c r="D21" s="16" t="str">
         <x:v>0.15× compute weight = 1,500,000 compute-equivalent tokens</x:v>
       </x:c>
     </x:row>
@@ -2708,12 +2816,353 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27de98fdc1d446ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8626d6fceb2444bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="14" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="36" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="70" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Measured Inference Goodput per Watt</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+      <x:c r="H1" s="3"/>
+      <x:c r="I1" s="3"/>
+      <x:c r="J1" s="3"/>
+      <x:c r="K1" s="3"/>
+      <x:c r="L1" s="3"/>
+      <x:c r="M1" s="3"/>
+      <x:c r="N1" s="3"/>
+      <x:c r="O1" s="3"/>
+      <x:c r="P1" s="3"/>
+      <x:c r="Q1" s="3"/>
+      <x:c r="R1" s="3"/>
+      <x:c r="S1" s="3"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="3"/>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+      <x:c r="H2" s="3"/>
+      <x:c r="I2" s="3"/>
+      <x:c r="J2" s="3"/>
+      <x:c r="K2" s="3"/>
+      <x:c r="L2" s="3"/>
+      <x:c r="M2" s="3"/>
+      <x:c r="N2" s="3"/>
+      <x:c r="O2" s="3"/>
+      <x:c r="P2" s="3"/>
+      <x:c r="Q2" s="3"/>
+      <x:c r="R2" s="3"/>
+      <x:c r="S2" s="3"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>MLPerf Server power results used for the independent absolute baseline and matched productivity velocity. H100e is not an input to this sheet.</x:v>
+      </x:c>
+      <x:c r="B3" s="6"/>
+      <x:c r="C3" s="6"/>
+      <x:c r="D3" s="6"/>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="6"/>
+      <x:c r="G3" s="6"/>
+      <x:c r="H3" s="6"/>
+      <x:c r="I3" s="6"/>
+      <x:c r="J3" s="6"/>
+      <x:c r="K3" s="6"/>
+      <x:c r="L3" s="6"/>
+      <x:c r="M3" s="6"/>
+      <x:c r="N3" s="6"/>
+      <x:c r="O3" s="6"/>
+      <x:c r="P3" s="6"/>
+      <x:c r="Q3" s="6"/>
+      <x:c r="R3" s="6"/>
+      <x:c r="S3" s="6"/>
+    </x:row>
+    <x:row r="4"/>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Observation ID</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Model</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Submitter</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Accelerator</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Active parameters</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="str">
+        <x:v>Measured tokens/s</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="str">
+        <x:v>Measured system W</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>Tokens/J</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>Reference productivity T/GW-day</x:v>
+      </x:c>
+      <x:c r="O5" s="12" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="P5" s="12" t="str">
+        <x:v>Raw result ID</x:v>
+      </x:c>
+      <x:c r="Q5" s="12" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+      <x:c r="R5" s="12" t="str">
+        <x:v>Source location</x:v>
+      </x:c>
+      <x:c r="S5" s="12" t="str">
+        <x:v>Comparability note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="205.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>mlperf-v5-0-llama2-70b-99-9-server-h100</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>MLPerf Inference v5.0</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>2025-04-02</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>llama2-70b-99.9</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>Server</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>Fujitsu</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>PRIMERGY CDI (8x H100-NVL-94GB, TensorRT)</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
+        <x:v>NVIDIA H100-NVL-94GB</x:v>
+      </x:c>
+      <x:c r="I6" s="16" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J6" s="17" t="n">
+        <x:v>70000000000</x:v>
+      </x:c>
+      <x:c r="K6" s="17" t="n">
+        <x:v>16848.6</x:v>
+      </x:c>
+      <x:c r="L6" s="17" t="n">
+        <x:v>4994.2610980392</x:v>
+      </x:c>
+      <x:c r="M6" s="17" t="n">
+        <x:v>3.37359214291278</x:v>
+      </x:c>
+      <x:c r="N6" s="17" t="n">
+        <x:v>204.03485280336494</x:v>
+      </x:c>
+      <x:c r="O6" s="16" t="str">
+        <x:v>productivity-trend-point</x:v>
+      </x:c>
+      <x:c r="P6" s="16" t="str">
+        <x:v>5.0-0023</x:v>
+      </x:c>
+      <x:c r="Q6" s="16" t="str">
+        <x:v>gate2-github-com-mlperf-inference-v5-0-power</x:v>
+      </x:c>
+      <x:c r="R6" s="16" t="str">
+        <x:v>ID 5.0-0023; llama2-70b-99.9; Server</x:v>
+      </x:c>
+      <x:c r="S6" s="16" t="str">
+        <x:v>Matched to the v5.1 Llama 2 70B 99.9 Server row. Reference-token equivalence multiplies measured tokens per joule by 70B/100B; the same factor cancels from the two-point growth rate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>mlperf-v5-1-llama2-70b-99-9-server-b200</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>MLPerf Inference v5.1</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>2025-09-09</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>llama2-70b-99.9</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>Server</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>Lenovo</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>ThinkSystem SR680a V3 (8x B200-SXM-180GB, TensorRT)</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>NVIDIA B200-SXM-180GB</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J7" s="17" t="n">
+        <x:v>70000000000</x:v>
+      </x:c>
+      <x:c r="K7" s="17" t="n">
+        <x:v>99203.9</x:v>
+      </x:c>
+      <x:c r="L7" s="17" t="n">
+        <x:v>10434.706455542</x:v>
+      </x:c>
+      <x:c r="M7" s="17" t="n">
+        <x:v>9.507109799654364</x:v>
+      </x:c>
+      <x:c r="N7" s="17" t="n">
+        <x:v>574.9900006830959</x:v>
+      </x:c>
+      <x:c r="O7" s="16" t="str">
+        <x:v>productivity-trend-point</x:v>
+      </x:c>
+      <x:c r="P7" s="16" t="str">
+        <x:v>5.1-0061</x:v>
+      </x:c>
+      <x:c r="Q7" s="16" t="str">
+        <x:v>gate2-github-com-mlperf-inference-v5-1-power</x:v>
+      </x:c>
+      <x:c r="R7" s="16" t="str">
+        <x:v>ID 5.1-0061; llama2-70b-99.9; Server</x:v>
+      </x:c>
+      <x:c r="S7" s="16" t="str">
+        <x:v>Matched to the v5.0 Llama 2 70B 99.9 Server row. The measured reference-token productivity is 2.8181× the v5.0 point over 160 days.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>mlperf-v5-1-llama31-405b-server-b200</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>MLPerf Inference v5.1</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>2025-09-09</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>llama3.1-405b</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str">
+        <x:v>Server</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>Lenovo</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>ThinkSystem SR780a V3 (8x B200-SXM-180GB, TensorRT)</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>NVIDIA B200-SXM-180GB</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J8" s="17" t="n">
+        <x:v>405000000000</x:v>
+      </x:c>
+      <x:c r="K8" s="17" t="n">
+        <x:v>1249.04</x:v>
+      </x:c>
+      <x:c r="L8" s="17" t="n">
+        <x:v>9566.1823383085</x:v>
+      </x:c>
+      <x:c r="M8" s="17" t="n">
+        <x:v>0.13056828270961604</x:v>
+      </x:c>
+      <x:c r="N8" s="17" t="n">
+        <x:v>45.688453485748845</x:v>
+      </x:c>
+      <x:c r="O8" s="16" t="str">
+        <x:v>absolute-productivity-baseline</x:v>
+      </x:c>
+      <x:c r="P8" s="16" t="str">
+        <x:v>5.1-0062</x:v>
+      </x:c>
+      <x:c r="Q8" s="16" t="str">
+        <x:v>gate2-github-com-mlperf-inference-v5-1-power</x:v>
+      </x:c>
+      <x:c r="R8" s="16" t="str">
+        <x:v>ID 5.1-0062; llama3.1-405b; Server</x:v>
+      </x:c>
+      <x:c r="S8" s="16" t="str">
+        <x:v>The gate uses this measured latency-constrained large-model result as its absolute baseline. Reference-token equivalence multiplies measured tokens per joule by 405B/100B; no H100-equivalent field enters the calculation.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:S2"/>
+    <x:mergeCell ref="A3:S3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00875049a3604f4f"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2795,10 +3244,10 @@
       <x:c r="B6" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C6" s="22" t="n">
+      <x:c r="C6" s="30" t="n">
         <x:v>1111672.5618999496</x:v>
       </x:c>
-      <x:c r="D6" s="22" t="n">
+      <x:c r="D6" s="30" t="n">
         <x:v>946</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
@@ -2821,10 +3270,10 @@
       <x:c r="B7" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C7" s="22" t="n">
+      <x:c r="C7" s="30" t="n">
         <x:v>768768.7220818596</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="n">
+      <x:c r="D7" s="30" t="n">
         <x:v>636</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
@@ -2847,10 +3296,10 @@
       <x:c r="B8" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C8" s="22" t="n">
+      <x:c r="C8" s="30" t="n">
         <x:v>763011.622031329</x:v>
       </x:c>
-      <x:c r="D8" s="22" t="n">
+      <x:c r="D8" s="30" t="n">
         <x:v>368</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
@@ -2873,10 +3322,10 @@
       <x:c r="B9" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="n">
+      <x:c r="C9" s="30" t="n">
         <x:v>685912.076806468</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="n">
+      <x:c r="D9" s="30" t="n">
         <x:v>910</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
@@ -2899,10 +3348,10 @@
       <x:c r="B10" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C10" s="22" t="n">
+      <x:c r="C10" s="30" t="n">
         <x:v>677109.6513390602</x:v>
       </x:c>
-      <x:c r="D10" s="22" t="n">
+      <x:c r="D10" s="30" t="n">
         <x:v>562</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
@@ -2925,10 +3374,10 @@
       <x:c r="B11" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C11" s="22" t="n">
+      <x:c r="C11" s="30" t="n">
         <x:v>616472.9661445174</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="n">
+      <x:c r="D11" s="30" t="n">
         <x:v>453</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
@@ -2951,10 +3400,10 @@
       <x:c r="B12" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C12" s="22" t="n">
+      <x:c r="C12" s="30" t="n">
         <x:v>509348.15563415864</x:v>
       </x:c>
-      <x:c r="D12" s="22" t="n">
+      <x:c r="D12" s="30" t="n">
         <x:v>421</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
@@ -2977,10 +3426,10 @@
       <x:c r="B13" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C13" s="22" t="n">
+      <x:c r="C13" s="30" t="n">
         <x:v>445679.63617988885</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="n">
+      <x:c r="D13" s="30" t="n">
         <x:v>369</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
@@ -3003,10 +3452,10 @@
       <x:c r="B14" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C14" s="22" t="n">
+      <x:c r="C14" s="30" t="n">
         <x:v>408792.3193532087</x:v>
       </x:c>
-      <x:c r="D14" s="22" t="n">
+      <x:c r="D14" s="30" t="n">
         <x:v>303</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
@@ -3029,10 +3478,10 @@
       <x:c r="B15" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C15" s="22" t="n">
+      <x:c r="C15" s="30" t="n">
         <x:v>343102.57705912075</x:v>
       </x:c>
-      <x:c r="D15" s="22" t="n">
+      <x:c r="D15" s="30" t="n">
         <x:v>183</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
@@ -3051,10 +3500,10 @@
       <x:c r="B16" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C16" s="22" t="n">
+      <x:c r="C16" s="30" t="n">
         <x:v>289034.86609398684</x:v>
       </x:c>
-      <x:c r="D16" s="22" t="n">
+      <x:c r="D16" s="30" t="n">
         <x:v>237</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
@@ -3077,10 +3526,10 @@
       <x:c r="B17" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C17" s="22" t="n">
+      <x:c r="C17" s="30" t="n">
         <x:v>287518.9489641233</x:v>
       </x:c>
-      <x:c r="D17" s="22" t="n">
+      <x:c r="D17" s="30" t="n">
         <x:v>141</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
@@ -3101,10 +3550,10 @@
       <x:c r="B18" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C18" s="22" t="n">
+      <x:c r="C18" s="30" t="n">
         <x:v>283675.08842849924</x:v>
       </x:c>
-      <x:c r="D18" s="22" t="n">
+      <x:c r="D18" s="30" t="n">
         <x:v>279</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
@@ -3127,10 +3576,10 @@
       <x:c r="B19" s="16" t="str">
         <x:v>Malaysia</x:v>
       </x:c>
-      <x:c r="C19" s="22" t="n">
+      <x:c r="C19" s="30" t="n">
         <x:v>281670.4396159676</x:v>
       </x:c>
-      <x:c r="D19" s="22" t="n">
+      <x:c r="D19" s="30" t="n">
         <x:v>240</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str"/>
@@ -3147,10 +3596,10 @@
       <x:c r="B20" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C20" s="22" t="n">
+      <x:c r="C20" s="30" t="n">
         <x:v>275795.85649317835</x:v>
       </x:c>
-      <x:c r="D20" s="22" t="n">
+      <x:c r="D20" s="30" t="n">
         <x:v>340</x:v>
       </x:c>
       <x:c r="E20" s="16" t="str">
@@ -3173,10 +3622,10 @@
       <x:c r="B21" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C21" s="22" t="n">
+      <x:c r="C21" s="30" t="n">
         <x:v>267812.02627589693</x:v>
       </x:c>
-      <x:c r="D21" s="22" t="n">
+      <x:c r="D21" s="30" t="n">
         <x:v>237</x:v>
       </x:c>
       <x:c r="E21" s="16" t="str">
@@ -3199,10 +3648,10 @@
       <x:c r="B22" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C22" s="22" t="n">
+      <x:c r="C22" s="30" t="n">
         <x:v>252652.85497726125</x:v>
       </x:c>
-      <x:c r="D22" s="22" t="n">
+      <x:c r="D22" s="30" t="n">
         <x:v>262</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
@@ -3225,10 +3674,10 @@
       <x:c r="B23" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C23" s="22" t="n">
+      <x:c r="C23" s="30" t="n">
         <x:v>244567.9636179889</x:v>
       </x:c>
-      <x:c r="D23" s="22" t="n">
+      <x:c r="D23" s="30" t="n">
         <x:v>105</x:v>
       </x:c>
       <x:c r="E23" s="16" t="str">
@@ -3247,10 +3696,10 @@
       <x:c r="B24" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C24" s="22" t="n">
+      <x:c r="C24" s="30" t="n">
         <x:v>242546.7407781708</x:v>
       </x:c>
-      <x:c r="D24" s="22" t="n">
+      <x:c r="D24" s="30" t="n">
         <x:v>238</x:v>
       </x:c>
       <x:c r="E24" s="16" t="str"/>
@@ -3269,10 +3718,10 @@
       <x:c r="B25" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C25" s="22" t="n">
+      <x:c r="C25" s="30" t="n">
         <x:v>215765.5381505811</x:v>
       </x:c>
-      <x:c r="D25" s="22" t="n">
+      <x:c r="D25" s="30" t="n">
         <x:v>178</x:v>
       </x:c>
       <x:c r="E25" s="16" t="str">
@@ -3295,10 +3744,10 @@
       <x:c r="B26" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C26" s="22" t="n">
+      <x:c r="C26" s="30" t="n">
         <x:v>214348.14354550533</x:v>
       </x:c>
-      <x:c r="D26" s="22" t="n">
+      <x:c r="D26" s="30" t="n">
         <x:v>284</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
@@ -3321,10 +3770,10 @@
       <x:c r="B27" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C27" s="22" t="n">
+      <x:c r="C27" s="30" t="n">
         <x:v>205154.11824153614</x:v>
       </x:c>
-      <x:c r="D27" s="22" t="n">
+      <x:c r="D27" s="30" t="n">
         <x:v>202</x:v>
       </x:c>
       <x:c r="E27" s="16" t="str">
@@ -3347,10 +3796,10 @@
       <x:c r="B28" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C28" s="22" t="n">
+      <x:c r="C28" s="30" t="n">
         <x:v>203132.89540171804</x:v>
       </x:c>
-      <x:c r="D28" s="22" t="n">
+      <x:c r="D28" s="30" t="n">
         <x:v>178</x:v>
       </x:c>
       <x:c r="E28" s="16" t="str">
@@ -3373,10 +3822,10 @@
       <x:c r="B29" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C29" s="22" t="n">
+      <x:c r="C29" s="30" t="n">
         <x:v>201616.97827185446</x:v>
       </x:c>
-      <x:c r="D29" s="22" t="n">
+      <x:c r="D29" s="30" t="n">
         <x:v>154</x:v>
       </x:c>
       <x:c r="E29" s="16" t="str">
@@ -3397,10 +3846,10 @@
       <x:c r="B30" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C30" s="22" t="n">
+      <x:c r="C30" s="30" t="n">
         <x:v>191005.5583628095</x:v>
       </x:c>
-      <x:c r="D30" s="22" t="n">
+      <x:c r="D30" s="30" t="n">
         <x:v>103</x:v>
       </x:c>
       <x:c r="E30" s="16" t="str">
@@ -3421,10 +3870,10 @@
       <x:c r="B31" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C31" s="22" t="n">
+      <x:c r="C31" s="30" t="n">
         <x:v>182920.66700353715</x:v>
       </x:c>
-      <x:c r="D31" s="22" t="n">
+      <x:c r="D31" s="30" t="n">
         <x:v>180</x:v>
       </x:c>
       <x:c r="E31" s="16" t="str"/>
@@ -3443,10 +3892,10 @@
       <x:c r="B32" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C32" s="22" t="n">
+      <x:c r="C32" s="30" t="n">
         <x:v>174835.77564426477</x:v>
       </x:c>
-      <x:c r="D32" s="22" t="n">
+      <x:c r="D32" s="30" t="n">
         <x:v>144</x:v>
       </x:c>
       <x:c r="E32" s="16" t="str"/>
@@ -3465,10 +3914,10 @@
       <x:c r="B33" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C33" s="22" t="n">
+      <x:c r="C33" s="30" t="n">
         <x:v>174517.43304699342</x:v>
       </x:c>
-      <x:c r="D33" s="22" t="n">
+      <x:c r="D33" s="30" t="n">
         <x:v>153</x:v>
       </x:c>
       <x:c r="E33" s="16" t="str">
@@ -3491,10 +3940,10 @@
       <x:c r="B34" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C34" s="22" t="n">
+      <x:c r="C34" s="30" t="n">
         <x:v>173319.85851440122</x:v>
       </x:c>
-      <x:c r="D34" s="22" t="n">
+      <x:c r="D34" s="30" t="n">
         <x:v>152</x:v>
       </x:c>
       <x:c r="E34" s="16" t="str">
@@ -3517,10 +3966,10 @@
       <x:c r="B35" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C35" s="22" t="n">
+      <x:c r="C35" s="30" t="n">
         <x:v>173247.6719844078</x:v>
       </x:c>
-      <x:c r="D35" s="22" t="n">
+      <x:c r="D35" s="30" t="n">
         <x:v>152</x:v>
       </x:c>
       <x:c r="E35" s="16" t="str">
@@ -3543,10 +3992,10 @@
       <x:c r="B36" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C36" s="22" t="n">
+      <x:c r="C36" s="30" t="n">
         <x:v>172814.5528044467</x:v>
       </x:c>
-      <x:c r="D36" s="22" t="n">
+      <x:c r="D36" s="30" t="n">
         <x:v>152</x:v>
       </x:c>
       <x:c r="E36" s="16" t="str">
@@ -3569,10 +4018,10 @@
       <x:c r="B37" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C37" s="22" t="n">
+      <x:c r="C37" s="30" t="n">
         <x:v>171298.6356745831</x:v>
       </x:c>
-      <x:c r="D37" s="22" t="n">
+      <x:c r="D37" s="30" t="n">
         <x:v>228</x:v>
       </x:c>
       <x:c r="E37" s="16" t="str">
@@ -3595,10 +4044,10 @@
       <x:c r="B38" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C38" s="22" t="n">
+      <x:c r="C38" s="30" t="n">
         <x:v>166760.9903991915</x:v>
       </x:c>
-      <x:c r="D38" s="22" t="n">
+      <x:c r="D38" s="30" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="E38" s="16" t="str">
@@ -3621,10 +4070,10 @@
       <x:c r="B39" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C39" s="22" t="n">
+      <x:c r="C39" s="30" t="n">
         <x:v>161697.82718544718</x:v>
       </x:c>
-      <x:c r="D39" s="22" t="n">
+      <x:c r="D39" s="30" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="E39" s="16" t="str">
@@ -3647,10 +4096,10 @@
       <x:c r="B40" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C40" s="22" t="n">
+      <x:c r="C40" s="30" t="n">
         <x:v>159551.768236855</x:v>
       </x:c>
-      <x:c r="D40" s="22" t="n">
+      <x:c r="D40" s="30" t="n">
         <x:v>132</x:v>
       </x:c>
       <x:c r="E40" s="16" t="str">
@@ -3673,10 +4122,10 @@
       <x:c r="B41" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C41" s="22" t="n">
+      <x:c r="C41" s="30" t="n">
         <x:v>157150.07579585648</x:v>
       </x:c>
-      <x:c r="D41" s="22" t="n">
+      <x:c r="D41" s="30" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="E41" s="16" t="str">
@@ -3697,10 +4146,10 @@
       <x:c r="B42" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C42" s="22" t="n">
+      <x:c r="C42" s="30" t="n">
         <x:v>155634.15866599293</x:v>
       </x:c>
-      <x:c r="D42" s="22" t="n">
+      <x:c r="D42" s="30" t="n">
         <x:v>190</x:v>
       </x:c>
       <x:c r="E42" s="16" t="str">
@@ -3723,10 +4172,10 @@
       <x:c r="B43" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C43" s="22" t="n">
+      <x:c r="C43" s="30" t="n">
         <x:v>153612.93582617483</x:v>
       </x:c>
-      <x:c r="D43" s="22" t="n">
+      <x:c r="D43" s="30" t="n">
         <x:v>161</x:v>
       </x:c>
       <x:c r="E43" s="16" t="str">
@@ -3747,10 +4196,10 @@
       <x:c r="B44" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C44" s="22" t="n">
+      <x:c r="C44" s="30" t="n">
         <x:v>151354.21930267813</x:v>
       </x:c>
-      <x:c r="D44" s="22" t="n">
+      <x:c r="D44" s="30" t="n">
         <x:v>133</x:v>
       </x:c>
       <x:c r="E44" s="16" t="str">
@@ -3773,10 +4222,10 @@
       <x:c r="B45" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C45" s="22" t="n">
+      <x:c r="C45" s="30" t="n">
         <x:v>130368.8731682668</x:v>
       </x:c>
-      <x:c r="D45" s="22" t="n">
+      <x:c r="D45" s="30" t="n">
         <x:v>137</x:v>
       </x:c>
       <x:c r="E45" s="16" t="str">
@@ -3797,10 +4246,10 @@
       <x:c r="B46" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C46" s="22" t="n">
+      <x:c r="C46" s="30" t="n">
         <x:v>123839</x:v>
       </x:c>
-      <x:c r="D46" s="22" t="n">
+      <x:c r="D46" s="30" t="n">
         <x:v>180</x:v>
       </x:c>
       <x:c r="E46" s="16" t="str">
@@ -3823,10 +4272,10 @@
       <x:c r="B47" s="16" t="str">
         <x:v>United Kingdom</x:v>
       </x:c>
-      <x:c r="C47" s="22" t="n">
+      <x:c r="C47" s="30" t="n">
         <x:v>123799.89893885801</x:v>
       </x:c>
-      <x:c r="D47" s="22" t="n">
+      <x:c r="D47" s="30" t="n">
         <x:v>88</x:v>
       </x:c>
       <x:c r="E47" s="16" t="str">
@@ -3849,10 +4298,10 @@
       <x:c r="B48" s="16" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="C48" s="22" t="n">
+      <x:c r="C48" s="30" t="n">
         <x:v>122789.28751894896</x:v>
       </x:c>
-      <x:c r="D48" s="22" t="n">
+      <x:c r="D48" s="30" t="n">
         <x:v>221</x:v>
       </x:c>
       <x:c r="E48" s="16" t="str">
@@ -3875,10 +4324,10 @@
       <x:c r="B49" s="16" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="C49" s="22" t="n">
+      <x:c r="C49" s="30" t="n">
         <x:v>117230.92470944922</x:v>
       </x:c>
-      <x:c r="D49" s="22" t="n">
+      <x:c r="D49" s="30" t="n">
         <x:v>241.8</x:v>
       </x:c>
       <x:c r="E49" s="16" t="str">
@@ -3899,10 +4348,10 @@
       <x:c r="B50" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C50" s="22" t="n">
+      <x:c r="C50" s="30" t="n">
         <x:v>108135.42193026781</x:v>
       </x:c>
-      <x:c r="D50" s="22" t="n">
+      <x:c r="D50" s="30" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="E50" s="16" t="str">
@@ -3923,10 +4372,10 @@
       <x:c r="B51" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C51" s="22" t="n">
+      <x:c r="C51" s="30" t="n">
         <x:v>99545.22486104093</x:v>
       </x:c>
-      <x:c r="D51" s="22" t="n">
+      <x:c r="D51" s="30" t="n">
         <x:v>87</x:v>
       </x:c>
       <x:c r="E51" s="16" t="str">
@@ -3949,10 +4398,10 @@
       <x:c r="B52" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C52" s="22" t="n">
+      <x:c r="C52" s="30" t="n">
         <x:v>99545.22486104093</x:v>
       </x:c>
-      <x:c r="D52" s="22" t="n">
+      <x:c r="D52" s="30" t="n">
         <x:v>87</x:v>
       </x:c>
       <x:c r="E52" s="16" t="str">
@@ -3975,10 +4424,10 @@
       <x:c r="B53" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C53" s="22" t="n">
+      <x:c r="C53" s="30" t="n">
         <x:v>93481.55634158666</x:v>
       </x:c>
-      <x:c r="D53" s="22" t="n">
+      <x:c r="D53" s="30" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="E53" s="16" t="str">
@@ -4001,10 +4450,10 @@
       <x:c r="B54" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C54" s="22" t="n">
+      <x:c r="C54" s="30" t="n">
         <x:v>91965.63921172309</x:v>
       </x:c>
-      <x:c r="D54" s="22" t="n">
+      <x:c r="D54" s="30" t="n">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E54" s="16" t="str">
@@ -4027,10 +4476,10 @@
       <x:c r="B55" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C55" s="22" t="n">
+      <x:c r="C55" s="30" t="n">
         <x:v>88428.49924204143</x:v>
       </x:c>
-      <x:c r="D55" s="22" t="n">
+      <x:c r="D55" s="30" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="E55" s="16" t="str">
@@ -4053,10 +4502,10 @@
       <x:c r="B56" s="16" t="str">
         <x:v>Indonesia</x:v>
       </x:c>
-      <x:c r="C56" s="22" t="n">
+      <x:c r="C56" s="30" t="n">
         <x:v>84386.05356240526</x:v>
       </x:c>
-      <x:c r="D56" s="22" t="n">
+      <x:c r="D56" s="30" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="E56" s="16" t="str">
@@ -4075,10 +4524,10 @@
       <x:c r="B57" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C57" s="22" t="n">
+      <x:c r="C57" s="30" t="n">
         <x:v>81354.21930267812</x:v>
       </x:c>
-      <x:c r="D57" s="22" t="n">
+      <x:c r="D57" s="30" t="n">
         <x:v>108</x:v>
       </x:c>
       <x:c r="E57" s="16" t="str">
@@ -4101,10 +4550,10 @@
       <x:c r="B58" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C58" s="22" t="n">
+      <x:c r="C58" s="30" t="n">
         <x:v>80343.60788276908</x:v>
       </x:c>
-      <x:c r="D58" s="22" t="n">
+      <x:c r="D58" s="30" t="n">
         <x:v>237</x:v>
       </x:c>
       <x:c r="E58" s="16" t="str">
@@ -4127,10 +4576,10 @@
       <x:c r="B59" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C59" s="22" t="n">
+      <x:c r="C59" s="30" t="n">
         <x:v>78827.6907529055</x:v>
       </x:c>
-      <x:c r="D59" s="22" t="n">
+      <x:c r="D59" s="30" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="E59" s="16" t="str">
@@ -4153,10 +4602,10 @@
       <x:c r="B60" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C60" s="22" t="n">
+      <x:c r="C60" s="30" t="n">
         <x:v>64679.13087417888</x:v>
       </x:c>
-      <x:c r="D60" s="22" t="n">
+      <x:c r="D60" s="30" t="n">
         <x:v>75</x:v>
       </x:c>
       <x:c r="E60" s="16" t="str">
@@ -4177,10 +4626,10 @@
       <x:c r="B61" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C61" s="22" t="n">
+      <x:c r="C61" s="30" t="n">
         <x:v>61141.99090449722</x:v>
       </x:c>
-      <x:c r="D61" s="22" t="n">
+      <x:c r="D61" s="30" t="n">
         <x:v>85</x:v>
       </x:c>
       <x:c r="E61" s="16" t="str"/>
@@ -4199,10 +4648,10 @@
       <x:c r="B62" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C62" s="22" t="n">
+      <x:c r="C62" s="30" t="n">
         <x:v>58564.93178372915</x:v>
       </x:c>
-      <x:c r="D62" s="22" t="n">
+      <x:c r="D62" s="30" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="E62" s="16" t="str">
@@ -4225,10 +4674,10 @@
       <x:c r="B63" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C63" s="22" t="n">
+      <x:c r="C63" s="30" t="n">
         <x:v>56846.89236988378</x:v>
       </x:c>
-      <x:c r="D63" s="22" t="n">
+      <x:c r="D63" s="30" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E63" s="16" t="str">
@@ -4251,10 +4700,10 @@
       <x:c r="B64" s="16" t="str">
         <x:v>Norway</x:v>
       </x:c>
-      <x:c r="C64" s="22" t="n">
+      <x:c r="C64" s="30" t="n">
         <x:v>50773.11773623042</x:v>
       </x:c>
-      <x:c r="D64" s="22" t="n">
+      <x:c r="D64" s="30" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="E64" s="16" t="str">
@@ -4277,10 +4726,10 @@
       <x:c r="B65" s="16" t="str">
         <x:v>Australia</x:v>
       </x:c>
-      <x:c r="C65" s="22" t="n">
+      <x:c r="C65" s="30" t="n">
         <x:v>46488.12531581607</x:v>
       </x:c>
-      <x:c r="D65" s="22" t="n">
+      <x:c r="D65" s="30" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="E65" s="16" t="str">
@@ -4299,10 +4748,10 @@
       <x:c r="B66" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C66" s="22" t="n">
+      <x:c r="C66" s="30" t="n">
         <x:v>46134.4113188479</x:v>
       </x:c>
-      <x:c r="D66" s="22" t="n">
+      <x:c r="D66" s="30" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="E66" s="16" t="str"/>
@@ -4321,10 +4770,10 @@
       <x:c r="B67" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C67" s="22" t="n">
+      <x:c r="C67" s="30" t="n">
         <x:v>45174.33046993431</x:v>
       </x:c>
-      <x:c r="D67" s="22" t="n">
+      <x:c r="D67" s="30" t="n">
         <x:v>47</x:v>
       </x:c>
       <x:c r="E67" s="16" t="str">
@@ -4345,10 +4794,10 @@
       <x:c r="B68" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C68" s="22" t="n">
+      <x:c r="C68" s="30" t="n">
         <x:v>38706.417382516425</x:v>
       </x:c>
-      <x:c r="D68" s="22" t="n">
+      <x:c r="D68" s="30" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="E68" s="16" t="str"/>
@@ -4367,10 +4816,10 @@
       <x:c r="B69" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C69" s="22" t="n">
+      <x:c r="C69" s="30" t="n">
         <x:v>32238.504295098533</x:v>
       </x:c>
-      <x:c r="D69" s="22" t="n">
+      <x:c r="D69" s="30" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E69" s="16" t="str">
@@ -4393,10 +4842,10 @@
       <x:c r="B70" s="16" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="C70" s="22" t="n">
+      <x:c r="C70" s="30" t="n">
         <x:v>31884.79029813037</x:v>
       </x:c>
-      <x:c r="D70" s="22" t="n">
+      <x:c r="D70" s="30" t="n">
         <x:v>169</x:v>
       </x:c>
       <x:c r="E70" s="16" t="str">
@@ -4419,10 +4868,10 @@
       <x:c r="B71" s="16" t="str">
         <x:v>Portugal</x:v>
       </x:c>
-      <x:c r="C71" s="22" t="n">
+      <x:c r="C71" s="30" t="n">
         <x:v>31834.259727134915</x:v>
       </x:c>
-      <x:c r="D71" s="22" t="n">
+      <x:c r="D71" s="30" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="E71" s="16" t="str">
@@ -4445,10 +4894,10 @@
       <x:c r="B72" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C72" s="22" t="n">
+      <x:c r="C72" s="30" t="n">
         <x:v>11470.43961596766</x:v>
       </x:c>
-      <x:c r="D72" s="22" t="n">
+      <x:c r="D72" s="30" t="n">
         <x:v>17.32971</x:v>
       </x:c>
       <x:c r="E72" s="16" t="str">
@@ -4471,10 +4920,10 @@
       <x:c r="B73" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C73" s="22" t="n">
+      <x:c r="C73" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D73" s="22" t="n">
+      <x:c r="D73" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E73" s="16" t="str">
@@ -4497,10 +4946,10 @@
       <x:c r="B74" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C74" s="22" t="n">
+      <x:c r="C74" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D74" s="22" t="n">
+      <x:c r="D74" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E74" s="16" t="str">
@@ -4523,10 +4972,10 @@
       <x:c r="B75" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C75" s="22" t="n">
+      <x:c r="C75" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D75" s="22" t="n">
+      <x:c r="D75" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E75" s="16" t="str">
@@ -4549,10 +4998,10 @@
       <x:c r="B76" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C76" s="22" t="n">
+      <x:c r="C76" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D76" s="22" t="n">
+      <x:c r="D76" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E76" s="16" t="str">
@@ -4575,10 +5024,10 @@
       <x:c r="B77" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C77" s="22" t="n">
+      <x:c r="C77" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D77" s="22" t="n">
+      <x:c r="D77" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E77" s="16" t="str">
@@ -4601,10 +5050,10 @@
       <x:c r="B78" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C78" s="22" t="n">
+      <x:c r="C78" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D78" s="22" t="n">
+      <x:c r="D78" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E78" s="16" t="str">
@@ -4627,10 +5076,10 @@
       <x:c r="B79" s="16" t="str">
         <x:v>Norway</x:v>
       </x:c>
-      <x:c r="C79" s="22" t="n">
+      <x:c r="C79" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D79" s="22" t="n">
+      <x:c r="D79" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E79" s="16" t="str">
@@ -4651,10 +5100,10 @@
       <x:c r="B80" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C80" s="22" t="n">
+      <x:c r="C80" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D80" s="22" t="n">
+      <x:c r="D80" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E80" s="16" t="str">
@@ -4677,10 +5126,10 @@
       <x:c r="B81" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C81" s="22" t="n">
+      <x:c r="C81" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D81" s="22" t="n">
+      <x:c r="D81" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E81" s="16" t="str">
@@ -4701,10 +5150,10 @@
       <x:c r="B82" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C82" s="22" t="n">
+      <x:c r="C82" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D82" s="22" t="n">
+      <x:c r="D82" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E82" s="16" t="str">
@@ -4725,10 +5174,10 @@
       <x:c r="B83" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C83" s="22" t="n">
+      <x:c r="C83" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D83" s="22" t="n">
+      <x:c r="D83" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E83" s="16" t="str">
@@ -4749,10 +5198,10 @@
       <x:c r="B84" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C84" s="22" t="n">
+      <x:c r="C84" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D84" s="22" t="n">
+      <x:c r="D84" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E84" s="16" t="str">
@@ -4775,10 +5224,10 @@
       <x:c r="B85" s="16" t="str">
         <x:v>United Arab Emirates</x:v>
       </x:c>
-      <x:c r="C85" s="22" t="n">
+      <x:c r="C85" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D85" s="22" t="n">
+      <x:c r="D85" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E85" s="16" t="str">
@@ -4801,10 +5250,10 @@
       <x:c r="B86" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C86" s="22" t="n">
+      <x:c r="C86" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D86" s="22" t="n">
+      <x:c r="D86" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E86" s="16" t="str">
@@ -4825,10 +5274,10 @@
       <x:c r="B87" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C87" s="22" t="n">
+      <x:c r="C87" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D87" s="22" t="n">
+      <x:c r="D87" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E87" s="16" t="str"/>
@@ -4847,10 +5296,10 @@
       <x:c r="B88" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="C88" s="22" t="n">
+      <x:c r="C88" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D88" s="22" t="n">
+      <x:c r="D88" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E88" s="16" t="str"/>
@@ -4871,12 +5320,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf05bb1b0646f4b83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ba68b4cd3614b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5608,12 +6057,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76dbd5e7c0da4135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b77d05a3d84c3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5773,26 +6222,72 @@
         <x:v>Country identifies the U.S. sites included in the quarterly timeline reconstruction. Current power is the registry’s current IT-power estimate and is retained as a facility-level audit field; the quarterly gate path is reconstructed from the dated timeline.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="97.19999694824219" hidden="0" customHeight="1">
+    <x:row r="10" ht="151.1999969482422" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
+        <x:v>gate2-github-com-mlperf-inference-v5-0-power</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>MLCommons</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>MLPerf Inference v5.0 summary results</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str">
+        <x:v>measured inference goodput, measured system power, productivity trend</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="str">
+        <x:v>https://raw.githubusercontent.com/mlcommons/inference_results_v5.0/main/summary_results.json</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>Official MLPerf result data. The selected row is an available, closed, datacenter Server result with a reported power measurement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="162" hidden="0" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>gate2-github-com-mlperf-inference-v5-1-power</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>MLCommons</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>MLPerf Inference v5.1 summary results</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>measured inference goodput, measured system power, absolute productivity baseline, productivity trend</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>https://raw.githubusercontent.com/mlcommons/inference_results_v5.1/main/summary_results.json</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>Official MLPerf result data. Both selected rows are available, closed, datacenter Server results with reported power measurements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="97.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A12" s="16" t="str">
         <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
-      <x:c r="B10" s="16" t="str">
+      <x:c r="B12" s="16" t="str">
         <x:v>U.S. Census Bureau</x:v>
       </x:c>
-      <x:c r="C10" s="16" t="str">
+      <x:c r="C12" s="16" t="str">
         <x:v>Population on a Date</x:v>
       </x:c>
-      <x:c r="D10" s="16" t="str">
+      <x:c r="D12" s="16" t="str">
         <x:v>2026-07-26</x:v>
       </x:c>
-      <x:c r="E10" s="16" t="str">
+      <x:c r="E12" s="16" t="str">
         <x:v>population</x:v>
       </x:c>
-      <x:c r="F10" s="16" t="str">
+      <x:c r="F12" s="16" t="str">
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
-      <x:c r="G10" s="16" t="str">
+      <x:c r="G12" s="16" t="str">
         <x:v>The model uses the rounded estimate of 342.8M residents; the selected 25% target is 85.7M users.</x:v>
       </x:c>
     </x:row>
@@ -5803,7 +6298,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8736dfb99f9d470f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R185db697ba804aa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update scenario defaults and Meaning action plan
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R14841b2bf70f4d10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R0a091bef3a9248cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R9d80095689d04485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="R1a7fc35224b24bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R848ea7aeb0bb48e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="Rdc294570e7164d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Radf4a4a525064650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rea81561ff8d94e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R03af11cffa6b457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R19e1168c774a449c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="Ra73d56f12697463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R508d58e643374956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="R06caffffb52d407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Rf4a34dfbb7dd463c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -305,7 +305,7 @@
         <c:axId val="48672768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="428500000"/>
+          <c:max val="857000000"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -370,7 +370,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R90d224de0a6d4a2e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d3677f05a094e10"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -847,10 +847,10 @@
         <x:v>Target users</x:v>
       </x:c>
       <x:c r="B15" s="24" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="C15" s="23" t="str">
-        <x:v>25% of U.S. population</x:v>
+        <x:v>50% of U.S. population</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -858,7 +858,7 @@
         <x:v>Current supply score</x:v>
       </x:c>
       <x:c r="B16" s="25" t="n">
-        <x:v>0.09074318166135269</x:v>
+        <x:v>0.045371590830676344</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
         <x:v>supported users / target users</x:v>
@@ -946,7 +946,7 @@
         <x:v>Continuous base-case crossing</x:v>
       </x:c>
       <x:c r="B24" s="29" t="n">
-        <x:v>46603.441982048615</x:v>
+        <x:v>46698.26714887731</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
         <x:v>100% of selected target</x:v>
@@ -959,7 +959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9325a32037e4a17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77aca973a42a49a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1200,10 +1200,10 @@
         <x:v>837.5373556125388</x:v>
       </x:c>
       <x:c r="R6" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S6" s="18" t="n">
-        <x:v>0.000009772897965140476</x:v>
+        <x:v>0.000004886448982570238</x:v>
       </x:c>
       <x:c r="T6" s="16" t="str">
         <x:v>F</x:v>
@@ -1271,10 +1271,10 @@
         <x:v>2836.9563242845466</x:v>
       </x:c>
       <x:c r="R7" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S7" s="18" t="n">
-        <x:v>0.00003310334100682085</x:v>
+        <x:v>0.000016551670503410424</x:v>
       </x:c>
       <x:c r="T7" s="16" t="str">
         <x:v>F</x:v>
@@ -1342,10 +1342,10 @@
         <x:v>7712.5195850115315</x:v>
       </x:c>
       <x:c r="R8" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S8" s="18" t="n">
-        <x:v>0.0000899943942241719</x:v>
+        <x:v>0.00004499719711208595</x:v>
       </x:c>
       <x:c r="T8" s="16" t="str">
         <x:v>F</x:v>
@@ -1413,10 +1413,10 @@
         <x:v>17875.506708732762</x:v>
       </x:c>
       <x:c r="R9" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S9" s="18" t="n">
-        <x:v>0.00020858234199221427</x:v>
+        <x:v>0.00010429117099610713</x:v>
       </x:c>
       <x:c r="T9" s="16" t="str">
         <x:v>F</x:v>
@@ -1484,10 +1484,10 @@
         <x:v>42736.76665152513</x:v>
       </x:c>
       <x:c r="R10" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S10" s="18" t="n">
-        <x:v>0.0004986787240551357</x:v>
+        <x:v>0.00024933936202756787</x:v>
       </x:c>
       <x:c r="T10" s="16" t="str">
         <x:v>F</x:v>
@@ -1555,10 +1555,10 @@
         <x:v>113794.75793722417</x:v>
       </x:c>
       <x:c r="R11" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S11" s="18" t="n">
-        <x:v>0.0013278268137365714</x:v>
+        <x:v>0.0006639134068682857</x:v>
       </x:c>
       <x:c r="T11" s="16" t="str">
         <x:v>F</x:v>
@@ -1626,10 +1626,10 @@
         <x:v>231989.642260386</x:v>
       </x:c>
       <x:c r="R12" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S12" s="18" t="n">
-        <x:v>0.0027069969925365926</x:v>
+        <x:v>0.0013534984962682963</x:v>
       </x:c>
       <x:c r="T12" s="16" t="str">
         <x:v>F</x:v>
@@ -1697,10 +1697,10 @@
         <x:v>626763.0654758726</x:v>
       </x:c>
       <x:c r="R13" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S13" s="18" t="n">
-        <x:v>0.007313454672997347</x:v>
+        <x:v>0.0036567273364986734</x:v>
       </x:c>
       <x:c r="T13" s="16" t="str">
         <x:v>F</x:v>
@@ -1768,10 +1768,10 @@
         <x:v>1328343.93951699</x:v>
       </x:c>
       <x:c r="R14" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S14" s="18" t="n">
-        <x:v>0.015499929282578645</x:v>
+        <x:v>0.007749964641289323</x:v>
       </x:c>
       <x:c r="T14" s="16" t="str">
         <x:v>F</x:v>
@@ -1839,10 +1839,10 @@
         <x:v>3817893.5119782407</x:v>
       </x:c>
       <x:c r="R15" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S15" s="18" t="n">
-        <x:v>0.04454951589239487</x:v>
+        <x:v>0.022274757946197436</x:v>
       </x:c>
       <x:c r="T15" s="16" t="str">
         <x:v>F</x:v>
@@ -1910,10 +1910,10 @@
         <x:v>7776690.668377926</x:v>
       </x:c>
       <x:c r="R16" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S16" s="18" t="n">
-        <x:v>0.09074318166135269</x:v>
+        <x:v>0.045371590830676344</x:v>
       </x:c>
       <x:c r="T16" s="16" t="str">
         <x:v>F</x:v>
@@ -1981,10 +1981,10 @@
         <x:v>16585666.017618544</x:v>
       </x:c>
       <x:c r="R17" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S17" s="18" t="n">
-        <x:v>0.19353169215424207</x:v>
+        <x:v>0.09676584607712103</x:v>
       </x:c>
       <x:c r="T17" s="16" t="str">
         <x:v>F</x:v>
@@ -2052,10 +2052,10 @@
         <x:v>34270741.59326548</x:v>
       </x:c>
       <x:c r="R18" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S18" s="18" t="n">
-        <x:v>0.3998919672493055</x:v>
+        <x:v>0.19994598362465274</x:v>
       </x:c>
       <x:c r="T18" s="16" t="str">
         <x:v>F</x:v>
@@ -2123,16 +2123,16 @@
         <x:v>64175039.74371664</x:v>
       </x:c>
       <x:c r="R19" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S19" s="18" t="n">
-        <x:v>0.7488336026104626</x:v>
+        <x:v>0.3744168013052313</x:v>
       </x:c>
       <x:c r="T19" s="16" t="str">
-        <x:v>C</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="U19" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="V19" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -2194,16 +2194,16 @@
         <x:v>121611697.0397346</x:v>
       </x:c>
       <x:c r="R20" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S20" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7095198193683465</x:v>
       </x:c>
       <x:c r="T20" s="16" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="U20" s="16" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="V20" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
@@ -2265,7 +2265,7 @@
         <x:v>248943311.9710166</x:v>
       </x:c>
       <x:c r="R21" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S21" s="18" t="n">
         <x:v>1</x:v>
@@ -2336,7 +2336,7 @@
         <x:v>537174086.5139235</x:v>
       </x:c>
       <x:c r="R22" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S22" s="18" t="n">
         <x:v>1</x:v>
@@ -2407,7 +2407,7 @@
         <x:v>1072794861.3651623</x:v>
       </x:c>
       <x:c r="R23" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S23" s="18" t="n">
         <x:v>1</x:v>
@@ -2478,7 +2478,7 @@
         <x:v>1984876693.602504</x:v>
       </x:c>
       <x:c r="R24" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S24" s="18" t="n">
         <x:v>1</x:v>
@@ -2549,7 +2549,7 @@
         <x:v>4244086037.882496</x:v>
       </x:c>
       <x:c r="R25" s="19" t="n">
-        <x:v>85700000</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="S25" s="18" t="n">
         <x:v>1</x:v>
@@ -2573,9 +2573,9 @@
     <x:mergeCell ref="A3:W3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e6cf5e1565b4a4d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3172ccc6127f4651"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f0a82152cfd496b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931900e3c7814986"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2649,7 +2649,7 @@
         <x:v>Selected target</x:v>
       </x:c>
       <x:c r="C7" s="20" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>share of residents</x:v>
@@ -2816,7 +2816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8626d6fceb2444bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ed5c3933ec246fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3157,7 +3157,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00875049a3604f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R428613e4ff71468d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5320,7 +5320,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ba68b4cd3614b53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf164e0b9f0540ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6057,7 +6057,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b77d05a3d84c3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd396e964e5154e4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6298,7 +6298,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R185db697ba804aa7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7b093100e1c4771"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh Personal AI evidence through 2026-09-03
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rea81561ff8d94e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R03af11cffa6b457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R19e1168c774a449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="Ra73d56f12697463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R508d58e643374956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="R06caffffb52d407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Rf4a34dfbb7dd463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2da30dcbf2644ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R4e57fe731aed462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R8b6747e16928477a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="Rfacee16119404a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R136faaaa791e4014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="Ra154bf24a5d44a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R52db042ed24f4e99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d3677f05a094e10"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f69d6086dc04ff9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -461,7 +461,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSiteRegistryTable" displayName="ComputeSiteRegistryTable" ref="A5:H88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ComputeSiteRegistryTable" displayName="ComputeSiteRegistryTable" ref="A5:H91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Site"/>
     <x:tableColumn id="2" name="Country"/>
@@ -477,7 +477,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ComputeSupportingEvidenceTable" displayName="ComputeSupportingEvidenceTable" ref="A5:M24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Metric"/>
@@ -498,7 +498,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ComputeSourcesTable" displayName="ComputeSourcesTable" ref="A5:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -726,7 +726,7 @@
     </x:row>
     <x:row r="3" ht="72" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Snapshot 2026-08-26. The supply gate combines operational IT power, inference productivity, allocation, and workload; it passes only at 100% of the selected population target.</x:v>
+        <x:v>Snapshot 2026-09-03. The supply gate combines operational IT power, inference productivity, allocation, and workload; it passes only at 100% of the selected population target.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -748,7 +748,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
         <x:v>Latest immutable snapshot selected automatically</x:v>
@@ -759,7 +759,7 @@
         <x:v>Current U.S. operational IT power</x:v>
       </x:c>
       <x:c r="B7" s="24" t="n">
-        <x:v>11.87932971</x:v>
+        <x:v>12.10932971</x:v>
       </x:c>
       <x:c r="C7" s="23" t="str">
         <x:v>IT GW</x:v>
@@ -814,7 +814,7 @@
         <x:v>Current H100e audit cross-check</x:v>
       </x:c>
       <x:c r="B12" s="24" t="n">
-        <x:v>13524006</x:v>
+        <x:v>13046294</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
         <x:v>audit only; excluded from capacity</x:v>
@@ -825,7 +825,7 @@
         <x:v>H100e-derived audit productivity</x:v>
       </x:c>
       <x:c r="B13" s="24" t="n">
-        <x:v>227.10136510717322</x:v>
+        <x:v>214.91829338098017</x:v>
       </x:c>
       <x:c r="C13" s="23" t="str">
         <x:v>trillion reference token-equivalents / IT GW-day; audit only</x:v>
@@ -836,7 +836,7 @@
         <x:v>Current supported users</x:v>
       </x:c>
       <x:c r="B14" s="24" t="n">
-        <x:v>7776690.668377926</x:v>
+        <x:v>7927257.989716033</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
         <x:v>Personal-AI user-equivalents</x:v>
@@ -858,7 +858,7 @@
         <x:v>Current supply score</x:v>
       </x:c>
       <x:c r="B16" s="25" t="n">
-        <x:v>0.045371590830676344</x:v>
+        <x:v>0.046250046614445935</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
         <x:v>supported users / target users</x:v>
@@ -902,7 +902,7 @@
         <x:v>IT-power mean projected log velocity</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
-        <x:v>0.15720673944051156</x:v>
+        <x:v>0.15695205385379454</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
         <x:v>log₂ IT GW / quarter</x:v>
@@ -913,7 +913,7 @@
         <x:v>IT-power projected log acceleration</x:v>
       </x:c>
       <x:c r="B21" s="28" t="n">
-        <x:v>-0.0015030413270408216</x:v>
+        <x:v>-0.0047256959081981055</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str">
         <x:v>log₂ IT GW / quarter²</x:v>
@@ -946,7 +946,7 @@
         <x:v>Continuous base-case crossing</x:v>
       </x:c>
       <x:c r="B24" s="29" t="n">
-        <x:v>46698.26714887731</x:v>
+        <x:v>46692.26532878472</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
         <x:v>100% of selected target</x:v>
@@ -959,7 +959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77aca973a42a49a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fe90c70b5054888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1176,16 +1176,16 @@
         <x:v>603</x:v>
       </x:c>
       <x:c r="H6" s="30" t="n">
-        <x:v>245664</x:v>
+        <x:v>240662</x:v>
       </x:c>
       <x:c r="I6" s="30" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="J6" s="30" t="n">
-        <x:v>519374.2071881607</x:v>
+        <x:v>508799.1543340381</x:v>
       </x:c>
       <x:c r="K6" s="31" t="n">
-        <x:v>103.6064288473573</x:v>
+        <x:v>101.49688346384778</x:v>
       </x:c>
       <x:c r="L6" s="31" t="n">
         <x:v>0.12357955167820671</x:v>
@@ -1232,49 +1232,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E7" s="30" t="n">
-        <x:v>887</x:v>
+        <x:v>875</x:v>
       </x:c>
       <x:c r="F7" s="30" t="n">
-        <x:v>0.887</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="G7" s="30" t="n">
-        <x:v>1121</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="H7" s="30" t="n">
-        <x:v>475238</x:v>
+        <x:v>465052</x:v>
       </x:c>
       <x:c r="I7" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="J7" s="30" t="n">
-        <x:v>535781.2852311161</x:v>
+        <x:v>531488</x:v>
       </x:c>
       <x:c r="K7" s="31" t="n">
-        <x:v>106.87936527801578</x:v>
+        <x:v>106.0229270016</x:v>
       </x:c>
       <x:c r="L7" s="31" t="n">
         <x:v>0.22321974084820626</x:v>
       </x:c>
       <x:c r="M7" s="31" t="n">
-        <x:v>0.9070939209616689</x:v>
+        <x:v>0.8874428333802962</x:v>
       </x:c>
       <x:c r="N7" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O7" s="31" t="n">
-        <x:v>0.9519637402300738</x:v>
+        <x:v>0.9503836794155376</x:v>
       </x:c>
       <x:c r="P7" s="19" t="n">
-        <x:v>47519018431.76615</x:v>
+        <x:v>46876145578.123314</x:v>
       </x:c>
       <x:c r="Q7" s="19" t="n">
-        <x:v>2836.9563242845466</x:v>
+        <x:v>2798.5758554103472</x:v>
       </x:c>
       <x:c r="R7" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S7" s="18" t="n">
-        <x:v>0.000016551670503410424</x:v>
+        <x:v>0.00001632774711441276</x:v>
       </x:c>
       <x:c r="T7" s="16" t="str">
         <x:v>F</x:v>
@@ -1303,49 +1303,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E8" s="30" t="n">
-        <x:v>1335</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="F8" s="30" t="n">
-        <x:v>1.335</x:v>
+        <x:v>1.323</x:v>
       </x:c>
       <x:c r="G8" s="30" t="n">
-        <x:v>1676</x:v>
+        <x:v>1661</x:v>
       </x:c>
       <x:c r="H8" s="30" t="n">
-        <x:v>722180</x:v>
+        <x:v>723011</x:v>
       </x:c>
       <x:c r="I8" s="30" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J8" s="30" t="n">
-        <x:v>540958.8014981274</x:v>
+        <x:v>546493.5752078609</x:v>
       </x:c>
       <x:c r="K8" s="31" t="n">
-        <x:v>107.91219279101125</x:v>
+        <x:v>109.01628716190477</x:v>
       </x:c>
       <x:c r="L8" s="31" t="n">
         <x:v>0.40319819927884876</x:v>
       </x:c>
       <x:c r="M8" s="31" t="n">
-        <x:v>0.5898337322738523</x:v>
+        <x:v>0.5964581395589856</x:v>
       </x:c>
       <x:c r="N8" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O8" s="31" t="n">
-        <x:v>0.6037082683951738</x:v>
+        <x:v>0.6366255558869831</x:v>
       </x:c>
       <x:c r="P8" s="19" t="n">
-        <x:v>129184703048.94315</x:v>
+        <x:v>128023492235.02005</x:v>
       </x:c>
       <x:c r="Q8" s="19" t="n">
-        <x:v>7712.5195850115315</x:v>
+        <x:v>7643.193566269853</x:v>
       </x:c>
       <x:c r="R8" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S8" s="18" t="n">
-        <x:v>0.00004499719711208595</x:v>
+        <x:v>0.00004459272792456157</x:v>
       </x:c>
       <x:c r="T8" s="16" t="str">
         <x:v>F</x:v>
@@ -1374,49 +1374,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E9" s="30" t="n">
-        <x:v>1713</x:v>
+        <x:v>1814</x:v>
       </x:c>
       <x:c r="F9" s="30" t="n">
-        <x:v>1.713</x:v>
+        <x:v>1.814</x:v>
       </x:c>
       <x:c r="G9" s="30" t="n">
-        <x:v>2165</x:v>
+        <x:v>2286</x:v>
       </x:c>
       <x:c r="H9" s="30" t="n">
-        <x:v>1012483</x:v>
+        <x:v>1066724</x:v>
       </x:c>
       <x:c r="I9" s="30" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="J9" s="30" t="n">
-        <x:v>591058.3771161705</x:v>
+        <x:v>588050.7166482911</x:v>
       </x:c>
       <x:c r="K9" s="31" t="n">
-        <x:v>117.90621645394046</x:v>
+        <x:v>117.30623871929437</x:v>
       </x:c>
       <x:c r="L9" s="31" t="n">
         <x:v>0.7282903711112904</x:v>
       </x:c>
       <x:c r="M9" s="31" t="n">
-        <x:v>0.35968540950908284</x:v>
+        <x:v>0.4553613942498458</x:v>
       </x:c>
       <x:c r="N9" s="31" t="n">
         <x:v>0.8530245754425181</x:v>
       </x:c>
       <x:c r="O9" s="31" t="n">
-        <x:v>0.48746731270438204</x:v>
+        <x:v>0.5610974453268476</x:v>
       </x:c>
       <x:c r="P9" s="19" t="n">
-        <x:v>299414737371.27374</x:v>
+        <x:v>317068495967.0114</x:v>
       </x:c>
       <x:c r="Q9" s="19" t="n">
-        <x:v>17875.506708732762</x:v>
+        <x:v>18929.462445791727</x:v>
       </x:c>
       <x:c r="R9" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S9" s="18" t="n">
-        <x:v>0.00010429117099610713</x:v>
+        <x:v>0.00011044027097894823</x:v>
       </x:c>
       <x:c r="T9" s="16" t="str">
         <x:v>F</x:v>
@@ -1445,49 +1445,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E10" s="30" t="n">
-        <x:v>2267.32971</x:v>
+        <x:v>2368.32971</x:v>
       </x:c>
       <x:c r="F10" s="30" t="n">
-        <x:v>2.26732971</x:v>
+        <x:v>2.36832971</x:v>
       </x:c>
       <x:c r="G10" s="30" t="n">
-        <x:v>2874</x:v>
+        <x:v>2995</x:v>
       </x:c>
       <x:c r="H10" s="30" t="n">
-        <x:v>1351240</x:v>
+        <x:v>1357224</x:v>
       </x:c>
       <x:c r="I10" s="30" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="J10" s="30" t="n">
-        <x:v>595960.9641422641</x:v>
+        <x:v>573072.2349465438</x:v>
       </x:c>
       <x:c r="K10" s="31" t="n">
-        <x:v>118.88420020218409</x:v>
+        <x:v>114.31828325828839</x:v>
       </x:c>
       <x:c r="L10" s="31" t="n">
         <x:v>1.3154990910229631</x:v>
       </x:c>
       <x:c r="M10" s="31" t="n">
-        <x:v>0.4044690483884812</x:v>
+        <x:v>0.38469548568734757</x:v>
       </x:c>
       <x:c r="N10" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O10" s="31" t="n">
-        <x:v>0.416386256410302</x:v>
+        <x:v>0.3474718996186219</x:v>
       </x:c>
       <x:c r="P10" s="19" t="n">
-        <x:v>715840841413.046</x:v>
+        <x:v>747728539379.4426</x:v>
       </x:c>
       <x:c r="Q10" s="19" t="n">
-        <x:v>42736.76665152513</x:v>
+        <x:v>44640.50981369807</x:v>
       </x:c>
       <x:c r="R10" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S10" s="18" t="n">
-        <x:v>0.00024933936202756787</x:v>
+        <x:v>0.00026044638164351264</x:v>
       </x:c>
       <x:c r="T10" s="16" t="str">
         <x:v>F</x:v>
@@ -1516,49 +1516,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E11" s="30" t="n">
-        <x:v>3342.32971</x:v>
+        <x:v>3431.32971</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
-        <x:v>3.34232971</x:v>
+        <x:v>3.43132971</x:v>
       </x:c>
       <x:c r="G11" s="30" t="n">
-        <x:v>4187</x:v>
+        <x:v>4293</x:v>
       </x:c>
       <x:c r="H11" s="30" t="n">
-        <x:v>2386876</x:v>
+        <x:v>2306541</x:v>
       </x:c>
       <x:c r="I11" s="30" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J11" s="30" t="n">
-        <x:v>714135.410656419</x:v>
+        <x:v>672200.3406661844</x:v>
       </x:c>
       <x:c r="K11" s="31" t="n">
-        <x:v>142.45801695105655</x:v>
+        <x:v>134.0926749971806</x:v>
       </x:c>
       <x:c r="L11" s="31" t="n">
         <x:v>2.3761646825587324</x:v>
       </x:c>
       <x:c r="M11" s="31" t="n">
-        <x:v>0.5598598578015919</x:v>
+        <x:v>0.5348978168477698</x:v>
       </x:c>
       <x:c r="N11" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O11" s="31" t="n">
-        <x:v>0.8208396780997056</x:v>
+        <x:v>0.76507209052291</x:v>
       </x:c>
       <x:c r="P11" s="19" t="n">
-        <x:v>1906062195448.505</x:v>
+        <x:v>1956817073067.9595</x:v>
       </x:c>
       <x:c r="Q11" s="19" t="n">
-        <x:v>113794.75793722417</x:v>
+        <x:v>116824.8998846543</x:v>
       </x:c>
       <x:c r="R11" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S11" s="18" t="n">
-        <x:v>0.0006639134068682857</x:v>
+        <x:v>0.0006815921813573763</x:v>
       </x:c>
       <x:c r="T11" s="16" t="str">
         <x:v>F</x:v>
@@ -1587,49 +1587,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E12" s="30" t="n">
-        <x:v>3772.32971</x:v>
+        <x:v>3861.32971</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
-        <x:v>3.77232971</x:v>
+        <x:v>3.86132971</x:v>
       </x:c>
       <x:c r="G12" s="30" t="n">
-        <x:v>4764</x:v>
+        <x:v>4870</x:v>
       </x:c>
       <x:c r="H12" s="30" t="n">
-        <x:v>3139660</x:v>
+        <x:v>3043660</x:v>
       </x:c>
       <x:c r="I12" s="30" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J12" s="30" t="n">
-        <x:v>832286.7409169279</x:v>
+        <x:v>788241.416452365</x:v>
       </x:c>
       <x:c r="K12" s="31" t="n">
-        <x:v>166.02722239567973</x:v>
+        <x:v>157.24092012645042</x:v>
       </x:c>
       <x:c r="L12" s="31" t="n">
         <x:v>4.292027746099666</x:v>
       </x:c>
       <x:c r="M12" s="31" t="n">
-        <x:v>0.17460171866453855</x:v>
+        <x:v>0.17032998952575285</x:v>
       </x:c>
       <x:c r="N12" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O12" s="31" t="n">
-        <x:v>0.3954847159961119</x:v>
+        <x:v>0.4000762705122298</x:v>
       </x:c>
       <x:c r="P12" s="19" t="n">
-        <x:v>3885826507861.4653</x:v>
+        <x:v>3977504220518.1543</x:v>
       </x:c>
       <x:c r="Q12" s="19" t="n">
-        <x:v>231989.642260386</x:v>
+        <x:v>237462.93853839728</x:v>
       </x:c>
       <x:c r="R12" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S12" s="18" t="n">
-        <x:v>0.0013534984962682963</x:v>
+        <x:v>0.0013854313800373238</x:v>
       </x:c>
       <x:c r="T12" s="16" t="str">
         <x:v>F</x:v>
@@ -1658,49 +1658,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E13" s="30" t="n">
-        <x:v>5642.32971</x:v>
+        <x:v>5747.32971</x:v>
       </x:c>
       <x:c r="F13" s="30" t="n">
-        <x:v>5.64232971</x:v>
+        <x:v>5.74732971</x:v>
       </x:c>
       <x:c r="G13" s="30" t="n">
-        <x:v>7211</x:v>
+        <x:v>7336</x:v>
       </x:c>
       <x:c r="H13" s="30" t="n">
-        <x:v>5291375</x:v>
+        <x:v>5215133</x:v>
       </x:c>
       <x:c r="I13" s="30" t="n">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="J13" s="30" t="n">
-        <x:v>937799.6806216416</x:v>
+        <x:v>907401.0476423494</x:v>
       </x:c>
       <x:c r="K13" s="31" t="n">
-        <x:v>187.07528124938307</x:v>
+        <x:v>181.01126466704832</x:v>
       </x:c>
       <x:c r="L13" s="31" t="n">
         <x:v>7.752620139717122</x:v>
       </x:c>
       <x:c r="M13" s="31" t="n">
-        <x:v>0.580835196113413</x:v>
+        <x:v>0.5737940674436219</x:v>
       </x:c>
       <x:c r="N13" s="31" t="n">
         <x:v>0.8530245754425181</x:v>
       </x:c>
       <x:c r="O13" s="31" t="n">
-        <x:v>0.7530343299629934</x:v>
+        <x:v>0.7768968380209245</x:v>
       </x:c>
       <x:c r="P13" s="19" t="n">
-        <x:v>10498281346720.865</x:v>
+        <x:v>10693647374241.736</x:v>
       </x:c>
       <x:c r="Q13" s="19" t="n">
-        <x:v>626763.0654758726</x:v>
+        <x:v>638426.7089099544</x:v>
       </x:c>
       <x:c r="R13" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S13" s="18" t="n">
-        <x:v>0.0036567273364986734</x:v>
+        <x:v>0.0037247765980744133</x:v>
       </x:c>
       <x:c r="T13" s="16" t="str">
         <x:v>F</x:v>
@@ -1729,49 +1729,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E14" s="30" t="n">
-        <x:v>6620.32971</x:v>
+        <x:v>6867.32971</x:v>
       </x:c>
       <x:c r="F14" s="30" t="n">
-        <x:v>6.62032971</x:v>
+        <x:v>6.86732971</x:v>
       </x:c>
       <x:c r="G14" s="30" t="n">
-        <x:v>8454.2</x:v>
+        <x:v>8737.2</x:v>
       </x:c>
       <x:c r="H14" s="30" t="n">
-        <x:v>6301294</x:v>
+        <x:v>6385550</x:v>
       </x:c>
       <x:c r="I14" s="30" t="n">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="J14" s="30" t="n">
-        <x:v>951809.6946866412</x:v>
+        <x:v>929844.6804878982</x:v>
       </x:c>
       <x:c r="K14" s="31" t="n">
-        <x:v>189.8700436871142</x:v>
+        <x:v>185.4883923667035</x:v>
       </x:c>
       <x:c r="L14" s="31" t="n">
         <x:v>14.003432080644302</x:v>
       </x:c>
       <x:c r="M14" s="31" t="n">
-        <x:v>0.2306120964759244</x:v>
+        <x:v>0.25685741569146714</x:v>
       </x:c>
       <x:c r="N14" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O14" s="31" t="n">
-        <x:v>0.25200545793085993</x:v>
+        <x:v>0.29210684160485556</x:v>
       </x:c>
       <x:c r="P14" s="19" t="n">
-        <x:v>22249760986909.582</x:v>
+        <x:v>23079884440650.176</x:v>
       </x:c>
       <x:c r="Q14" s="19" t="n">
-        <x:v>1328343.93951699</x:v>
+        <x:v>1377903.5486955328</x:v>
       </x:c>
       <x:c r="R14" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S14" s="18" t="n">
-        <x:v>0.007749964641289323</x:v>
+        <x:v>0.008039110552482688</x:v>
       </x:c>
       <x:c r="T14" s="16" t="str">
         <x:v>F</x:v>
@@ -1800,49 +1800,49 @@
         <x:v>observed_quarter_end</x:v>
       </x:c>
       <x:c r="E15" s="30" t="n">
-        <x:v>10534.32971</x:v>
+        <x:v>10764.32971</x:v>
       </x:c>
       <x:c r="F15" s="30" t="n">
-        <x:v>10.53432971</x:v>
+        <x:v>10.76432971</x:v>
       </x:c>
       <x:c r="G15" s="30" t="n">
-        <x:v>13559.8</x:v>
+        <x:v>13823.8</x:v>
       </x:c>
       <x:c r="H15" s="30" t="n">
-        <x:v>11223855</x:v>
+        <x:v>11015123</x:v>
       </x:c>
       <x:c r="I15" s="30" t="n">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="J15" s="30" t="n">
-        <x:v>1065455.0701356395</x:v>
+        <x:v>1023298.5514896496</x:v>
       </x:c>
       <x:c r="K15" s="31" t="n">
-        <x:v>212.5403868468818</x:v>
+        <x:v>204.13086960652006</x:v>
       </x:c>
       <x:c r="L15" s="31" t="n">
         <x:v>25.294172357627367</x:v>
       </x:c>
       <x:c r="M15" s="31" t="n">
-        <x:v>0.670123545698909</x:v>
+        <x:v>0.6484373501516276</x:v>
       </x:c>
       <x:c r="N15" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O15" s="31" t="n">
-        <x:v>0.8328482478612571</x:v>
+        <x:v>0.786602812376163</x:v>
       </x:c>
       <x:c r="P15" s="19" t="n">
-        <x:v>63949716325635.53</x:v>
+        <x:v>65345954639776.57</x:v>
       </x:c>
       <x:c r="Q15" s="19" t="n">
-        <x:v>3817893.5119782407</x:v>
+        <x:v>3901251.023270243</x:v>
       </x:c>
       <x:c r="R15" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S15" s="18" t="n">
-        <x:v>0.022274757946197436</x:v>
+        <x:v>0.022761091150934904</x:v>
       </x:c>
       <x:c r="T15" s="16" t="str">
         <x:v>F</x:v>
@@ -1865,55 +1865,55 @@
         <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-09-03</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
         <x:v>observed_qtd</x:v>
       </x:c>
       <x:c r="E16" s="30" t="n">
-        <x:v>11879.32971</x:v>
+        <x:v>12109.32971</x:v>
       </x:c>
       <x:c r="F16" s="30" t="n">
-        <x:v>11.87932971</x:v>
+        <x:v>12.10932971</x:v>
       </x:c>
       <x:c r="G16" s="30" t="n">
-        <x:v>15229.8</x:v>
+        <x:v>15493.8</x:v>
       </x:c>
       <x:c r="H16" s="30" t="n">
-        <x:v>13524006</x:v>
+        <x:v>13046294</x:v>
       </x:c>
       <x:c r="I16" s="30" t="n">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="J16" s="30" t="n">
-        <x:v>1138448.5766579502</x:v>
+        <x:v>1077375.4049512951</x:v>
       </x:c>
       <x:c r="K16" s="31" t="n">
-        <x:v>227.10136510717322</x:v>
+        <x:v>214.91829338098017</x:v>
       </x:c>
       <x:c r="L16" s="31" t="n">
         <x:v>45.688453485748845</x:v>
       </x:c>
       <x:c r="M16" s="31" t="n">
-        <x:v>0.1733549148332778</x:v>
+        <x:v>0.1698605231463417</x:v>
       </x:c>
       <x:c r="N16" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O16" s="31" t="n">
-        <x:v>0.26895428526377074</x:v>
+        <x:v>0.24415444039374634</x:v>
       </x:c>
       <x:c r="P16" s="19" t="n">
-        <x:v>130259568695330.25</x:v>
+        <x:v>132781571327743.56</x:v>
       </x:c>
       <x:c r="Q16" s="19" t="n">
-        <x:v>7776690.668377926</x:v>
+        <x:v>7927257.989716033</x:v>
       </x:c>
       <x:c r="R16" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S16" s="18" t="n">
-        <x:v>0.045371590830676344</x:v>
+        <x:v>0.046250046614445935</x:v>
       </x:c>
       <x:c r="T16" s="16" t="str">
         <x:v>F</x:v>
@@ -1942,49 +1942,49 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E17" s="30" t="n">
-        <x:v>14026.32971</x:v>
+        <x:v>14424.32971</x:v>
       </x:c>
       <x:c r="F17" s="30" t="n">
-        <x:v>14.02632971</x:v>
+        <x:v>14.42432971</x:v>
       </x:c>
       <x:c r="G17" s="30" t="n">
-        <x:v>18051.3</x:v>
+        <x:v>18559.3</x:v>
       </x:c>
       <x:c r="H17" s="30" t="n">
-        <x:v>17399770</x:v>
+        <x:v>16993413</x:v>
       </x:c>
       <x:c r="I17" s="30" t="n">
-        <x:v>64</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="J17" s="30" t="n">
-        <x:v>1240507.6994300885</x:v>
+        <x:v>1178107.6376962545</x:v>
       </x:c>
       <x:c r="K17" s="31" t="n">
-        <x:v>247.46044550695223</x:v>
+        <x:v>235.01268151208947</x:v>
       </x:c>
       <x:c r="L17" s="31" t="n">
         <x:v>82.52631287577897</x:v>
       </x:c>
       <x:c r="M17" s="31" t="n">
-        <x:v>0.23968411173075843</x:v>
+        <x:v>0.25238526977715825</x:v>
       </x:c>
       <x:c r="N17" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O17" s="31" t="n">
-        <x:v>0.36354567443740393</x:v>
+        <x:v>0.3813355908123839</x:v>
       </x:c>
       <x:c r="P17" s="19" t="n">
-        <x:v>277809905795110.62</x:v>
+        <x:v>285692819201005.06</x:v>
       </x:c>
       <x:c r="Q17" s="19" t="n">
-        <x:v>16585666.017618544</x:v>
+        <x:v>17056287.71349284</x:v>
       </x:c>
       <x:c r="R17" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S17" s="18" t="n">
-        <x:v>0.09676584607712103</x:v>
+        <x:v>0.09951159692819626</x:v>
       </x:c>
       <x:c r="T17" s="16" t="str">
         <x:v>F</x:v>
@@ -2013,49 +2013,49 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E18" s="30" t="n">
-        <x:v>16045.32971</x:v>
+        <x:v>16615.32971</x:v>
       </x:c>
       <x:c r="F18" s="30" t="n">
-        <x:v>16.04532971</x:v>
+        <x:v>16.61532971</x:v>
       </x:c>
       <x:c r="G18" s="30" t="n">
-        <x:v>20792.8</x:v>
+        <x:v>21507.8</x:v>
       </x:c>
       <x:c r="H18" s="30" t="n">
-        <x:v>20368064</x:v>
+        <x:v>20356475</x:v>
       </x:c>
       <x:c r="I18" s="30" t="n">
-        <x:v>65</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J18" s="30" t="n">
-        <x:v>1269407.6325091608</x:v>
+        <x:v>1225162.2661299568</x:v>
       </x:c>
       <x:c r="K18" s="31" t="n">
-        <x:v>253.22549663735143</x:v>
+        <x:v>244.3992893668554</x:v>
       </x:c>
       <x:c r="L18" s="31" t="n">
         <x:v>149.06594111344396</x:v>
       </x:c>
       <x:c r="M18" s="31" t="n">
-        <x:v>0.1940158891305166</x:v>
+        <x:v>0.20401064250457246</x:v>
       </x:c>
       <x:c r="N18" s="31" t="n">
         <x:v>0.8530245754425181</x:v>
       </x:c>
       <x:c r="O18" s="31" t="n">
-        <x:v>0.227240621716696</x:v>
+        <x:v>0.2605121246687574</x:v>
       </x:c>
       <x:c r="P18" s="19" t="n">
-        <x:v>574034921687196.8</x:v>
+        <x:v>594427142431515.9</x:v>
       </x:c>
       <x:c r="Q18" s="19" t="n">
-        <x:v>34270741.59326548</x:v>
+        <x:v>35488187.60785169</x:v>
       </x:c>
       <x:c r="R18" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S18" s="18" t="n">
-        <x:v>0.19994598362465274</x:v>
+        <x:v>0.20704893586844628</x:v>
       </x:c>
       <x:c r="T18" s="16" t="str">
         <x:v>F</x:v>
@@ -2084,49 +2084,49 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E19" s="30" t="n">
-        <x:v>16634.32971</x:v>
+        <x:v>17243.32971</x:v>
       </x:c>
       <x:c r="F19" s="30" t="n">
-        <x:v>16.634329710000003</x:v>
+        <x:v>17.24332971</x:v>
       </x:c>
       <x:c r="G19" s="30" t="n">
-        <x:v>21589.8</x:v>
+        <x:v>22360.8</x:v>
       </x:c>
       <x:c r="H19" s="30" t="n">
-        <x:v>21439292</x:v>
+        <x:v>21333752</x:v>
       </x:c>
       <x:c r="I19" s="30" t="n">
-        <x:v>65</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J19" s="30" t="n">
-        <x:v>1288858.1850768183</x:v>
+        <x:v>1237217.6580041742</x:v>
       </x:c>
       <x:c r="K19" s="31" t="n">
-        <x:v>257.10555510531594</x:v>
+        <x:v>246.80413751517827</x:v>
       </x:c>
       <x:c r="L19" s="31" t="n">
         <x:v>269.25539292521074</x:v>
       </x:c>
       <x:c r="M19" s="31" t="n">
-        <x:v>0.052010297783469106</x:v>
+        <x:v>0.05352346591293333</x:v>
       </x:c>
       <x:c r="N19" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O19" s="31" t="n">
-        <x:v>0.07394840621576648</x:v>
+        <x:v>0.0676499561946251</x:v>
       </x:c>
       <x:c r="P19" s="19" t="n">
-        <x:v>1074931915707253.8</x:v>
+        <x:v>1114286283937202.4</x:v>
       </x:c>
       <x:c r="Q19" s="19" t="n">
-        <x:v>64175039.74371664</x:v>
+        <x:v>66524554.264907606</x:v>
       </x:c>
       <x:c r="R19" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S19" s="18" t="n">
-        <x:v>0.3744168013052313</x:v>
+        <x:v>0.388124587309846</x:v>
       </x:c>
       <x:c r="T19" s="16" t="str">
         <x:v>F</x:v>
@@ -2155,49 +2155,49 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E20" s="30" t="n">
-        <x:v>17451.32971</x:v>
+        <x:v>18358.32971</x:v>
       </x:c>
       <x:c r="F20" s="30" t="n">
-        <x:v>17.451329710000003</x:v>
+        <x:v>18.358329710000003</x:v>
       </x:c>
       <x:c r="G20" s="30" t="n">
-        <x:v>22700.2</x:v>
+        <x:v>23828.2</x:v>
       </x:c>
       <x:c r="H20" s="30" t="n">
-        <x:v>23242366</x:v>
+        <x:v>23808883</x:v>
       </x:c>
       <x:c r="I20" s="30" t="n">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J20" s="30" t="n">
-        <x:v>1331839.257307803</x:v>
+        <x:v>1296898.1043537427</x:v>
       </x:c>
       <x:c r="K20" s="31" t="n">
-        <x:v>265.67955693338394</x:v>
+        <x:v>258.70938393041854</x:v>
       </x:c>
       <x:c r="L20" s="31" t="n">
         <x:v>486.3516513415762</x:v>
       </x:c>
       <x:c r="M20" s="31" t="n">
-        <x:v>0.06917323410675813</x:v>
+        <x:v>0.09039641679658939</x:v>
       </x:c>
       <x:c r="N20" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O20" s="31" t="n">
-        <x:v>0.11649967427711161</x:v>
+        <x:v>0.15836222077526685</x:v>
       </x:c>
       <x:c r="P20" s="19" t="n">
-        <x:v>2036995925415554.5</x:v>
+        <x:v>2142864952879589</x:v>
       </x:c>
       <x:c r="Q20" s="19" t="n">
-        <x:v>121611697.0397346</x:v>
+        <x:v>127932235.99281128</x:v>
       </x:c>
       <x:c r="R20" s="19" t="n">
         <x:v>171400000</x:v>
       </x:c>
       <x:c r="S20" s="18" t="n">
-        <x:v>0.7095198193683465</x:v>
+        <x:v>0.7463957759207193</x:v>
       </x:c>
       <x:c r="T20" s="16" t="str">
         <x:v>C</x:v>
@@ -2226,43 +2226,43 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E21" s="30" t="n">
-        <x:v>19777.32971</x:v>
+        <x:v>20684.32971</x:v>
       </x:c>
       <x:c r="F21" s="30" t="n">
-        <x:v>19.77732971</x:v>
+        <x:v>20.68432971</x:v>
       </x:c>
       <x:c r="G21" s="30" t="n">
-        <x:v>25804.3</x:v>
+        <x:v>26932.3</x:v>
       </x:c>
       <x:c r="H21" s="30" t="n">
-        <x:v>30057691</x:v>
+        <x:v>30517082</x:v>
       </x:c>
       <x:c r="I21" s="30" t="n">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J21" s="30" t="n">
-        <x:v>1519805.3246188208</x:v>
+        <x:v>1475372.0535235077</x:v>
       </x:c>
       <x:c r="K21" s="31" t="n">
-        <x:v>303.17562953200115</x:v>
+        <x:v>294.31193842744057</x:v>
       </x:c>
       <x:c r="L21" s="31" t="n">
         <x:v>878.489103571566</x:v>
       </x:c>
       <x:c r="M21" s="31" t="n">
-        <x:v>0.18051068258604275</x:v>
+        <x:v>0.17210340233638277</x:v>
       </x:c>
       <x:c r="N21" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O21" s="31" t="n">
-        <x:v>0.37097724915453156</x:v>
+        <x:v>0.3581170825391524</x:v>
       </x:c>
       <x:c r="P21" s="19" t="n">
-        <x:v>4169800475514528</x:v>
+        <x:v>4361029983579986</x:v>
       </x:c>
       <x:c r="Q21" s="19" t="n">
-        <x:v>248943311.9710166</x:v>
+        <x:v>260359999.01970065</x:v>
       </x:c>
       <x:c r="R21" s="19" t="n">
         <x:v>171400000</x:v>
@@ -2297,43 +2297,43 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E22" s="30" t="n">
-        <x:v>23626.32971</x:v>
+        <x:v>24705.32971</x:v>
       </x:c>
       <x:c r="F22" s="30" t="n">
-        <x:v>23.62632971</x:v>
+        <x:v>24.70532971</x:v>
       </x:c>
       <x:c r="G22" s="30" t="n">
-        <x:v>30729.3</x:v>
+        <x:v>32064.3</x:v>
       </x:c>
       <x:c r="H22" s="30" t="n">
-        <x:v>37048243</x:v>
+        <x:v>38104906</x:v>
       </x:c>
       <x:c r="I22" s="30" t="n">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J22" s="30" t="n">
-        <x:v>1568091.3393974642</x:v>
+        <x:v>1542375.9345569971</x:v>
       </x:c>
       <x:c r="K22" s="31" t="n">
-        <x:v>312.80787827529224</x:v>
+        <x:v>307.67808702842035</x:v>
       </x:c>
       <x:c r="L22" s="31" t="n">
         <x:v>1586.800626594274</x:v>
       </x:c>
       <x:c r="M22" s="31" t="n">
-        <x:v>0.25654787787862965</x:v>
+        <x:v>0.25628410289321923</x:v>
       </x:c>
       <x:c r="N22" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O22" s="31" t="n">
-        <x:v>0.3016709376392015</x:v>
+        <x:v>0.320359736093625</x:v>
       </x:c>
       <x:c r="P22" s="19" t="n">
-        <x:v>8997665949108219</x:v>
+        <x:v>9408583839371074</x:v>
       </x:c>
       <x:c r="Q22" s="19" t="n">
-        <x:v>537174086.5139235</x:v>
+        <x:v>561706497.8728999</x:v>
       </x:c>
       <x:c r="R22" s="19" t="n">
         <x:v>171400000</x:v>
@@ -2368,43 +2368,43 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E23" s="30" t="n">
-        <x:v>26122.32971</x:v>
+        <x:v>26684.32971</x:v>
       </x:c>
       <x:c r="F23" s="30" t="n">
-        <x:v>26.122329710000002</x:v>
+        <x:v>26.68432971</x:v>
       </x:c>
       <x:c r="G23" s="30" t="n">
-        <x:v>33779.3</x:v>
+        <x:v>34493.3</x:v>
       </x:c>
       <x:c r="H23" s="30" t="n">
-        <x:v>46037632</x:v>
+        <x:v>43728959</x:v>
       </x:c>
       <x:c r="I23" s="30" t="n">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J23" s="30" t="n">
-        <x:v>1762386.1466833923</x:v>
+        <x:v>1638750.5129503964</x:v>
       </x:c>
       <x:c r="K23" s="31" t="n">
-        <x:v>351.5664281760725</x:v>
+        <x:v>326.9031963249865</x:v>
       </x:c>
       <x:c r="L23" s="31" t="n">
         <x:v>2866.2122481919423</x:v>
       </x:c>
       <x:c r="M23" s="31" t="n">
-        <x:v>0.1448880411016562</x:v>
+        <x:v>0.11117046268898356</x:v>
       </x:c>
       <x:c r="N23" s="31" t="n">
         <x:v>0.8530245754425181</x:v>
       </x:c>
       <x:c r="O23" s="31" t="n">
-        <x:v>0.3134085038100096</x:v>
+        <x:v>0.19861224800051858</x:v>
       </x:c>
       <x:c r="P23" s="19" t="n">
-        <x:v>17969313927866468</x:v>
+        <x:v>18355908635902596</x:v>
       </x:c>
       <x:c r="Q23" s="19" t="n">
-        <x:v>1072794861.3651623</x:v>
+        <x:v>1095875142.441946</x:v>
       </x:c>
       <x:c r="R23" s="19" t="n">
         <x:v>171400000</x:v>
@@ -2439,43 +2439,43 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E24" s="30" t="n">
-        <x:v>26757.32971</x:v>
+        <x:v>27319.32971</x:v>
       </x:c>
       <x:c r="F24" s="30" t="n">
-        <x:v>26.75732971</x:v>
+        <x:v>27.31932971</x:v>
       </x:c>
       <x:c r="G24" s="30" t="n">
-        <x:v>34541.3</x:v>
+        <x:v>35255.3</x:v>
       </x:c>
       <x:c r="H24" s="30" t="n">
-        <x:v>47106859</x:v>
+        <x:v>44704704</x:v>
       </x:c>
       <x:c r="I24" s="30" t="n">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J24" s="30" t="n">
-        <x:v>1760521.6780056637</x:v>
+        <x:v>1636376.3121038887</x:v>
       </x:c>
       <x:c r="K24" s="31" t="n">
-        <x:v>351.19449799793944</x:v>
+        <x:v>326.4295831426824</x:v>
       </x:c>
       <x:c r="L24" s="31" t="n">
         <x:v>5177.192719741742</x:v>
       </x:c>
       <x:c r="M24" s="31" t="n">
-        <x:v>0.034650578303203616</x:v>
+        <x:v>0.03392931461551374</x:v>
       </x:c>
       <x:c r="N24" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O24" s="31" t="n">
-        <x:v>0.03312351026722382</x:v>
+        <x:v>0.03183764087566132</x:v>
       </x:c>
       <x:c r="P24" s="19" t="n">
-        <x:v>33246684617841944</x:v>
+        <x:v>33944984371880710</x:v>
       </x:c>
       <x:c r="Q24" s="19" t="n">
-        <x:v>1984876693.602504</x:v>
+        <x:v>2026566231.1570575</x:v>
       </x:c>
       <x:c r="R24" s="19" t="n">
         <x:v>171400000</x:v>
@@ -2510,43 +2510,43 @@
         <x:v>projected</x:v>
       </x:c>
       <x:c r="E25" s="30" t="n">
-        <x:v>31674.32971</x:v>
+        <x:v>32236.32971</x:v>
       </x:c>
       <x:c r="F25" s="30" t="n">
-        <x:v>31.674329710000002</x:v>
+        <x:v>32.23632971</x:v>
       </x:c>
       <x:c r="G25" s="30" t="n">
-        <x:v>41462.3</x:v>
+        <x:v>42176.3</x:v>
       </x:c>
       <x:c r="H25" s="30" t="n">
-        <x:v>61887051</x:v>
+        <x:v>59484896</x:v>
       </x:c>
       <x:c r="I25" s="30" t="n">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="J25" s="30" t="n">
-        <x:v>1953855.111272061</x:v>
+        <x:v>1845275.0835820881</x:v>
       </x:c>
       <x:c r="K25" s="31" t="n">
-        <x:v>389.7612699329068</x:v>
+        <x:v>368.1013785532224</x:v>
       </x:c>
       <x:c r="L25" s="31" t="n">
         <x:v>9351.47928219723</x:v>
       </x:c>
       <x:c r="M25" s="31" t="n">
-        <x:v>0.2433799423435694</x:v>
+        <x:v>0.23876540715879813</x:v>
       </x:c>
       <x:c r="N25" s="31" t="n">
         <x:v>0.853024575442511</x:v>
       </x:c>
       <x:c r="O25" s="31" t="n">
-        <x:v>0.39370043833106294</x:v>
+        <x:v>0.41209675032399673</x:v>
       </x:c>
       <x:c r="P25" s="19" t="n">
-        <x:v>71088441134531810</x:v>
+        <x:v>72349768660114580</x:v>
       </x:c>
       <x:c r="Q25" s="19" t="n">
-        <x:v>4244086037.882496</x:v>
+        <x:v>4319389173.738184</x:v>
       </x:c>
       <x:c r="R25" s="19" t="n">
         <x:v>171400000</x:v>
@@ -2573,9 +2573,9 @@
     <x:mergeCell ref="A3:W3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3172ccc6127f4651"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb50b13147c944b4"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931900e3c7814986"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bc8d2cb74c3413b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2816,7 +2816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ed5c3933ec246fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R859095cce6a34854"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3157,7 +3157,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R428613e4ff71468d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe20e8b42b534539"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3289,27 +3289,27 @@
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="8" ht="54" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>Google Pryor (North)</x:v>
+        <x:v>Anthropic-Amazon New Carlisle</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C8" s="30" t="n">
-        <x:v>763011.622031329</x:v>
+        <x:v>685912.076806468</x:v>
       </x:c>
       <x:c r="D8" s="30" t="n">
-        <x:v>368</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>Google #confident</x:v>
+        <x:v>Amazon #confident</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
+        <x:v>Anthropic #confident</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>4581 Webb St, Pryor, OK 74361</x:v>
+        <x:v>55001 Larrison Blvd, New Carlisle, IN 46552</x:v>
       </x:c>
       <x:c r="H8" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -3317,51 +3317,51 @@
     </x:row>
     <x:row r="9" ht="54" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
-        <x:v>Anthropic-Amazon New Carlisle</x:v>
+        <x:v>Meta Prometheus</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C9" s="30" t="n">
-        <x:v>685912.076806468</x:v>
+        <x:v>679568.3173319859</x:v>
       </x:c>
       <x:c r="D9" s="30" t="n">
-        <x:v>910</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>Amazon #confident</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>Anthropic #confident</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
-        <x:v>55001 Larrison Blvd, New Carlisle, IN 46552</x:v>
+        <x:v>1 Community Cir, New Albany, OH 43054</x:v>
       </x:c>
       <x:c r="H9" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="54" hidden="0" customHeight="1">
+    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>Meta Prometheus</x:v>
+        <x:v>Google Pryor (North)</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C10" s="30" t="n">
-        <x:v>677109.6513390602</x:v>
+        <x:v>636685.1945426983</x:v>
       </x:c>
       <x:c r="D10" s="30" t="n">
-        <x:v>562</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google DeepMind #speculative</x:v>
       </x:c>
       <x:c r="G10" s="16" t="str">
-        <x:v>1 Community Cir, New Albany, OH 43054</x:v>
+        <x:v>4581 Webb St, Pryor, OK 74361</x:v>
       </x:c>
       <x:c r="H10" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -3375,7 +3375,7 @@
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C11" s="30" t="n">
-        <x:v>616472.9661445174</x:v>
+        <x:v>550783.2238504295</x:v>
       </x:c>
       <x:c r="D11" s="30" t="n">
         <x:v>453</x:v>
@@ -3453,7 +3453,7 @@
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C14" s="30" t="n">
-        <x:v>408792.3193532087</x:v>
+        <x:v>331985.85144012125</x:v>
       </x:c>
       <x:c r="D14" s="30" t="n">
         <x:v>303</x:v>
@@ -3479,7 +3479,7 @@
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C15" s="30" t="n">
-        <x:v>343102.57705912075</x:v>
+        <x:v>289540.17180394137</x:v>
       </x:c>
       <x:c r="D15" s="30" t="n">
         <x:v>183</x:v>
@@ -3493,51 +3493,47 @@
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="54" hidden="0" customHeight="1">
+    <x:row r="16" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="str">
-        <x:v>Google Council Bluffs (East)</x:v>
+        <x:v>DayOne Nusajaya</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>United States</x:v>
+        <x:v>Malaysia</x:v>
       </x:c>
       <x:c r="C16" s="30" t="n">
-        <x:v>289034.86609398684</x:v>
+        <x:v>281670.4396159676</x:v>
       </x:c>
       <x:c r="D16" s="30" t="n">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E16" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
-      <x:c r="F16" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
-      </x:c>
-      <x:c r="G16" s="16" t="str">
-        <x:v>10410 Bunge Ave, Council Bluffs, IA 51503</x:v>
-      </x:c>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="E16" s="16" t="str"/>
+      <x:c r="F16" s="16" t="str"/>
+      <x:c r="G16" s="16" t="str"/>
       <x:c r="H16" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="17" ht="54" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:v>Google Lincoln</x:v>
+        <x:v>Colossus 1</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C17" s="30" t="n">
-        <x:v>287518.9489641233</x:v>
+        <x:v>275795.85649317835</x:v>
       </x:c>
       <x:c r="D17" s="30" t="n">
-        <x:v>141</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
-      <x:c r="F17" s="16" t="str"/>
+        <x:v>SpaceXAI #confident</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="str">
+        <x:v>Anthropic #confident</x:v>
+      </x:c>
       <x:c r="G17" s="16" t="str">
-        <x:v>5475 Cloud Ct, Lincoln, NE 68514</x:v>
+        <x:v>3231 Riverport Rd, Memphis, TN 38109</x:v>
       </x:c>
       <x:c r="H17" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -3545,181 +3541,191 @@
     </x:row>
     <x:row r="18" ht="54" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="str">
-        <x:v>Google Bristow</x:v>
+        <x:v>Google Council Bluffs (East)</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C18" s="30" t="n">
-        <x:v>283675.08842849924</x:v>
+        <x:v>255684.68923698837</x:v>
       </x:c>
       <x:c r="D18" s="30" t="n">
-        <x:v>279</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
-        <x:v>Google</x:v>
+        <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F18" s="16" t="str">
-        <x:v>Google DeepMind</x:v>
+        <x:v>Google DeepMind #speculative</x:v>
       </x:c>
       <x:c r="G18" s="16" t="str">
-        <x:v>13001 Rollins Ford Road, Bristow, VA 20136</x:v>
+        <x:v>10410 Bunge Ave, Council Bluffs, IA 51503</x:v>
       </x:c>
       <x:c r="H18" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="19" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A19" s="16" t="str">
-        <x:v>DayOne Nusajaya</x:v>
+        <x:v>CoreWeave Denton TX</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
-        <x:v>Malaysia</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="C19" s="30" t="n">
-        <x:v>281670.4396159676</x:v>
+        <x:v>252652.85497726125</x:v>
       </x:c>
       <x:c r="D19" s="30" t="n">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="E19" s="16" t="str"/>
-      <x:c r="F19" s="16" t="str"/>
-      <x:c r="G19" s="16" t="str"/>
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="E19" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F19" s="16" t="str">
+        <x:v>OpenAI #likely</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str">
+        <x:v>8171 Jim Christal Rd, Denton, TX 76207</x:v>
+      </x:c>
       <x:c r="H19" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" hidden="0" customHeight="1">
       <x:c r="A20" s="16" t="str">
-        <x:v>Colossus 1</x:v>
+        <x:v>QTS Richmond 1</x:v>
       </x:c>
       <x:c r="B20" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C20" s="30" t="n">
-        <x:v>275795.85649317835</x:v>
+        <x:v>242546.7407781708</x:v>
       </x:c>
       <x:c r="D20" s="30" t="n">
-        <x:v>340</x:v>
-      </x:c>
-      <x:c r="E20" s="16" t="str">
-        <x:v>SpaceXAI #confident</x:v>
-      </x:c>
-      <x:c r="F20" s="16" t="str">
-        <x:v>Anthropic #confident</x:v>
-      </x:c>
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E20" s="16" t="str"/>
+      <x:c r="F20" s="16" t="str"/>
       <x:c r="G20" s="16" t="str">
-        <x:v>3231 Riverport Rd, Memphis, TN 38109</x:v>
+        <x:v>6000 Technology Blvd, Sandston, VA 23150</x:v>
       </x:c>
       <x:c r="H20" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="21" ht="54" hidden="0" customHeight="1">
       <x:c r="A21" s="16" t="str">
-        <x:v>Google Omaha</x:v>
+        <x:v>Meta Rosemount</x:v>
       </x:c>
       <x:c r="B21" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C21" s="30" t="n">
-        <x:v>267812.02627589693</x:v>
+        <x:v>215675.08842849924</x:v>
       </x:c>
       <x:c r="D21" s="30" t="n">
-        <x:v>237</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E21" s="16" t="str">
-        <x:v>Google #confident</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="G21" s="16" t="str">
-        <x:v>11110 State St, Omaha, NE 68142</x:v>
+        <x:v>1772-2396 145th St, Rosemount, MN 55068, USA</x:v>
       </x:c>
       <x:c r="H21" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="22" ht="129.60000610351562" hidden="0" customHeight="1">
       <x:c r="A22" s="16" t="str">
-        <x:v>CoreWeave Denton TX</x:v>
+        <x:v>Amazon Madison Mega Site</x:v>
       </x:c>
       <x:c r="B22" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C22" s="30" t="n">
-        <x:v>252652.85497726125</x:v>
+        <x:v>214348.14354550533</x:v>
       </x:c>
       <x:c r="D22" s="30" t="n">
-        <x:v>262</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>CoreWeave #confident</x:v>
+        <x:v>Amazon #confident</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
-        <x:v>OpenAI #likely</x:v>
+        <x:v>Anthropic #speculative</x:v>
       </x:c>
       <x:c r="G22" s="16" t="str">
-        <x:v>8171 Jim Christal Rd, Denton, TX 76207</x:v>
+        <x:v>Amazon Data Services Inc, Madison Mega Site Nissan Parkway and Highway 22 Canton, Mississippi Madison County</x:v>
       </x:c>
       <x:c r="H22" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="23" ht="54" hidden="0" customHeight="1">
       <x:c r="A23" s="16" t="str">
-        <x:v>Google Kansas City East</x:v>
+        <x:v>Google Bristow</x:v>
       </x:c>
       <x:c r="B23" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C23" s="30" t="n">
-        <x:v>244567.9636179889</x:v>
+        <x:v>209860.53562405254</x:v>
       </x:c>
       <x:c r="D23" s="30" t="n">
-        <x:v>105</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="E23" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
-      <x:c r="F23" s="16" t="str"/>
-      <x:c r="G23" s="16" t="str"/>
+        <x:v>Google</x:v>
+      </x:c>
+      <x:c r="F23" s="16" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="G23" s="16" t="str">
+        <x:v>13001 Rollins Ford Road, Bristow, VA 20136</x:v>
+      </x:c>
       <x:c r="H23" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" hidden="0" customHeight="1">
       <x:c r="A24" s="16" t="str">
-        <x:v>QTS Richmond 1</x:v>
+        <x:v>Microsoft Goodyear</x:v>
       </x:c>
       <x:c r="B24" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C24" s="30" t="n">
-        <x:v>242546.7407781708</x:v>
+        <x:v>205154.11824153614</x:v>
       </x:c>
       <x:c r="D24" s="30" t="n">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="E24" s="16" t="str"/>
-      <x:c r="F24" s="16" t="str"/>
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="E24" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F24" s="16" t="str">
+        <x:v>OpenAI #likely, Microsoft #confident</x:v>
+      </x:c>
       <x:c r="G24" s="16" t="str">
-        <x:v>6000 Technology Blvd, Sandston, VA 23150</x:v>
+        <x:v>14250 W Broadway Rd, Goodyear, AZ 85338</x:v>
       </x:c>
       <x:c r="H24" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="54" hidden="0" customHeight="1">
+    <x:row r="25" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A25" s="16" t="str">
-        <x:v>Meta Rosemount</x:v>
+        <x:v>Meta Jeffersonville</x:v>
       </x:c>
       <x:c r="B25" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C25" s="30" t="n">
-        <x:v>215765.5381505811</x:v>
+        <x:v>203132.89540171804</x:v>
       </x:c>
       <x:c r="D25" s="30" t="n">
         <x:v>178</x:v>
@@ -3731,85 +3737,79 @@
         <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="G25" s="16" t="str">
-        <x:v>1772-2396 145th St, Rosemount, MN 55068, USA</x:v>
+        <x:v>500 8th St, Jeffersonville, IN 47130, USA</x:v>
       </x:c>
       <x:c r="H25" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="129.60000610351562" hidden="0" customHeight="1">
+    <x:row r="26" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A26" s="16" t="str">
-        <x:v>Amazon Madison Mega Site</x:v>
+        <x:v>Google Kansas City East</x:v>
       </x:c>
       <x:c r="B26" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C26" s="30" t="n">
-        <x:v>214348.14354550533</x:v>
+        <x:v>202627.5896917635</x:v>
       </x:c>
       <x:c r="D26" s="30" t="n">
-        <x:v>284</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F26" s="16" t="str"/>
+      <x:c r="G26" s="16" t="str"/>
+      <x:c r="H26" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A27" s="16" t="str">
+        <x:v>AWS New Albany</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="n">
+        <x:v>201111.67256189996</x:v>
+      </x:c>
+      <x:c r="D27" s="30" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
         <x:v>Amazon #confident</x:v>
       </x:c>
-      <x:c r="F26" s="16" t="str">
-        <x:v>Anthropic #speculative</x:v>
-      </x:c>
-      <x:c r="G26" s="16" t="str">
-        <x:v>Amazon Data Services Inc, Madison Mega Site Nissan Parkway and Highway 22 Canton, Mississippi Madison County</x:v>
-      </x:c>
-      <x:c r="H26" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="54" hidden="0" customHeight="1">
-      <x:c r="A27" s="16" t="str">
-        <x:v>Microsoft Goodyear</x:v>
-      </x:c>
-      <x:c r="B27" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C27" s="30" t="n">
-        <x:v>205154.11824153614</x:v>
-      </x:c>
-      <x:c r="D27" s="30" t="n">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="E27" s="16" t="str">
-        <x:v>Microsoft #confident</x:v>
-      </x:c>
-      <x:c r="F27" s="16" t="str">
-        <x:v>OpenAI #likely, Microsoft #confident</x:v>
-      </x:c>
+      <x:c r="F27" s="16" t="str"/>
       <x:c r="G27" s="16" t="str">
-        <x:v>14250 W Broadway Rd, Goodyear, AZ 85338</x:v>
+        <x:v>13360 Miller Rd NW</x:v>
       </x:c>
       <x:c r="H27" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="28" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A28" s="16" t="str">
-        <x:v>Meta Jeffersonville</x:v>
+        <x:v>Google Omaha</x:v>
       </x:c>
       <x:c r="B28" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C28" s="30" t="n">
-        <x:v>203132.89540171804</x:v>
+        <x:v>198585.14401212733</x:v>
       </x:c>
       <x:c r="D28" s="30" t="n">
-        <x:v>178</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E28" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F28" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google DeepMind #speculative</x:v>
       </x:c>
       <x:c r="G28" s="16" t="str">
-        <x:v>500 8th St, Jeffersonville, IN 47130, USA</x:v>
+        <x:v>11110 State St, Omaha, NE 68142</x:v>
       </x:c>
       <x:c r="H28" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -3817,23 +3817,23 @@
     </x:row>
     <x:row r="29" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A29" s="16" t="str">
-        <x:v>Google The Dalles</x:v>
+        <x:v>Google Lincoln</x:v>
       </x:c>
       <x:c r="B29" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C29" s="30" t="n">
-        <x:v>201616.97827185446</x:v>
+        <x:v>197574.53259221828</x:v>
       </x:c>
       <x:c r="D29" s="30" t="n">
-        <x:v>154</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E29" s="16" t="str">
         <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F29" s="16" t="str"/>
       <x:c r="G29" s="16" t="str">
-        <x:v>3500 River Rd, The Dalles, OR</x:v>
+        <x:v>5475 Cloud Ct, Lincoln, NE 68514</x:v>
       </x:c>
       <x:c r="H29" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -3841,45 +3841,45 @@
     </x:row>
     <x:row r="30" ht="54" hidden="0" customHeight="1">
       <x:c r="A30" s="16" t="str">
-        <x:v>Google Midlothian</x:v>
+        <x:v>QTS Richmond 2</x:v>
       </x:c>
       <x:c r="B30" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C30" s="30" t="n">
-        <x:v>191005.5583628095</x:v>
+        <x:v>182920.66700353715</x:v>
       </x:c>
       <x:c r="D30" s="30" t="n">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="E30" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E30" s="16" t="str"/>
       <x:c r="F30" s="16" t="str"/>
       <x:c r="G30" s="16" t="str">
-        <x:v>3250 Railport Parkway, Midlothian, TX 76065</x:v>
+        <x:v>6030–6070 Technology Blvd, Sandston, VA 23150</x:v>
       </x:c>
       <x:c r="H30" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="54" hidden="0" customHeight="1">
+    <x:row r="31" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A31" s="16" t="str">
-        <x:v>QTS Richmond 2</x:v>
+        <x:v>Google The Dalles</x:v>
       </x:c>
       <x:c r="B31" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C31" s="30" t="n">
-        <x:v>182920.66700353715</x:v>
+        <x:v>175341.0813542193</x:v>
       </x:c>
       <x:c r="D31" s="30" t="n">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="E31" s="16" t="str"/>
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E31" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
       <x:c r="F31" s="16" t="str"/>
       <x:c r="G31" s="16" t="str">
-        <x:v>6030–6070 Technology Blvd, Sandston, VA 23150</x:v>
+        <x:v>3500 River Rd, The Dalles, OR</x:v>
       </x:c>
       <x:c r="H31" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -4117,100 +4117,100 @@
     </x:row>
     <x:row r="41" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A41" s="16" t="str">
-        <x:v>Google Arcola</x:v>
+        <x:v>Microsoft Project Osmium</x:v>
       </x:c>
       <x:c r="B41" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C41" s="30" t="n">
-        <x:v>157150.07579585648</x:v>
+        <x:v>155634.15866599293</x:v>
       </x:c>
       <x:c r="D41" s="30" t="n">
-        <x:v>77</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="E41" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
-      <x:c r="F41" s="16" t="str"/>
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F41" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
       <x:c r="G41" s="16" t="str">
-        <x:v>42575 Arcola Blvd, Sterling, VA 20166</x:v>
+        <x:v>5855 SW Kerry St, Cumming, IA 50061</x:v>
       </x:c>
       <x:c r="H41" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="42" ht="54" hidden="0" customHeight="1">
       <x:c r="A42" s="16" t="str">
-        <x:v>Microsoft Project Osmium</x:v>
+        <x:v>Meta Eagle Mountain</x:v>
       </x:c>
       <x:c r="B42" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C42" s="30" t="n">
-        <x:v>155634.15866599293</x:v>
+        <x:v>151354.21930267813</x:v>
       </x:c>
       <x:c r="D42" s="30" t="n">
-        <x:v>190</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E42" s="16" t="str">
-        <x:v>Microsoft #confident</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="F42" s="16" t="str">
-        <x:v>OpenAI #speculative</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="G42" s="16" t="str">
-        <x:v>5855 SW Kerry St, Cumming, IA 50061</x:v>
+        <x:v>1275 N Community Cir, Eagle Mountain, UT 84005</x:v>
       </x:c>
       <x:c r="H42" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="43" ht="54" hidden="0" customHeight="1">
       <x:c r="A43" s="16" t="str">
-        <x:v>Google Storey County</x:v>
+        <x:v>Google Midlothian</x:v>
       </x:c>
       <x:c r="B43" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C43" s="30" t="n">
-        <x:v>153612.93582617483</x:v>
+        <x:v>143506.8216270844</x:v>
       </x:c>
       <x:c r="D43" s="30" t="n">
-        <x:v>161</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E43" s="16" t="str">
         <x:v>Google #confident</x:v>
       </x:c>
-      <x:c r="F43" s="16" t="str">
+      <x:c r="F43" s="16" t="str"/>
+      <x:c r="G43" s="16" t="str">
+        <x:v>3250 Railport Parkway, Midlothian, TX 76065</x:v>
+      </x:c>
+      <x:c r="H43" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A44" s="16" t="str">
+        <x:v>Google Storey County</x:v>
+      </x:c>
+      <x:c r="B44" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C44" s="30" t="n">
+        <x:v>133906.01313794847</x:v>
+      </x:c>
+      <x:c r="D44" s="30" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="E44" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F44" s="16" t="str">
         <x:v>Google DeepMind #speculative</x:v>
       </x:c>
-      <x:c r="G43" s="16" t="str"/>
-      <x:c r="H43" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="54" hidden="0" customHeight="1">
-      <x:c r="A44" s="16" t="str">
-        <x:v>Meta Eagle Mountain</x:v>
-      </x:c>
-      <x:c r="B44" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C44" s="30" t="n">
-        <x:v>151354.21930267813</x:v>
-      </x:c>
-      <x:c r="D44" s="30" t="n">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="E44" s="16" t="str">
-        <x:v>Meta #confident</x:v>
-      </x:c>
-      <x:c r="F44" s="16" t="str">
-        <x:v>Meta #confident</x:v>
-      </x:c>
-      <x:c r="G44" s="16" t="str">
-        <x:v>1275 N Community Cir, Eagle Mountain, UT 84005</x:v>
-      </x:c>
+      <x:c r="G44" s="16" t="str"/>
       <x:c r="H44" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
@@ -4343,7 +4343,7 @@
     </x:row>
     <x:row r="50" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A50" s="16" t="str">
-        <x:v>Google Red Oak</x:v>
+        <x:v>Google Arcola</x:v>
       </x:c>
       <x:c r="B50" s="16" t="str">
         <x:v>United States</x:v>
@@ -4359,102 +4359,100 @@
       </x:c>
       <x:c r="F50" s="16" t="str"/>
       <x:c r="G50" s="16" t="str">
+        <x:v>42575 Arcola Blvd, Sterling, VA 20166</x:v>
+      </x:c>
+      <x:c r="H50" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A51" s="16" t="str">
+        <x:v>Google Red Oak</x:v>
+      </x:c>
+      <x:c r="B51" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C51" s="30" t="n">
+        <x:v>108135.42193026781</x:v>
+      </x:c>
+      <x:c r="D51" s="30" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E51" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F51" s="16" t="str"/>
+      <x:c r="G51" s="16" t="str">
         <x:v>330 Austin Blvd, Red Oak, TX 75154</x:v>
       </x:c>
-      <x:c r="H50" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A51" s="16" t="str">
+      <x:c r="H51" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="64.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A52" s="16" t="str">
+        <x:v>Google Papillion</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C52" s="30" t="n">
+        <x:v>100555.83628094998</x:v>
+      </x:c>
+      <x:c r="D52" s="30" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E52" s="16" t="str">
+        <x:v>Google #confident</x:v>
+      </x:c>
+      <x:c r="F52" s="16" t="str">
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G52" s="16" t="str">
+        <x:v>14651-15249 Gold Coast Rd 68138 Papillion Nebraska, USA</x:v>
+      </x:c>
+      <x:c r="H52" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A53" s="16" t="str">
         <x:v>Meta Gallatin</x:v>
       </x:c>
-      <x:c r="B51" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C51" s="30" t="n">
+      <x:c r="B53" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C53" s="30" t="n">
         <x:v>99545.22486104093</x:v>
       </x:c>
-      <x:c r="D51" s="30" t="n">
+      <x:c r="D53" s="30" t="n">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="E51" s="16" t="str">
+      <x:c r="E53" s="16" t="str">
         <x:v>Meta #confident</x:v>
       </x:c>
-      <x:c r="F51" s="16" t="str">
+      <x:c r="F53" s="16" t="str">
         <x:v>Meta #confident</x:v>
       </x:c>
-      <x:c r="G51" s="16" t="str">
+      <x:c r="G53" s="16" t="str">
         <x:v>1 Meta Lp, Gallatin, TN 37066</x:v>
       </x:c>
-      <x:c r="H51" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="54" hidden="0" customHeight="1">
-      <x:c r="A52" s="16" t="str">
+      <x:c r="H53" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="54" hidden="0" customHeight="1">
+      <x:c r="A54" s="16" t="str">
         <x:v>Meta Los Lunas</x:v>
       </x:c>
-      <x:c r="B52" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C52" s="30" t="n">
+      <x:c r="B54" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C54" s="30" t="n">
         <x:v>99545.22486104093</x:v>
       </x:c>
-      <x:c r="D52" s="30" t="n">
+      <x:c r="D54" s="30" t="n">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="E52" s="16" t="str">
-        <x:v>Meta #confident</x:v>
-      </x:c>
-      <x:c r="F52" s="16" t="str">
-        <x:v>Meta #confident</x:v>
-      </x:c>
-      <x:c r="G52" s="16" t="str">
-        <x:v>4250 Messenger Lp, Los Lunas, NM 87031</x:v>
-      </x:c>
-      <x:c r="H52" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A53" s="16" t="str">
-        <x:v>CoreWeave Ellendale ND</x:v>
-      </x:c>
-      <x:c r="B53" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C53" s="30" t="n">
-        <x:v>93481.55634158666</x:v>
-      </x:c>
-      <x:c r="D53" s="30" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="E53" s="16" t="str">
-        <x:v>CoreWeave #confident</x:v>
-      </x:c>
-      <x:c r="F53" s="16" t="str">
-        <x:v>OpenAI #speculative</x:v>
-      </x:c>
-      <x:c r="G53" s="16" t="str">
-        <x:v>9685 87th Ave SE, Ellendale, ND 58436</x:v>
-      </x:c>
-      <x:c r="H53" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="64.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A54" s="16" t="str">
-        <x:v>Meta Sarpy</x:v>
-      </x:c>
-      <x:c r="B54" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C54" s="30" t="n">
-        <x:v>91965.63921172309</x:v>
-      </x:c>
-      <x:c r="D54" s="30" t="n">
-        <x:v>80</x:v>
       </x:c>
       <x:c r="E54" s="16" t="str">
         <x:v>Meta #confident</x:v>
@@ -4463,24 +4461,24 @@
         <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="G54" s="16" t="str">
-        <x:v>14436-14998 Fairview Rd, Springfield, NE 68059, USA</x:v>
+        <x:v>4250 Messenger Lp, Los Lunas, NM 87031</x:v>
       </x:c>
       <x:c r="H54" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="54" hidden="0" customHeight="1">
+    <x:row r="55" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A55" s="16" t="str">
-        <x:v>CoreWeave Chester VA</x:v>
+        <x:v>CoreWeave Ellendale ND</x:v>
       </x:c>
       <x:c r="B55" s="16" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C55" s="30" t="n">
-        <x:v>88428.49924204143</x:v>
+        <x:v>93481.55634158666</x:v>
       </x:c>
       <x:c r="D55" s="30" t="n">
-        <x:v>82</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E55" s="16" t="str">
         <x:v>CoreWeave #confident</x:v>
@@ -4489,321 +4487,327 @@
         <x:v>OpenAI #speculative</x:v>
       </x:c>
       <x:c r="G55" s="16" t="str">
-        <x:v>1401 Meadowville Technology Parkway, Chester, VA</x:v>
+        <x:v>9685 87th Ave SE, Ellendale, ND 58436</x:v>
       </x:c>
       <x:c r="H55" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="56" ht="64.80000305175781" hidden="0" customHeight="1">
       <x:c r="A56" s="16" t="str">
-        <x:v>Oracle Batam</x:v>
+        <x:v>Meta Sarpy</x:v>
       </x:c>
       <x:c r="B56" s="16" t="str">
-        <x:v>Indonesia</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="C56" s="30" t="n">
-        <x:v>84386.05356240526</x:v>
+        <x:v>91965.63921172309</x:v>
       </x:c>
       <x:c r="D56" s="30" t="n">
-        <x:v>72</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E56" s="16" t="str">
-        <x:v>Oracle #likely</x:v>
-      </x:c>
-      <x:c r="F56" s="16" t="str"/>
-      <x:c r="G56" s="16" t="str"/>
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="F56" s="16" t="str">
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G56" s="16" t="str">
+        <x:v>14436-14998 Fairview Rd, Springfield, NE 68059, USA</x:v>
+      </x:c>
       <x:c r="H56" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" hidden="0" customHeight="1">
       <x:c r="A57" s="16" t="str">
+        <x:v>CoreWeave Chester VA</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C57" s="30" t="n">
+        <x:v>88428.49924204143</x:v>
+      </x:c>
+      <x:c r="D57" s="30" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E57" s="16" t="str">
+        <x:v>CoreWeave #confident</x:v>
+      </x:c>
+      <x:c r="F57" s="16" t="str">
+        <x:v>OpenAI #speculative</x:v>
+      </x:c>
+      <x:c r="G57" s="16" t="str">
+        <x:v>1401 Meadowville Technology Parkway, Chester, VA</x:v>
+      </x:c>
+      <x:c r="H57" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A58" s="16" t="str">
+        <x:v>Oracle Batam</x:v>
+      </x:c>
+      <x:c r="B58" s="16" t="str">
+        <x:v>Indonesia</x:v>
+      </x:c>
+      <x:c r="C58" s="30" t="n">
+        <x:v>84386.05356240526</x:v>
+      </x:c>
+      <x:c r="D58" s="30" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E58" s="16" t="str">
+        <x:v>Oracle #likely</x:v>
+      </x:c>
+      <x:c r="F58" s="16" t="str"/>
+      <x:c r="G58" s="16" t="str"/>
+      <x:c r="H58" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="54" hidden="0" customHeight="1">
+      <x:c r="A59" s="16" t="str">
         <x:v>AWS Berwick</x:v>
       </x:c>
-      <x:c r="B57" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C57" s="30" t="n">
+      <x:c r="B59" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C59" s="30" t="n">
         <x:v>81354.21930267812</x:v>
       </x:c>
-      <x:c r="D57" s="30" t="n">
+      <x:c r="D59" s="30" t="n">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="E57" s="16" t="str">
+      <x:c r="E59" s="16" t="str">
         <x:v>Amazon #confident</x:v>
       </x:c>
-      <x:c r="F57" s="16" t="str">
+      <x:c r="F59" s="16" t="str">
         <x:v>Anthropic #speculative</x:v>
       </x:c>
-      <x:c r="G57" s="16" t="str">
+      <x:c r="G59" s="16" t="str">
         <x:v>1125 Electron Ave, Berwick, PA 18603</x:v>
       </x:c>
-      <x:c r="H57" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="64.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A58" s="16" t="str">
-        <x:v>Google Papillion</x:v>
-      </x:c>
-      <x:c r="B58" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C58" s="30" t="n">
-        <x:v>80343.60788276908</x:v>
-      </x:c>
-      <x:c r="D58" s="30" t="n">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E58" s="16" t="str">
-        <x:v>Google #confident</x:v>
-      </x:c>
-      <x:c r="F58" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
-      </x:c>
-      <x:c r="G58" s="16" t="str">
-        <x:v>14651-15249 Gold Coast Rd 68138 Papillion Nebraska, USA</x:v>
-      </x:c>
-      <x:c r="H58" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A59" s="16" t="str">
+      <x:c r="H59" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A60" s="16" t="str">
         <x:v>CoreWeave Marble NC</x:v>
       </x:c>
-      <x:c r="B59" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C59" s="30" t="n">
+      <x:c r="B60" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C60" s="30" t="n">
         <x:v>78827.6907529055</x:v>
       </x:c>
-      <x:c r="D59" s="30" t="n">
+      <x:c r="D60" s="30" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="E59" s="16" t="str">
+      <x:c r="E60" s="16" t="str">
         <x:v>CoreWeave #confident</x:v>
       </x:c>
-      <x:c r="F59" s="16" t="str">
+      <x:c r="F60" s="16" t="str">
         <x:v>OpenAI #speculative</x:v>
       </x:c>
-      <x:c r="G59" s="16" t="str">
+      <x:c r="G60" s="16" t="str">
         <x:v>155 Palmer Ln, Marble, NC 28905</x:v>
       </x:c>
-      <x:c r="H59" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="54" hidden="0" customHeight="1">
-      <x:c r="A60" s="16" t="str">
+      <x:c r="H60" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A61" s="16" t="str">
+        <x:v>Core42 Lake Mariner</x:v>
+      </x:c>
+      <x:c r="B61" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C61" s="30" t="n">
+        <x:v>71753.4108135422</x:v>
+      </x:c>
+      <x:c r="D61" s="30" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E61" s="16" t="str">
+        <x:v>Core42 #confident</x:v>
+      </x:c>
+      <x:c r="F61" s="16" t="str">
+        <x:v>G42 #likely</x:v>
+      </x:c>
+      <x:c r="G61" s="16" t="str">
+        <x:v>7725 Lake Rd, Barker, NY 14012</x:v>
+      </x:c>
+      <x:c r="H61" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="54" hidden="0" customHeight="1">
+      <x:c r="A62" s="16" t="str">
         <x:v>Microsoft SAT40</x:v>
       </x:c>
-      <x:c r="B60" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C60" s="30" t="n">
+      <x:c r="B62" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C62" s="30" t="n">
         <x:v>64679.13087417888</x:v>
       </x:c>
-      <x:c r="D60" s="30" t="n">
+      <x:c r="D62" s="30" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="E60" s="16" t="str">
+      <x:c r="E62" s="16" t="str">
         <x:v>Microsoft #confident</x:v>
       </x:c>
-      <x:c r="F60" s="16" t="str"/>
-      <x:c r="G60" s="16" t="str">
+      <x:c r="F62" s="16" t="str"/>
+      <x:c r="G62" s="16" t="str">
         <x:v>15000 Lambda Drive, San Antonio, TX 78245</x:v>
       </x:c>
-      <x:c r="H60" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="54" hidden="0" customHeight="1">
-      <x:c r="A61" s="16" t="str">
+      <x:c r="H62" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="54" hidden="0" customHeight="1">
+      <x:c r="A63" s="16" t="str">
         <x:v>STACK Infrastructure NVA02</x:v>
       </x:c>
-      <x:c r="B61" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C61" s="30" t="n">
+      <x:c r="B63" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C63" s="30" t="n">
         <x:v>61141.99090449722</x:v>
       </x:c>
-      <x:c r="D61" s="30" t="n">
+      <x:c r="D63" s="30" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="E61" s="16" t="str"/>
-      <x:c r="F61" s="16" t="str"/>
-      <x:c r="G61" s="16" t="str">
+      <x:c r="E63" s="16" t="str"/>
+      <x:c r="F63" s="16" t="str"/>
+      <x:c r="G63" s="16" t="str">
         <x:v>9590 Hornbaker Rd, Manassas, VA 20109</x:v>
       </x:c>
-      <x:c r="H61" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A62" s="16" t="str">
+      <x:c r="H63" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A64" s="16" t="str">
         <x:v>Anthropic Lake Mariner</x:v>
       </x:c>
-      <x:c r="B62" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C62" s="30" t="n">
+      <x:c r="B64" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C64" s="30" t="n">
         <x:v>58564.93178372915</x:v>
-      </x:c>
-      <x:c r="D62" s="30" t="n">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E62" s="16" t="str">
-        <x:v>AI XPV Platform #confident</x:v>
-      </x:c>
-      <x:c r="F62" s="16" t="str">
-        <x:v>Anthropic #likely</x:v>
-      </x:c>
-      <x:c r="G62" s="16" t="str">
-        <x:v>7725 Lake Rd, Barker, NY 14012</x:v>
-      </x:c>
-      <x:c r="H62" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A63" s="16" t="str">
-        <x:v>Microsoft-Nebius New Jersey</x:v>
-      </x:c>
-      <x:c r="B63" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C63" s="30" t="n">
-        <x:v>56846.89236988378</x:v>
-      </x:c>
-      <x:c r="D63" s="30" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E63" s="16" t="str">
-        <x:v>Nebius #confident</x:v>
-      </x:c>
-      <x:c r="F63" s="16" t="str">
-        <x:v>Microsoft #likely</x:v>
-      </x:c>
-      <x:c r="G63" s="16" t="str">
-        <x:v>3963 S Lincoln Ave, Vineland, New Jersey</x:v>
-      </x:c>
-      <x:c r="H63" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A64" s="16" t="str">
-        <x:v>CoreWeave Norway</x:v>
-      </x:c>
-      <x:c r="B64" s="16" t="str">
-        <x:v>Norway</x:v>
-      </x:c>
-      <x:c r="C64" s="30" t="n">
-        <x:v>50773.11773623042</x:v>
       </x:c>
       <x:c r="D64" s="30" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="E64" s="16" t="str">
+        <x:v>AI XPV Platform #confident</x:v>
+      </x:c>
+      <x:c r="F64" s="16" t="str">
+        <x:v>Anthropic #likely</x:v>
+      </x:c>
+      <x:c r="G64" s="16" t="str">
+        <x:v>7725 Lake Rd, Barker, NY 14012</x:v>
+      </x:c>
+      <x:c r="H64" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A65" s="16" t="str">
+        <x:v>Microsoft-Nebius New Jersey</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C65" s="30" t="n">
+        <x:v>56846.89236988378</x:v>
+      </x:c>
+      <x:c r="D65" s="30" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E65" s="16" t="str">
+        <x:v>Nebius #confident</x:v>
+      </x:c>
+      <x:c r="F65" s="16" t="str">
+        <x:v>Microsoft #likely</x:v>
+      </x:c>
+      <x:c r="G65" s="16" t="str">
+        <x:v>3963 S Lincoln Ave, Vineland, New Jersey</x:v>
+      </x:c>
+      <x:c r="H65" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A66" s="16" t="str">
+        <x:v>CoreWeave Norway</x:v>
+      </x:c>
+      <x:c r="B66" s="16" t="str">
+        <x:v>Norway</x:v>
+      </x:c>
+      <x:c r="C66" s="30" t="n">
+        <x:v>50773.11773623042</x:v>
+      </x:c>
+      <x:c r="D66" s="30" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E66" s="16" t="str">
         <x:v>CoreWeave #confident</x:v>
       </x:c>
-      <x:c r="F64" s="16" t="str">
+      <x:c r="F66" s="16" t="str">
         <x:v>OpenAI #speculative</x:v>
       </x:c>
-      <x:c r="G64" s="16" t="str">
+      <x:c r="G66" s="16" t="str">
         <x:v>Stølevegen 39, 4715 Øvrebø, Norway</x:v>
       </x:c>
-      <x:c r="H64" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A65" s="16" t="str">
+      <x:c r="H66" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A67" s="16" t="str">
         <x:v>Southgate Melbourne</x:v>
       </x:c>
-      <x:c r="B65" s="16" t="str">
+      <x:c r="B67" s="16" t="str">
         <x:v>Australia</x:v>
       </x:c>
-      <x:c r="C65" s="30" t="n">
+      <x:c r="C67" s="30" t="n">
         <x:v>46488.12531581607</x:v>
       </x:c>
-      <x:c r="D65" s="30" t="n">
+      <x:c r="D67" s="30" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="E65" s="16" t="str">
+      <x:c r="E67" s="16" t="str">
         <x:v>Firmus #confident</x:v>
       </x:c>
-      <x:c r="F65" s="16" t="str"/>
-      <x:c r="G65" s="16" t="str"/>
-      <x:c r="H65" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A66" s="16" t="str">
+      <x:c r="F67" s="16" t="str"/>
+      <x:c r="G67" s="16" t="str"/>
+      <x:c r="H67" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A68" s="16" t="str">
         <x:v>Stream Phoenix</x:v>
       </x:c>
-      <x:c r="B66" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C66" s="30" t="n">
+      <x:c r="B68" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C68" s="30" t="n">
         <x:v>46134.4113188479</x:v>
       </x:c>
-      <x:c r="D66" s="30" t="n">
+      <x:c r="D68" s="30" t="n">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="E66" s="16" t="str"/>
-      <x:c r="F66" s="16" t="str"/>
-      <x:c r="G66" s="16" t="str">
-        <x:v>2950 S. Litchfield Road</x:v>
-      </x:c>
-      <x:c r="H66" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="54" hidden="0" customHeight="1">
-      <x:c r="A67" s="16" t="str">
-        <x:v>Microsoft SAT14</x:v>
-      </x:c>
-      <x:c r="B67" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C67" s="30" t="n">
-        <x:v>45174.33046993431</x:v>
-      </x:c>
-      <x:c r="D67" s="30" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E67" s="16" t="str">
-        <x:v>Microsoft #confident</x:v>
-      </x:c>
-      <x:c r="F67" s="16" t="str"/>
-      <x:c r="G67" s="16" t="str">
-        <x:v>3545 Wiseman Boulevard, San Antonio, TX 78251</x:v>
-      </x:c>
-      <x:c r="H67" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A68" s="16" t="str">
-        <x:v>Vantage TX1</x:v>
-      </x:c>
-      <x:c r="B68" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C68" s="30" t="n">
-        <x:v>38706.417382516425</x:v>
-      </x:c>
-      <x:c r="D68" s="30" t="n">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="E68" s="16" t="str"/>
       <x:c r="F68" s="16" t="str"/>
       <x:c r="G68" s="16" t="str">
-        <x:v>14720 Omicron Dr, San Antonio, TX 78245</x:v>
+        <x:v>2950 S. Litchfield Road</x:v>
       </x:c>
       <x:c r="H68" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -4811,155 +4815,149 @@
     </x:row>
     <x:row r="69" ht="54" hidden="0" customHeight="1">
       <x:c r="A69" s="16" t="str">
+        <x:v>Microsoft SAT14</x:v>
+      </x:c>
+      <x:c r="B69" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C69" s="30" t="n">
+        <x:v>45174.33046993431</x:v>
+      </x:c>
+      <x:c r="D69" s="30" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="E69" s="16" t="str">
+        <x:v>Microsoft #confident</x:v>
+      </x:c>
+      <x:c r="F69" s="16" t="str"/>
+      <x:c r="G69" s="16" t="str">
+        <x:v>3545 Wiseman Boulevard, San Antonio, TX 78251</x:v>
+      </x:c>
+      <x:c r="H69" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A70" s="16" t="str">
+        <x:v>Vantage TX1</x:v>
+      </x:c>
+      <x:c r="B70" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C70" s="30" t="n">
+        <x:v>38706.417382516425</x:v>
+      </x:c>
+      <x:c r="D70" s="30" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E70" s="16" t="str"/>
+      <x:c r="F70" s="16" t="str"/>
+      <x:c r="G70" s="16" t="str">
+        <x:v>14720 Omicron Dr, San Antonio, TX 78245</x:v>
+      </x:c>
+      <x:c r="H70" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="54" hidden="0" customHeight="1">
+      <x:c r="A71" s="16" t="str">
         <x:v>CoreWeave Dalton 1 &amp; 2</x:v>
       </x:c>
-      <x:c r="B69" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C69" s="30" t="n">
+      <x:c r="B71" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C71" s="30" t="n">
         <x:v>32238.504295098533</x:v>
       </x:c>
-      <x:c r="D69" s="30" t="n">
+      <x:c r="D71" s="30" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="E69" s="16" t="str">
+      <x:c r="E71" s="16" t="str">
         <x:v>CoreWeave #confident</x:v>
       </x:c>
-      <x:c r="F69" s="16" t="str">
+      <x:c r="F71" s="16" t="str">
         <x:v>OpenAI #speculative</x:v>
       </x:c>
-      <x:c r="G69" s="16" t="str">
+      <x:c r="G71" s="16" t="str">
         <x:v>2205 Industrial South Rd, Dalton, GA, 30721</x:v>
       </x:c>
-      <x:c r="H69" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="118.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A70" s="16" t="str">
+      <x:c r="H71" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A72" s="16" t="str">
         <x:v>Alibaba Zhangbei</x:v>
       </x:c>
-      <x:c r="B70" s="16" t="str">
+      <x:c r="B72" s="16" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="C70" s="30" t="n">
+      <x:c r="C72" s="30" t="n">
         <x:v>31884.79029813037</x:v>
       </x:c>
-      <x:c r="D70" s="30" t="n">
+      <x:c r="D72" s="30" t="n">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="E70" s="16" t="str">
+      <x:c r="E72" s="16" t="str">
         <x:v>Alibaba #confident</x:v>
       </x:c>
-      <x:c r="F70" s="16" t="str">
+      <x:c r="F72" s="16" t="str">
         <x:v>Alibaba #likely</x:v>
       </x:c>
-      <x:c r="G70" s="16" t="str">
+      <x:c r="G72" s="16" t="str">
         <x:v>Alibaba Zhangbei Yun Calculation Data Center, Zhangbei County, Zhangjiakou, Hebei, China, 076471</x:v>
       </x:c>
-      <x:c r="H70" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A71" s="16" t="str">
+      <x:c r="H72" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="75.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A73" s="16" t="str">
         <x:v>Start Campus Sines Data Campus</x:v>
       </x:c>
-      <x:c r="B71" s="16" t="str">
+      <x:c r="B73" s="16" t="str">
         <x:v>Portugal</x:v>
       </x:c>
-      <x:c r="C71" s="30" t="n">
+      <x:c r="C73" s="30" t="n">
         <x:v>31834.259727134915</x:v>
       </x:c>
-      <x:c r="D71" s="30" t="n">
+      <x:c r="D73" s="30" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="E71" s="16" t="str">
+      <x:c r="E73" s="16" t="str">
         <x:v>Nscale #confident</x:v>
       </x:c>
-      <x:c r="F71" s="16" t="str">
+      <x:c r="F73" s="16" t="str">
         <x:v>Microsoft #confident</x:v>
       </x:c>
-      <x:c r="G71" s="16" t="str">
+      <x:c r="G73" s="16" t="str">
         <x:v>Start Campus - Sustainable Data Center Services, Sines, Portugal</x:v>
       </x:c>
-      <x:c r="H71" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="54" hidden="0" customHeight="1">
-      <x:c r="A72" s="16" t="str">
+      <x:c r="H73" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="54" hidden="0" customHeight="1">
+      <x:c r="A74" s="16" t="str">
         <x:v>xAI QTS Atlanta</x:v>
       </x:c>
-      <x:c r="B72" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C72" s="30" t="n">
+      <x:c r="B74" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C74" s="30" t="n">
         <x:v>11470.43961596766</x:v>
       </x:c>
-      <x:c r="D72" s="30" t="n">
+      <x:c r="D74" s="30" t="n">
         <x:v>17.32971</x:v>
       </x:c>
-      <x:c r="E72" s="16" t="str">
+      <x:c r="E74" s="16" t="str">
         <x:v>SpaceXAI #confident</x:v>
       </x:c>
-      <x:c r="F72" s="16" t="str">
+      <x:c r="F74" s="16" t="str">
         <x:v>SpaceXAI #confident</x:v>
       </x:c>
-      <x:c r="G72" s="16" t="str">
+      <x:c r="G74" s="16" t="str">
         <x:v>1025 Jefferson Street NW, Atlanta, GA 30318</x:v>
-      </x:c>
-      <x:c r="H72" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="54" hidden="0" customHeight="1">
-      <x:c r="A73" s="16" t="str">
-        <x:v>CoreWeave Muskogee OK</x:v>
-      </x:c>
-      <x:c r="B73" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C73" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D73" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E73" s="16" t="str">
-        <x:v>CoreWeave #confident</x:v>
-      </x:c>
-      <x:c r="F73" s="16" t="str">
-        <x:v>OpenAI #speculative</x:v>
-      </x:c>
-      <x:c r="G73" s="16" t="str">
-        <x:v>1525 W 43rd St S, Muskogee, OK 74401, USA</x:v>
-      </x:c>
-      <x:c r="H73" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A74" s="16" t="str">
-        <x:v>Crusoe Abilene Expansion</x:v>
-      </x:c>
-      <x:c r="B74" s="16" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="C74" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D74" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E74" s="16" t="str">
-        <x:v>Microsoft #confident</x:v>
-      </x:c>
-      <x:c r="F74" s="16" t="str">
-        <x:v>Microsoft #likely</x:v>
-      </x:c>
-      <x:c r="G74" s="16" t="str">
-        <x:v>5502 Spinks Rd, Abilene, TX 79601</x:v>
       </x:c>
       <x:c r="H74" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -4967,7 +4965,7 @@
     </x:row>
     <x:row r="75" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A75" s="16" t="str">
-        <x:v>Goodnight</x:v>
+        <x:v>Anthropic Barber Lake</x:v>
       </x:c>
       <x:c r="B75" s="16" t="str">
         <x:v>United States</x:v>
@@ -4979,21 +4977,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E75" s="16" t="str">
-        <x:v>Google #speculative</x:v>
+        <x:v>Cipher Mining #confident</x:v>
       </x:c>
       <x:c r="F75" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
-      </x:c>
-      <x:c r="G75" s="16" t="str">
-        <x:v>10001 Lima Rd, Claude, TX 79019</x:v>
-      </x:c>
+        <x:v>Anthropic #confident</x:v>
+      </x:c>
+      <x:c r="G75" s="16" t="str"/>
       <x:c r="H75" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="64.80000305175781" hidden="0" customHeight="1">
+    <x:row r="76" ht="54" hidden="0" customHeight="1">
       <x:c r="A76" s="16" t="str">
-        <x:v>Google Cedar Rapids</x:v>
+        <x:v>CoreWeave Muskogee OK</x:v>
       </x:c>
       <x:c r="B76" s="16" t="str">
         <x:v>United States</x:v>
@@ -5005,21 +5001,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E76" s="16" t="str">
-        <x:v>Google #confident</x:v>
+        <x:v>CoreWeave #confident</x:v>
       </x:c>
       <x:c r="F76" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
+        <x:v>OpenAI #speculative</x:v>
       </x:c>
       <x:c r="G76" s="16" t="str">
-        <x:v>5800 EDGEWOOD RD SW CEDAR RAPIDS, IA 52404</x:v>
+        <x:v>1525 W 43rd St S, Muskogee, OK 74401, USA</x:v>
       </x:c>
       <x:c r="H76" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="77" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A77" s="16" t="str">
-        <x:v>Google Fort Wayne</x:v>
+        <x:v>Crusoe Abilene Expansion</x:v>
       </x:c>
       <x:c r="B77" s="16" t="str">
         <x:v>United States</x:v>
@@ -5031,13 +5027,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E77" s="16" t="str">
-        <x:v>Google #confident</x:v>
+        <x:v>Microsoft #confident</x:v>
       </x:c>
       <x:c r="F77" s="16" t="str">
-        <x:v>Google DeepMind #speculative</x:v>
+        <x:v>Microsoft #likely</x:v>
       </x:c>
       <x:c r="G77" s="16" t="str">
-        <x:v>6015 Adams Center Road, Fort Wayne, IN 46806</x:v>
+        <x:v>5502 Spinks Rd, Abilene, TX 79601</x:v>
       </x:c>
       <x:c r="H77" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -5045,7 +5041,7 @@
     </x:row>
     <x:row r="78" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A78" s="16" t="str">
-        <x:v>Meta Hyperion</x:v>
+        <x:v>Goodnight</x:v>
       </x:c>
       <x:c r="B78" s="16" t="str">
         <x:v>United States</x:v>
@@ -5057,24 +5053,24 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E78" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google #speculative</x:v>
       </x:c>
       <x:c r="F78" s="16" t="str">
-        <x:v>Meta #confident</x:v>
+        <x:v>Google DeepMind #speculative</x:v>
       </x:c>
       <x:c r="G78" s="16" t="str">
-        <x:v>Holly Ridge, LA 71269</x:v>
+        <x:v>10001 Lima Rd, Claude, TX 79019</x:v>
       </x:c>
       <x:c r="H78" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="79" ht="64.80000305175781" hidden="0" customHeight="1">
       <x:c r="A79" s="16" t="str">
-        <x:v>Microsoft Narvik Norway</x:v>
+        <x:v>Google Cedar Rapids</x:v>
       </x:c>
       <x:c r="B79" s="16" t="str">
-        <x:v>Norway</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="C79" s="30" t="n">
         <x:v>0</x:v>
@@ -5083,19 +5079,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E79" s="16" t="str">
-        <x:v>Nscale #likely</x:v>
+        <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F79" s="16" t="str">
-        <x:v>Microsoft #likely</x:v>
-      </x:c>
-      <x:c r="G79" s="16" t="str"/>
+        <x:v>Google DeepMind #speculative</x:v>
+      </x:c>
+      <x:c r="G79" s="16" t="str">
+        <x:v>5800 EDGEWOOD RD SW CEDAR RAPIDS, IA 52404</x:v>
+      </x:c>
       <x:c r="H79" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A80" s="16" t="str">
-        <x:v>OpenAI Stargate Lordstown</x:v>
+        <x:v>Google Fort Wayne</x:v>
       </x:c>
       <x:c r="B80" s="16" t="str">
         <x:v>United States</x:v>
@@ -5107,13 +5105,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E80" s="16" t="str">
-        <x:v>Softbank #confident</x:v>
+        <x:v>Google #confident</x:v>
       </x:c>
       <x:c r="F80" s="16" t="str">
-        <x:v>OpenAI #confident</x:v>
+        <x:v>Google DeepMind #speculative</x:v>
       </x:c>
       <x:c r="G80" s="16" t="str">
-        <x:v>2300 Hallock Young Rd, Warren, OH 44481</x:v>
+        <x:v>6015 Adams Center Road, Fort Wayne, IN 46806</x:v>
       </x:c>
       <x:c r="H80" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
@@ -5121,7 +5119,7 @@
     </x:row>
     <x:row r="81" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A81" s="16" t="str">
-        <x:v>OpenAI Stargate Michigan</x:v>
+        <x:v>Meta Hyperion</x:v>
       </x:c>
       <x:c r="B81" s="16" t="str">
         <x:v>United States</x:v>
@@ -5133,22 +5131,24 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E81" s="16" t="str">
-        <x:v>Oracle #confident</x:v>
+        <x:v>Meta #confident</x:v>
       </x:c>
       <x:c r="F81" s="16" t="str">
-        <x:v>OpenAI #confident</x:v>
-      </x:c>
-      <x:c r="G81" s="16" t="str"/>
+        <x:v>Meta #confident</x:v>
+      </x:c>
+      <x:c r="G81" s="16" t="str">
+        <x:v>Holly Ridge, LA 71269</x:v>
+      </x:c>
       <x:c r="H81" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A82" s="16" t="str">
-        <x:v>OpenAI Stargate Milam</x:v>
+        <x:v>Microsoft Narvik Norway</x:v>
       </x:c>
       <x:c r="B82" s="16" t="str">
-        <x:v>United States</x:v>
+        <x:v>Norway</x:v>
       </x:c>
       <x:c r="C82" s="30" t="n">
         <x:v>0</x:v>
@@ -5157,19 +5157,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E82" s="16" t="str">
-        <x:v>Softbank #confident</x:v>
+        <x:v>Nscale #likely</x:v>
       </x:c>
       <x:c r="F82" s="16" t="str">
-        <x:v>OpenAI #confident</x:v>
+        <x:v>Microsoft #likely</x:v>
       </x:c>
       <x:c r="G82" s="16" t="str"/>
       <x:c r="H82" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="32.400001525878906" hidden="0" customHeight="1">
+    <x:row r="83" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A83" s="16" t="str">
-        <x:v>OpenAI Stargate New Mexico</x:v>
+        <x:v>OpenAI Stargate Lordstown</x:v>
       </x:c>
       <x:c r="B83" s="16" t="str">
         <x:v>United States</x:v>
@@ -5181,19 +5181,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E83" s="16" t="str">
-        <x:v>Oracle #confident</x:v>
+        <x:v>Softbank #confident</x:v>
       </x:c>
       <x:c r="F83" s="16" t="str">
         <x:v>OpenAI #confident</x:v>
       </x:c>
-      <x:c r="G83" s="16" t="str"/>
+      <x:c r="G83" s="16" t="str">
+        <x:v>2300 Hallock Young Rd, Warren, OH 44481</x:v>
+      </x:c>
       <x:c r="H83" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="64.80000305175781" hidden="0" customHeight="1">
+    <x:row r="84" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A84" s="16" t="str">
-        <x:v>OpenAI Stargate Shackelford</x:v>
+        <x:v>OpenAI Stargate Michigan</x:v>
       </x:c>
       <x:c r="B84" s="16" t="str">
         <x:v>United States</x:v>
@@ -5210,19 +5212,17 @@
       <x:c r="F84" s="16" t="str">
         <x:v>OpenAI #confident</x:v>
       </x:c>
-      <x:c r="G84" s="16" t="str">
-        <x:v>175 Private Road 1604, Abilene, TX 79601, Shackelford County</x:v>
-      </x:c>
+      <x:c r="G84" s="16" t="str"/>
       <x:c r="H84" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" ht="86.4000015258789" hidden="0" customHeight="1">
+    <x:row r="85" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A85" s="16" t="str">
-        <x:v>OpenAI Stargate UAE</x:v>
+        <x:v>OpenAI Stargate Milam</x:v>
       </x:c>
       <x:c r="B85" s="16" t="str">
-        <x:v>United Arab Emirates</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="C85" s="30" t="n">
         <x:v>0</x:v>
@@ -5231,21 +5231,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E85" s="16" t="str">
-        <x:v>G42 #likely</x:v>
+        <x:v>Softbank #confident</x:v>
       </x:c>
       <x:c r="F85" s="16" t="str">
         <x:v>OpenAI #confident</x:v>
       </x:c>
-      <x:c r="G85" s="16" t="str">
-        <x:v>Nexus L&amp;T Project Office, Al Bihouth, Al Dhafrah, Abu Dhabi, United Arab Emirates</x:v>
-      </x:c>
+      <x:c r="G85" s="16" t="str"/>
       <x:c r="H85" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A86" s="16" t="str">
-        <x:v>OpenAI Stargate Wisconsin</x:v>
+        <x:v>OpenAI Stargate New Mexico</x:v>
       </x:c>
       <x:c r="B86" s="16" t="str">
         <x:v>United States</x:v>
@@ -5267,9 +5265,9 @@
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="87" ht="64.80000305175781" hidden="0" customHeight="1">
       <x:c r="A87" s="16" t="str">
-        <x:v>QTS Cedar Rapids</x:v>
+        <x:v>OpenAI Stargate Shackelford</x:v>
       </x:c>
       <x:c r="B87" s="16" t="str">
         <x:v>United States</x:v>
@@ -5280,21 +5278,25 @@
       <x:c r="D87" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E87" s="16" t="str"/>
-      <x:c r="F87" s="16" t="str"/>
+      <x:c r="E87" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F87" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
       <x:c r="G87" s="16" t="str">
-        <x:v>6200 76th Ave SW, Fairfax, IA 52228</x:v>
+        <x:v>175 Private Road 1604, Abilene, TX 79601, Shackelford County</x:v>
       </x:c>
       <x:c r="H87" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="54" hidden="0" customHeight="1">
+    <x:row r="88" ht="86.4000015258789" hidden="0" customHeight="1">
       <x:c r="A88" s="16" t="str">
-        <x:v>QTS Eagle Mountain</x:v>
+        <x:v>OpenAI Stargate UAE</x:v>
       </x:c>
       <x:c r="B88" s="16" t="str">
-        <x:v>United States</x:v>
+        <x:v>United Arab Emirates</x:v>
       </x:c>
       <x:c r="C88" s="30" t="n">
         <x:v>0</x:v>
@@ -5302,14 +5304,86 @@
       <x:c r="D88" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E88" s="16" t="str"/>
+      <x:c r="E88" s="16" t="str">
+        <x:v>G42 #likely</x:v>
+      </x:c>
       <x:c r="F88" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G88" s="16" t="str">
+        <x:v>Nexus L&amp;T Project Office, Al Bihouth, Al Dhafrah, Abu Dhabi, United Arab Emirates</x:v>
+      </x:c>
+      <x:c r="H88" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="32.400001525878906" hidden="0" customHeight="1">
+      <x:c r="A89" s="16" t="str">
+        <x:v>OpenAI Stargate Wisconsin</x:v>
+      </x:c>
+      <x:c r="B89" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C89" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D89" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E89" s="16" t="str">
+        <x:v>Oracle #confident</x:v>
+      </x:c>
+      <x:c r="F89" s="16" t="str">
+        <x:v>OpenAI #confident</x:v>
+      </x:c>
+      <x:c r="G89" s="16" t="str"/>
+      <x:c r="H89" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A90" s="16" t="str">
+        <x:v>QTS Cedar Rapids</x:v>
+      </x:c>
+      <x:c r="B90" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C90" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D90" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E90" s="16" t="str"/>
+      <x:c r="F90" s="16" t="str"/>
+      <x:c r="G90" s="16" t="str">
+        <x:v>6200 76th Ave SW, Fairfax, IA 52228</x:v>
+      </x:c>
+      <x:c r="H90" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="54" hidden="0" customHeight="1">
+      <x:c r="A91" s="16" t="str">
+        <x:v>QTS Eagle Mountain</x:v>
+      </x:c>
+      <x:c r="B91" s="16" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="C91" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D91" s="30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E91" s="16" t="str"/>
+      <x:c r="F91" s="16" t="str">
         <x:v>Meta #speculative</x:v>
       </x:c>
-      <x:c r="G88" s="16" t="str">
+      <x:c r="G91" s="16" t="str">
         <x:v>652 E Hyperscale Way, Eagle Mountain, UT 84013</x:v>
       </x:c>
-      <x:c r="H88" s="16" t="str">
+      <x:c r="H91" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
     </x:row>
@@ -5320,7 +5394,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf164e0b9f0540ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dffc153ecec46d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6050,6 +6124,168 @@
         <x:v>No</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A21" s="16" t="str">
+        <x:v>epoch-aws-new-albany-added-20260828</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>AWS New Albany added to Epoch registry</x:v>
+      </x:c>
+      <x:c r="C21" s="16"/>
+      <x:c r="D21" s="16" t="str">
+        <x:v>site</x:v>
+      </x:c>
+      <x:c r="E21" s="16" t="str">
+        <x:v>U.S. AI data-center registry</x:v>
+      </x:c>
+      <x:c r="F21" s="16" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="G21" s="16" t="str">
+        <x:v>publisher-change-log</x:v>
+      </x:c>
+      <x:c r="H21" s="16" t="str">
+        <x:v>newly added</x:v>
+      </x:c>
+      <x:c r="I21" s="16" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="J21" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-updates</x:v>
+      </x:c>
+      <x:c r="K21" s="16" t="str">
+        <x:v>Epoch added AWS New Albany to its tracked data-center set after the prior cutoff.</x:v>
+      </x:c>
+      <x:c r="L21" s="16" t="str">
+        <x:v>Site inclusion can affect the reconstructed U.S. path; the direct value is taken only from Epoch's dated registry and timeline CSVs.</x:v>
+      </x:c>
+      <x:c r="M21" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A22" s="16" t="str">
+        <x:v>epoch-google-bristow-power-revision-20260828</x:v>
+      </x:c>
+      <x:c r="B22" s="16" t="str">
+        <x:v>Google Bristow revised IT power</x:v>
+      </x:c>
+      <x:c r="C22" s="16" t="n">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="D22" s="16" t="str">
+        <x:v>MW IT</x:v>
+      </x:c>
+      <x:c r="E22" s="16" t="str">
+        <x:v>Google Bristow</x:v>
+      </x:c>
+      <x:c r="F22" s="16" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="G22" s="16" t="str">
+        <x:v>publisher-change-log</x:v>
+      </x:c>
+      <x:c r="H22" s="16" t="str">
+        <x:v>revised from 279 MW</x:v>
+      </x:c>
+      <x:c r="I22" s="16" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="J22" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-updates</x:v>
+      </x:c>
+      <x:c r="K22" s="16" t="str">
+        <x:v>Epoch revised Google Bristow power downward from 279 MW to 238 MW.</x:v>
+      </x:c>
+      <x:c r="L22" s="16" t="str">
+        <x:v>Facility revision is contextual here; the gate uses the recomputed latest state at every quarter cutoff from the full timeline.</x:v>
+      </x:c>
+      <x:c r="M22" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A23" s="16" t="str">
+        <x:v>epoch-qts-eagle-mountain-b300-revision-20260901</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>QTS Eagle Mountain projected B300 chips</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="n">
+        <x:v>137300</x:v>
+      </x:c>
+      <x:c r="D23" s="16" t="str">
+        <x:v>chips</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="str">
+        <x:v>QTS Eagle Mountain</x:v>
+      </x:c>
+      <x:c r="F23" s="16" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="G23" s="16" t="str">
+        <x:v>publisher-change-log</x:v>
+      </x:c>
+      <x:c r="H23" s="16" t="str">
+        <x:v>projected; revised from 91,600</x:v>
+      </x:c>
+      <x:c r="I23" s="16" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="J23" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-updates</x:v>
+      </x:c>
+      <x:c r="K23" s="16" t="str">
+        <x:v>Epoch increased projected B300 chips at QTS Eagle Mountain from 91,600 to 137,300.</x:v>
+      </x:c>
+      <x:c r="L23" s="16" t="str">
+        <x:v>Chip counts and H100-equivalents are audit context only; they do not substitute for IT power or measured inference productivity.</x:v>
+      </x:c>
+      <x:c r="M23" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="205.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A24" s="16" t="str">
+        <x:v>cipher-on-site-generation-pipeline-20260903</x:v>
+      </x:c>
+      <x:c r="B24" s="16" t="str">
+        <x:v>Prospective on-site generation capacity</x:v>
+      </x:c>
+      <x:c r="C24" s="16" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="D24" s="16" t="str">
+        <x:v>MW generation</x:v>
+      </x:c>
+      <x:c r="E24" s="16" t="str">
+        <x:v>Multiple Cipher U.S. HPC data-center sites</x:v>
+      </x:c>
+      <x:c r="F24" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="G24" s="16" t="str">
+        <x:v>company-announcement-forward-looking</x:v>
+      </x:c>
+      <x:c r="H24" s="16" t="str">
+        <x:v>up to; targeted before end-2027</x:v>
+      </x:c>
+      <x:c r="I24" s="16" t="str">
+        <x:v>Announcement paragraphs 1-4</x:v>
+      </x:c>
+      <x:c r="J24" s="16" t="str">
+        <x:v>gate2-cipherdigital-com-bring-your-own-generation</x:v>
+      </x:c>
+      <x:c r="K24" s="16" t="str">
+        <x:v>Cipher says lateral pipelines under development could support up to 2.5 GW of on-site natural-gas generation before the end of 2027 for additional leasable HPC capacity.</x:v>
+      </x:c>
+      <x:c r="L24" s="16" t="str">
+        <x:v>Generation nameplate is not IT power, the tenant and Personal-AI allocation are unknown, and the timing is forward-looking. Excluded from the direct U.S. operational IT-power path.</x:v>
+      </x:c>
+      <x:c r="M24" s="16" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:M2"/>
@@ -6057,7 +6293,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd396e964e5154e4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75e27d83750948c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6130,165 +6366,211 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="6" ht="140.39999389648438" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
+        <x:v>gate2-cipherdigital-com-bring-your-own-generation</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>Cipher Digital Inc.</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="str">
+        <x:v>Cipher Digital Begins Development of Lateral Pipelines to Facilitate Data Center Expansion via Bring-Your-Own-Generation</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>U.S. power pipeline evidence, HPC data-center supply context</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>https://investors.cipherdigital.com/news-releases/news-release-details/cipher-digital-begins-development-lateral-pipelines-facilitate/</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>Company announcement and forward-looking statement. The 2.5 GW is generation capacity, not measured operational IT load.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A7" s="16" t="str">
         <x:v>gate2-diffuse-personal-ai-gate-2-compute-supply-calculation-contract</x:v>
       </x:c>
-      <x:c r="B6" s="16" t="str">
+      <x:c r="B7" s="16" t="str">
         <x:v>Diffuse Personal AI</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="str">
+      <x:c r="C7" s="16" t="str">
         <x:v>Gate 2 · Compute supply calculation contract</x:v>
       </x:c>
-      <x:c r="D6" s="16" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
-      <x:c r="E6" s="16" t="str">
+      <x:c r="D7" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
         <x:v>methodology, normalization, model configuration</x:v>
       </x:c>
-      <x:c r="F6" s="16" t="str">
+      <x:c r="F7" s="16" t="str">
         <x:v>https://github.com/buwilliams/diffuse-personal-ai/blob/main/intent/02-model/06-report-card-calculations.md</x:v>
       </x:c>
-      <x:c r="G6" s="16" t="str">
+      <x:c r="G7" s="16" t="str">
         <x:v>Holds definitions and assumptions that are authored by the forecast rather than fetched as observations.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="291.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A7" s="16" t="str">
+    <x:row r="8" ht="291.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A8" s="16" t="str">
         <x:v>gate2-dwarkesh-com-dylan-patel-compute-outlook</x:v>
       </x:c>
-      <x:c r="B7" s="16" t="str">
+      <x:c r="B8" s="16" t="str">
         <x:v>Dwarkesh Podcast</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="str">
+      <x:c r="C8" s="16" t="str">
         <x:v>Dylan Patel – Anthropic &amp; OpenAI will have most of the world’s compute by 2028</x:v>
       </x:c>
-      <x:c r="D7" s="16" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
-      <x:c r="E7" s="16" t="str">
+      <x:c r="D8" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str">
         <x:v>capacity outlook, allocation cross-check, supply constraint context</x:v>
       </x:c>
-      <x:c r="F7" s="16" t="str">
+      <x:c r="F8" s="16" t="str">
         <x:v>https://www.dwarkesh.com/p/dylan-patel-3</x:v>
       </x:c>
-      <x:c r="G7" s="16" t="str">
+      <x:c r="G8" s="16" t="str">
         <x:v>Expert-interview estimates from Dylan Patel of SemiAnalysis. The official transcript accompanies the video at https://www.youtube.com/watch?v=aV26V1UvkJw. Global GW flows and frontier-lab allocations are not directly merged with the U.S. H100e countdown path.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="205.1999969482422" hidden="0" customHeight="1">
-      <x:c r="A8" s="16" t="str">
+    <x:row r="9" ht="205.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A9" s="16" t="str">
         <x:v>gate2-epoch-ai-ai-data-center-timelines-csv</x:v>
-      </x:c>
-      <x:c r="B8" s="16" t="str">
-        <x:v>Epoch AI</x:v>
-      </x:c>
-      <x:c r="C8" s="16" t="str">
-        <x:v>AI Data Center Timelines CSV</x:v>
-      </x:c>
-      <x:c r="D8" s="16" t="str">
-        <x:v>2026-08-25</x:v>
-      </x:c>
-      <x:c r="E8" s="16" t="str">
-        <x:v>IT-power observation, IT-power projection, H100e productivity audit bridge</x:v>
-      </x:c>
-      <x:c r="F8" s="16" t="str">
-        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
-      </x:c>
-      <x:c r="G8" s="16" t="str">
-        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff. U.S. geography is joined from Epoch’s data-center registry.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="270" hidden="0" customHeight="1">
-      <x:c r="A9" s="16" t="str">
-        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:v>Epoch AI</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
+        <x:v>AI Data Center Timelines CSV</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>IT-power observation, IT-power projection, H100e productivity audit bridge</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>Observed quarters use the latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff. U.S. geography is joined from Epoch’s data-center registry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="270" hidden="0" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-csv</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>Epoch AI</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
         <x:v>AI Data Centers CSV</x:v>
       </x:c>
-      <x:c r="D9" s="16" t="str">
-        <x:v>2026-08-25</x:v>
-      </x:c>
-      <x:c r="E9" s="16" t="str">
+      <x:c r="D10" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str">
         <x:v>site registry, geography filter, facility audit</x:v>
       </x:c>
-      <x:c r="F9" s="16" t="str">
+      <x:c r="F10" s="16" t="str">
         <x:v>https://epoch.ai/data/data_centers/data_centers.csv</x:v>
       </x:c>
-      <x:c r="G9" s="16" t="str">
+      <x:c r="G10" s="16" t="str">
         <x:v>Country identifies the U.S. sites included in the quarterly timeline reconstruction. Current power is the registry’s current IT-power estimate and is retained as a facility-level audit field; the quarterly gate path is reconstructed from the dated timeline.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="151.1999969482422" hidden="0" customHeight="1">
-      <x:c r="A10" s="16" t="str">
+    <x:row r="11" ht="172.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>gate2-epoch-ai-ai-data-centers-updates</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>Epoch AI</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>AI Data Centers Updates</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>data-center change log, capacity revision audit, pipeline context</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>https://epoch.ai/data/ai-data-centers/updates</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>The direct gate inputs come from Epoch's September 3 registry and timeline CSVs. This source preserves the publisher's post-August-26 change log as an audit trail.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A12" s="16" t="str">
         <x:v>gate2-github-com-mlperf-inference-v5-0-power</x:v>
       </x:c>
-      <x:c r="B10" s="16" t="str">
+      <x:c r="B12" s="16" t="str">
         <x:v>MLCommons</x:v>
       </x:c>
-      <x:c r="C10" s="16" t="str">
+      <x:c r="C12" s="16" t="str">
         <x:v>MLPerf Inference v5.0 summary results</x:v>
       </x:c>
-      <x:c r="D10" s="16" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
-      <x:c r="E10" s="16" t="str">
+      <x:c r="D12" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str">
         <x:v>measured inference goodput, measured system power, productivity trend</x:v>
       </x:c>
-      <x:c r="F10" s="16" t="str">
+      <x:c r="F12" s="16" t="str">
         <x:v>https://raw.githubusercontent.com/mlcommons/inference_results_v5.0/main/summary_results.json</x:v>
       </x:c>
-      <x:c r="G10" s="16" t="str">
+      <x:c r="G12" s="16" t="str">
         <x:v>Official MLPerf result data. The selected row is an available, closed, datacenter Server result with a reported power measurement.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="162" hidden="0" customHeight="1">
-      <x:c r="A11" s="16" t="str">
+    <x:row r="13" ht="162" hidden="0" customHeight="1">
+      <x:c r="A13" s="16" t="str">
         <x:v>gate2-github-com-mlperf-inference-v5-1-power</x:v>
       </x:c>
-      <x:c r="B11" s="16" t="str">
+      <x:c r="B13" s="16" t="str">
         <x:v>MLCommons</x:v>
       </x:c>
-      <x:c r="C11" s="16" t="str">
+      <x:c r="C13" s="16" t="str">
         <x:v>MLPerf Inference v5.1 summary results</x:v>
       </x:c>
-      <x:c r="D11" s="16" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
-      <x:c r="E11" s="16" t="str">
+      <x:c r="D13" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str">
         <x:v>measured inference goodput, measured system power, absolute productivity baseline, productivity trend</x:v>
       </x:c>
-      <x:c r="F11" s="16" t="str">
+      <x:c r="F13" s="16" t="str">
         <x:v>https://raw.githubusercontent.com/mlcommons/inference_results_v5.1/main/summary_results.json</x:v>
       </x:c>
-      <x:c r="G11" s="16" t="str">
+      <x:c r="G13" s="16" t="str">
         <x:v>Official MLPerf result data. Both selected rows are available, closed, datacenter Server results with reported power measurements.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="97.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A12" s="16" t="str">
+    <x:row r="14" ht="108" hidden="0" customHeight="1">
+      <x:c r="A14" s="16" t="str">
         <x:v>gate2-us-census-bureau-population-on-a-date</x:v>
       </x:c>
-      <x:c r="B12" s="16" t="str">
+      <x:c r="B14" s="16" t="str">
         <x:v>U.S. Census Bureau</x:v>
       </x:c>
-      <x:c r="C12" s="16" t="str">
+      <x:c r="C14" s="16" t="str">
         <x:v>Population on a Date</x:v>
       </x:c>
-      <x:c r="D12" s="16" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="E12" s="16" t="str">
+      <x:c r="D14" s="16" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="E14" s="16" t="str">
         <x:v>population</x:v>
       </x:c>
-      <x:c r="F12" s="16" t="str">
+      <x:c r="F14" s="16" t="str">
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
-      <x:c r="G12" s="16" t="str">
-        <x:v>The model uses the rounded estimate of 342.8M residents; the selected 25% target is 85.7M users.</x:v>
+      <x:c r="G14" s="16" t="str">
+        <x:v>The model uses the rounded estimate of 342.8M residents; the selected 50% target is 171.4M users.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6298,7 +6580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7b093100e1c4771"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c4c7616cb94c0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Revise Astra capability shock forecast
</commit_message>
<xml_diff>
--- a/artifacts/report-cards/personal-ai-compute-report-card.xlsx
+++ b/artifacts/report-cards/personal-ai-compute-report-card.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2da30dcbf2644ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R4e57fe731aed462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R8b6747e16928477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="Rfacee16119404a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R136faaaa791e4014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="Ra154bf24a5d44a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R52db042ed24f4e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R04cd63c68c99486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="2" r:id="R083f90d626834c2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R24d501a5f8f94e75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference Productivity" sheetId="4" r:id="R6af0e4314ced4fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Registry" sheetId="5" r:id="R0910c19e8ec64373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Evidence" sheetId="6" r:id="R903336819d7744ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R80566fb36ffc4774"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f69d6086dc04ff9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bcbcb91fde74a2c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -959,7 +959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fe90c70b5054888"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcc68d1b1c4343ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2573,9 +2573,9 @@
     <x:mergeCell ref="A3:W3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb50b13147c944b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488ba67f1a1041e1"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bc8d2cb74c3413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf9264817614f00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2816,7 +2816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R859095cce6a34854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9c05ed53e2e480b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3157,7 +3157,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe20e8b42b534539"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf62104192ec4454b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5394,7 +5394,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dffc153ecec46d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1178e13520b14a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6293,7 +6293,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75e27d83750948c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59fece4c608c4dcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6580,7 +6580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c4c7616cb94c0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb487bcf9caf34418"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>